<commit_message>
๊Update code and excel 2/4/2026
</commit_message>
<xml_diff>
--- a/Investment_Budget_69.xlsx
+++ b/Investment_Budget_69.xlsx
@@ -518,31 +518,31 @@
     <xf numFmtId="4" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -896,135 +896,135 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="203">
-      <c r="A2" s="16">
+    <row r="2" spans="1:17">
+      <c r="A2" s="19">
         <v>1</v>
       </c>
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="C2" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="D2" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="17" t="s">
+      <c r="E2" s="21" t="s">
         <v>20</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="G2" s="16" t="s">
+      <c r="G2" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="H2" s="18">
+      <c r="H2" s="20">
         <v>350000</v>
       </c>
-      <c r="I2" s="18">
+      <c r="I2" s="20">
         <v>350000</v>
       </c>
-      <c r="J2" s="16">
+      <c r="J2" s="19">
         <v>0</v>
       </c>
-      <c r="K2" s="16">
+      <c r="K2" s="19">
         <v>50</v>
       </c>
-      <c r="L2" s="16" t="s">
+      <c r="L2" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="M2" s="19">
-        <v>46113</v>
-      </c>
-      <c r="N2" s="16"/>
-      <c r="O2" s="16"/>
-      <c r="P2" s="20"/>
-      <c r="Q2" s="16"/>
-    </row>
-    <row r="3" spans="1:17" ht="159.5">
-      <c r="A3" s="16"/>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
-      <c r="D3" s="17"/>
-      <c r="E3" s="17"/>
+      <c r="M2" s="23">
+        <v>46026</v>
+      </c>
+      <c r="N2" s="19"/>
+      <c r="O2" s="19"/>
+      <c r="P2" s="24"/>
+      <c r="Q2" s="19"/>
+    </row>
+    <row r="3" spans="1:17">
+      <c r="A3" s="19"/>
+      <c r="B3" s="19"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
       <c r="F3" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="G3" s="16"/>
-      <c r="H3" s="18"/>
-      <c r="I3" s="18"/>
-      <c r="J3" s="16"/>
-      <c r="K3" s="16"/>
-      <c r="L3" s="16"/>
-      <c r="M3" s="19"/>
-      <c r="N3" s="16"/>
-      <c r="O3" s="16"/>
-      <c r="P3" s="20"/>
-      <c r="Q3" s="16"/>
-    </row>
-    <row r="4" spans="1:17" ht="130.5">
-      <c r="A4" s="21">
+      <c r="G3" s="19"/>
+      <c r="H3" s="20"/>
+      <c r="I3" s="20"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="19"/>
+      <c r="L3" s="19"/>
+      <c r="M3" s="23"/>
+      <c r="N3" s="19"/>
+      <c r="O3" s="19"/>
+      <c r="P3" s="24"/>
+      <c r="Q3" s="19"/>
+    </row>
+    <row r="4" spans="1:17">
+      <c r="A4" s="16">
         <v>2</v>
       </c>
-      <c r="B4" s="21" t="s">
+      <c r="B4" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="C4" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="22" t="s">
+      <c r="D4" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="E4" s="22" t="s">
+      <c r="E4" s="18" t="s">
         <v>27</v>
       </c>
       <c r="F4" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="G4" s="21"/>
-      <c r="H4" s="23">
+      <c r="G4" s="16"/>
+      <c r="H4" s="17">
         <v>460000</v>
       </c>
-      <c r="I4" s="23">
+      <c r="I4" s="17">
         <v>410995.5</v>
       </c>
-      <c r="J4" s="23">
+      <c r="J4" s="17">
         <v>49004.5</v>
       </c>
-      <c r="K4" s="21">
+      <c r="K4" s="16">
         <v>20</v>
       </c>
-      <c r="L4" s="21" t="s">
+      <c r="L4" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="M4" s="24">
-        <v>46113</v>
-      </c>
-      <c r="N4" s="21"/>
-      <c r="O4" s="21"/>
-      <c r="P4" s="21"/>
-      <c r="Q4" s="21"/>
-    </row>
-    <row r="5" spans="1:17" ht="232">
-      <c r="A5" s="21"/>
-      <c r="B5" s="21"/>
-      <c r="C5" s="21"/>
-      <c r="D5" s="22"/>
-      <c r="E5" s="22"/>
+      <c r="M4" s="22">
+        <v>46026</v>
+      </c>
+      <c r="N4" s="16"/>
+      <c r="O4" s="16"/>
+      <c r="P4" s="16"/>
+      <c r="Q4" s="16"/>
+    </row>
+    <row r="5" spans="1:17">
+      <c r="A5" s="16"/>
+      <c r="B5" s="16"/>
+      <c r="C5" s="16"/>
+      <c r="D5" s="18"/>
+      <c r="E5" s="18"/>
       <c r="F5" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="G5" s="21"/>
-      <c r="H5" s="23"/>
-      <c r="I5" s="23"/>
-      <c r="J5" s="23"/>
-      <c r="K5" s="21"/>
-      <c r="L5" s="21"/>
-      <c r="M5" s="24"/>
-      <c r="N5" s="21"/>
-      <c r="O5" s="21"/>
-      <c r="P5" s="21"/>
-      <c r="Q5" s="21"/>
+      <c r="G5" s="16"/>
+      <c r="H5" s="17"/>
+      <c r="I5" s="17"/>
+      <c r="J5" s="17"/>
+      <c r="K5" s="16"/>
+      <c r="L5" s="16"/>
+      <c r="M5" s="22"/>
+      <c r="N5" s="16"/>
+      <c r="O5" s="16"/>
+      <c r="P5" s="16"/>
+      <c r="Q5" s="16"/>
     </row>
     <row r="6" spans="1:17" ht="58">
       <c r="A6" s="2">
@@ -1062,7 +1062,7 @@
         <v>34</v>
       </c>
       <c r="M6" s="6">
-        <v>46113</v>
+        <v>46026</v>
       </c>
       <c r="N6" s="12" t="s">
         <v>35</v>
@@ -1109,7 +1109,7 @@
         <v>34</v>
       </c>
       <c r="M7" s="11">
-        <v>46113</v>
+        <v>46026</v>
       </c>
       <c r="N7" s="7"/>
       <c r="O7" s="7"/>
@@ -1152,7 +1152,7 @@
         <v>34</v>
       </c>
       <c r="M8" s="6">
-        <v>46113</v>
+        <v>46026</v>
       </c>
       <c r="N8" s="13" t="s">
         <v>43</v>
@@ -1161,133 +1161,133 @@
       <c r="P8" s="2"/>
       <c r="Q8" s="2"/>
     </row>
-    <row r="9" spans="1:17" ht="159.5">
-      <c r="A9" s="21">
+    <row r="9" spans="1:17">
+      <c r="A9" s="16">
         <v>6</v>
       </c>
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="21" t="s">
+      <c r="C9" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="D9" s="22" t="s">
+      <c r="D9" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="E9" s="22" t="s">
+      <c r="E9" s="18" t="s">
         <v>45</v>
       </c>
       <c r="F9" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="G9" s="21"/>
-      <c r="H9" s="23">
+      <c r="G9" s="16"/>
+      <c r="H9" s="17">
         <v>160000</v>
       </c>
-      <c r="I9" s="23">
+      <c r="I9" s="17">
         <v>160000</v>
       </c>
-      <c r="J9" s="21">
+      <c r="J9" s="16">
         <v>0</v>
       </c>
-      <c r="K9" s="21">
+      <c r="K9" s="16">
         <v>50</v>
       </c>
-      <c r="L9" s="21" t="s">
+      <c r="L9" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="M9" s="24">
-        <v>46113</v>
-      </c>
-      <c r="N9" s="21"/>
-      <c r="O9" s="21"/>
-      <c r="P9" s="21"/>
-      <c r="Q9" s="21"/>
-    </row>
-    <row r="10" spans="1:17" ht="116">
-      <c r="A10" s="21"/>
-      <c r="B10" s="21"/>
-      <c r="C10" s="21"/>
-      <c r="D10" s="22"/>
-      <c r="E10" s="22"/>
+      <c r="M9" s="22">
+        <v>46026</v>
+      </c>
+      <c r="N9" s="16"/>
+      <c r="O9" s="16"/>
+      <c r="P9" s="16"/>
+      <c r="Q9" s="16"/>
+    </row>
+    <row r="10" spans="1:17">
+      <c r="A10" s="16"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
       <c r="F10" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="G10" s="21"/>
-      <c r="H10" s="23"/>
-      <c r="I10" s="23"/>
-      <c r="J10" s="21"/>
-      <c r="K10" s="21"/>
-      <c r="L10" s="21"/>
-      <c r="M10" s="24"/>
-      <c r="N10" s="21"/>
-      <c r="O10" s="21"/>
-      <c r="P10" s="21"/>
-      <c r="Q10" s="21"/>
-    </row>
-    <row r="11" spans="1:17" ht="145">
-      <c r="A11" s="16">
+      <c r="G10" s="16"/>
+      <c r="H10" s="17"/>
+      <c r="I10" s="17"/>
+      <c r="J10" s="16"/>
+      <c r="K10" s="16"/>
+      <c r="L10" s="16"/>
+      <c r="M10" s="22"/>
+      <c r="N10" s="16"/>
+      <c r="O10" s="16"/>
+      <c r="P10" s="16"/>
+      <c r="Q10" s="16"/>
+    </row>
+    <row r="11" spans="1:17">
+      <c r="A11" s="19">
         <v>7</v>
       </c>
-      <c r="B11" s="16" t="s">
+      <c r="B11" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="16" t="s">
+      <c r="C11" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="D11" s="17" t="s">
+      <c r="D11" s="21" t="s">
         <v>49</v>
       </c>
-      <c r="E11" s="17" t="s">
+      <c r="E11" s="21" t="s">
         <v>50</v>
       </c>
       <c r="F11" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="G11" s="16"/>
-      <c r="H11" s="18">
+      <c r="G11" s="19"/>
+      <c r="H11" s="20">
         <v>1490000</v>
       </c>
-      <c r="I11" s="18">
+      <c r="I11" s="20">
         <v>1033230</v>
       </c>
-      <c r="J11" s="18">
+      <c r="J11" s="20">
         <v>456770</v>
       </c>
-      <c r="K11" s="16">
+      <c r="K11" s="19">
         <v>15</v>
       </c>
-      <c r="L11" s="16" t="s">
+      <c r="L11" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="M11" s="19">
-        <v>46113</v>
-      </c>
-      <c r="N11" s="16"/>
-      <c r="O11" s="16"/>
-      <c r="P11" s="16"/>
-      <c r="Q11" s="16"/>
-    </row>
-    <row r="12" spans="1:17" ht="319">
-      <c r="A12" s="16"/>
-      <c r="B12" s="16"/>
-      <c r="C12" s="16"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
+      <c r="M11" s="23">
+        <v>46026</v>
+      </c>
+      <c r="N11" s="19"/>
+      <c r="O11" s="19"/>
+      <c r="P11" s="19"/>
+      <c r="Q11" s="19"/>
+    </row>
+    <row r="12" spans="1:17" ht="29">
+      <c r="A12" s="19"/>
+      <c r="B12" s="19"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="21"/>
+      <c r="E12" s="21"/>
       <c r="F12" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="G12" s="16"/>
-      <c r="H12" s="18"/>
-      <c r="I12" s="18"/>
-      <c r="J12" s="18"/>
-      <c r="K12" s="16"/>
-      <c r="L12" s="16"/>
-      <c r="M12" s="19"/>
-      <c r="N12" s="16"/>
-      <c r="O12" s="16"/>
-      <c r="P12" s="16"/>
-      <c r="Q12" s="16"/>
+      <c r="G12" s="19"/>
+      <c r="H12" s="20"/>
+      <c r="I12" s="20"/>
+      <c r="J12" s="20"/>
+      <c r="K12" s="19"/>
+      <c r="L12" s="19"/>
+      <c r="M12" s="23"/>
+      <c r="N12" s="19"/>
+      <c r="O12" s="19"/>
+      <c r="P12" s="19"/>
+      <c r="Q12" s="19"/>
     </row>
     <row r="13" spans="1:17">
       <c r="A13" s="7">
@@ -1325,138 +1325,138 @@
         <v>24</v>
       </c>
       <c r="M13" s="11">
-        <v>46113</v>
+        <v>46026</v>
       </c>
       <c r="N13" s="7"/>
       <c r="O13" s="7"/>
       <c r="P13" s="7"/>
       <c r="Q13" s="7"/>
     </row>
-    <row r="14" spans="1:17" ht="159.5">
-      <c r="A14" s="16">
+    <row r="14" spans="1:17">
+      <c r="A14" s="19">
         <v>9</v>
       </c>
-      <c r="B14" s="16" t="s">
+      <c r="B14" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="C14" s="16" t="s">
+      <c r="C14" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="D14" s="17" t="s">
+      <c r="D14" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="E14" s="17" t="s">
+      <c r="E14" s="21" t="s">
         <v>58</v>
       </c>
       <c r="F14" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="G14" s="16"/>
-      <c r="H14" s="18">
+      <c r="G14" s="19"/>
+      <c r="H14" s="20">
         <v>1200000</v>
       </c>
-      <c r="I14" s="18">
+      <c r="I14" s="20">
         <v>1100000</v>
       </c>
-      <c r="J14" s="18">
+      <c r="J14" s="20">
         <v>100000</v>
       </c>
-      <c r="K14" s="16">
+      <c r="K14" s="19">
         <v>10</v>
       </c>
-      <c r="L14" s="16" t="s">
+      <c r="L14" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="M14" s="19">
+      <c r="M14" s="23">
         <v>46104</v>
       </c>
-      <c r="N14" s="16"/>
-      <c r="O14" s="16"/>
-      <c r="P14" s="16"/>
-      <c r="Q14" s="16"/>
-    </row>
-    <row r="15" spans="1:17" ht="275.5">
-      <c r="A15" s="16"/>
-      <c r="B15" s="16"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="17"/>
+      <c r="N14" s="19"/>
+      <c r="O14" s="19"/>
+      <c r="P14" s="19"/>
+      <c r="Q14" s="19"/>
+    </row>
+    <row r="15" spans="1:17">
+      <c r="A15" s="19"/>
+      <c r="B15" s="19"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="21"/>
+      <c r="E15" s="21"/>
       <c r="F15" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="G15" s="16"/>
-      <c r="H15" s="18"/>
-      <c r="I15" s="18"/>
-      <c r="J15" s="18"/>
-      <c r="K15" s="16"/>
-      <c r="L15" s="16"/>
-      <c r="M15" s="19"/>
-      <c r="N15" s="16"/>
-      <c r="O15" s="16"/>
-      <c r="P15" s="16"/>
-      <c r="Q15" s="16"/>
-    </row>
-    <row r="16" spans="1:17" ht="145">
-      <c r="A16" s="21">
+      <c r="G15" s="19"/>
+      <c r="H15" s="20"/>
+      <c r="I15" s="20"/>
+      <c r="J15" s="20"/>
+      <c r="K15" s="19"/>
+      <c r="L15" s="19"/>
+      <c r="M15" s="23"/>
+      <c r="N15" s="19"/>
+      <c r="O15" s="19"/>
+      <c r="P15" s="19"/>
+      <c r="Q15" s="19"/>
+    </row>
+    <row r="16" spans="1:17">
+      <c r="A16" s="16">
         <v>10</v>
       </c>
-      <c r="B16" s="21" t="s">
+      <c r="B16" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="C16" s="21" t="s">
+      <c r="C16" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="D16" s="22" t="s">
+      <c r="D16" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="E16" s="22" t="s">
+      <c r="E16" s="18" t="s">
         <v>50</v>
       </c>
       <c r="F16" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="G16" s="21"/>
-      <c r="H16" s="23">
+      <c r="G16" s="16"/>
+      <c r="H16" s="17">
         <v>1430000</v>
       </c>
-      <c r="I16" s="21"/>
-      <c r="J16" s="23">
+      <c r="I16" s="16"/>
+      <c r="J16" s="17">
         <v>1430000</v>
       </c>
-      <c r="K16" s="21">
+      <c r="K16" s="16">
         <v>5</v>
       </c>
-      <c r="L16" s="21" t="s">
+      <c r="L16" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="M16" s="24">
+      <c r="M16" s="22">
         <v>46104</v>
       </c>
-      <c r="N16" s="21"/>
-      <c r="O16" s="21"/>
-      <c r="P16" s="21"/>
-      <c r="Q16" s="21"/>
-    </row>
-    <row r="17" spans="1:17" ht="319">
-      <c r="A17" s="21"/>
-      <c r="B17" s="21"/>
-      <c r="C17" s="21"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="22"/>
+      <c r="N16" s="16"/>
+      <c r="O16" s="16"/>
+      <c r="P16" s="16"/>
+      <c r="Q16" s="16"/>
+    </row>
+    <row r="17" spans="1:17" ht="29">
+      <c r="A17" s="16"/>
+      <c r="B17" s="16"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="18"/>
+      <c r="E17" s="18"/>
       <c r="F17" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="G17" s="21"/>
-      <c r="H17" s="23"/>
-      <c r="I17" s="21"/>
-      <c r="J17" s="23"/>
-      <c r="K17" s="21"/>
-      <c r="L17" s="21"/>
-      <c r="M17" s="24"/>
-      <c r="N17" s="21"/>
-      <c r="O17" s="21"/>
-      <c r="P17" s="21"/>
-      <c r="Q17" s="21"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="17"/>
+      <c r="I17" s="16"/>
+      <c r="J17" s="17"/>
+      <c r="K17" s="16"/>
+      <c r="L17" s="16"/>
+      <c r="M17" s="22"/>
+      <c r="N17" s="16"/>
+      <c r="O17" s="16"/>
+      <c r="P17" s="16"/>
+      <c r="Q17" s="16"/>
     </row>
     <row r="18" spans="1:17">
       <c r="A18" s="2">
@@ -1497,67 +1497,67 @@
         <v>62</v>
       </c>
     </row>
-    <row r="19" spans="1:17" ht="145">
-      <c r="A19" s="21">
+    <row r="19" spans="1:17">
+      <c r="A19" s="16">
         <v>12</v>
       </c>
-      <c r="B19" s="21" t="s">
+      <c r="B19" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="C19" s="21" t="s">
+      <c r="C19" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="D19" s="22" t="s">
+      <c r="D19" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="E19" s="22" t="s">
+      <c r="E19" s="18" t="s">
         <v>50</v>
       </c>
       <c r="F19" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="G19" s="21"/>
-      <c r="H19" s="23">
+      <c r="G19" s="16"/>
+      <c r="H19" s="17">
         <v>920000</v>
       </c>
-      <c r="I19" s="21"/>
-      <c r="J19" s="23">
+      <c r="I19" s="16"/>
+      <c r="J19" s="17">
         <v>920000</v>
       </c>
-      <c r="K19" s="21">
+      <c r="K19" s="16">
         <v>5</v>
       </c>
-      <c r="L19" s="21" t="s">
+      <c r="L19" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="M19" s="24">
+      <c r="M19" s="22">
         <v>46104</v>
       </c>
-      <c r="N19" s="21"/>
-      <c r="O19" s="21"/>
-      <c r="P19" s="21"/>
-      <c r="Q19" s="21"/>
-    </row>
-    <row r="20" spans="1:17" ht="319">
-      <c r="A20" s="21"/>
-      <c r="B20" s="21"/>
-      <c r="C20" s="21"/>
-      <c r="D20" s="22"/>
-      <c r="E20" s="22"/>
+      <c r="N19" s="16"/>
+      <c r="O19" s="16"/>
+      <c r="P19" s="16"/>
+      <c r="Q19" s="16"/>
+    </row>
+    <row r="20" spans="1:17" ht="29">
+      <c r="A20" s="16"/>
+      <c r="B20" s="16"/>
+      <c r="C20" s="16"/>
+      <c r="D20" s="18"/>
+      <c r="E20" s="18"/>
       <c r="F20" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="G20" s="21"/>
-      <c r="H20" s="23"/>
-      <c r="I20" s="21"/>
-      <c r="J20" s="23"/>
-      <c r="K20" s="21"/>
-      <c r="L20" s="21"/>
-      <c r="M20" s="24"/>
-      <c r="N20" s="21"/>
-      <c r="O20" s="21"/>
-      <c r="P20" s="21"/>
-      <c r="Q20" s="21"/>
+      <c r="G20" s="16"/>
+      <c r="H20" s="17"/>
+      <c r="I20" s="16"/>
+      <c r="J20" s="17"/>
+      <c r="K20" s="16"/>
+      <c r="L20" s="16"/>
+      <c r="M20" s="22"/>
+      <c r="N20" s="16"/>
+      <c r="O20" s="16"/>
+      <c r="P20" s="16"/>
+      <c r="Q20" s="16"/>
     </row>
     <row r="21" spans="1:17">
       <c r="A21" s="2">
@@ -1598,233 +1598,233 @@
         <v>62</v>
       </c>
     </row>
-    <row r="22" spans="1:17" ht="101.5">
-      <c r="A22" s="21">
+    <row r="22" spans="1:17">
+      <c r="A22" s="16">
         <v>14</v>
       </c>
-      <c r="B22" s="21" t="s">
+      <c r="B22" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="C22" s="21" t="s">
+      <c r="C22" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="D22" s="22" t="s">
+      <c r="D22" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="E22" s="22" t="s">
+      <c r="E22" s="18" t="s">
         <v>66</v>
       </c>
       <c r="F22" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="G22" s="21" t="s">
+      <c r="G22" s="16" t="s">
         <v>69</v>
       </c>
-      <c r="H22" s="23">
+      <c r="H22" s="17">
         <v>100000</v>
       </c>
-      <c r="I22" s="21"/>
-      <c r="J22" s="23">
+      <c r="I22" s="16"/>
+      <c r="J22" s="17">
         <v>100000</v>
       </c>
-      <c r="K22" s="21"/>
-      <c r="L22" s="21"/>
-      <c r="M22" s="21"/>
-      <c r="N22" s="21"/>
-      <c r="O22" s="21"/>
-      <c r="P22" s="21"/>
-      <c r="Q22" s="21"/>
-    </row>
-    <row r="23" spans="1:17" ht="261">
-      <c r="A23" s="21"/>
-      <c r="B23" s="21"/>
-      <c r="C23" s="21"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="22"/>
+      <c r="K22" s="16"/>
+      <c r="L22" s="16"/>
+      <c r="M22" s="16"/>
+      <c r="N22" s="16"/>
+      <c r="O22" s="16"/>
+      <c r="P22" s="16"/>
+      <c r="Q22" s="16"/>
+    </row>
+    <row r="23" spans="1:17">
+      <c r="A23" s="16"/>
+      <c r="B23" s="16"/>
+      <c r="C23" s="16"/>
+      <c r="D23" s="18"/>
+      <c r="E23" s="18"/>
       <c r="F23" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="G23" s="21"/>
-      <c r="H23" s="23"/>
-      <c r="I23" s="21"/>
-      <c r="J23" s="23"/>
-      <c r="K23" s="21"/>
-      <c r="L23" s="21"/>
-      <c r="M23" s="21"/>
-      <c r="N23" s="21"/>
-      <c r="O23" s="21"/>
-      <c r="P23" s="21"/>
-      <c r="Q23" s="21"/>
-    </row>
-    <row r="24" spans="1:17" ht="116">
-      <c r="A24" s="16">
+      <c r="G23" s="16"/>
+      <c r="H23" s="17"/>
+      <c r="I23" s="16"/>
+      <c r="J23" s="17"/>
+      <c r="K23" s="16"/>
+      <c r="L23" s="16"/>
+      <c r="M23" s="16"/>
+      <c r="N23" s="16"/>
+      <c r="O23" s="16"/>
+      <c r="P23" s="16"/>
+      <c r="Q23" s="16"/>
+    </row>
+    <row r="24" spans="1:17">
+      <c r="A24" s="19">
         <v>15</v>
       </c>
-      <c r="B24" s="16" t="s">
+      <c r="B24" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="C24" s="16" t="s">
+      <c r="C24" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="D24" s="17" t="s">
+      <c r="D24" s="21" t="s">
         <v>70</v>
       </c>
-      <c r="E24" s="17" t="s">
+      <c r="E24" s="21" t="s">
         <v>71</v>
       </c>
       <c r="F24" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="G24" s="16" t="s">
+      <c r="G24" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="H24" s="18">
+      <c r="H24" s="20">
         <v>370000</v>
       </c>
-      <c r="I24" s="16"/>
-      <c r="J24" s="18">
+      <c r="I24" s="19"/>
+      <c r="J24" s="20">
         <v>370000</v>
       </c>
-      <c r="K24" s="16"/>
-      <c r="L24" s="16"/>
-      <c r="M24" s="16"/>
-      <c r="N24" s="16"/>
-      <c r="O24" s="16"/>
-      <c r="P24" s="16"/>
-      <c r="Q24" s="16"/>
-    </row>
-    <row r="25" spans="1:17" ht="87">
-      <c r="A25" s="16"/>
-      <c r="B25" s="16"/>
-      <c r="C25" s="16"/>
-      <c r="D25" s="17"/>
-      <c r="E25" s="17"/>
+      <c r="K24" s="19"/>
+      <c r="L24" s="19"/>
+      <c r="M24" s="19"/>
+      <c r="N24" s="19"/>
+      <c r="O24" s="19"/>
+      <c r="P24" s="19"/>
+      <c r="Q24" s="19"/>
+    </row>
+    <row r="25" spans="1:17">
+      <c r="A25" s="19"/>
+      <c r="B25" s="19"/>
+      <c r="C25" s="19"/>
+      <c r="D25" s="21"/>
+      <c r="E25" s="21"/>
       <c r="F25" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="G25" s="16"/>
-      <c r="H25" s="18"/>
-      <c r="I25" s="16"/>
-      <c r="J25" s="18"/>
-      <c r="K25" s="16"/>
-      <c r="L25" s="16"/>
-      <c r="M25" s="16"/>
-      <c r="N25" s="16"/>
-      <c r="O25" s="16"/>
-      <c r="P25" s="16"/>
-      <c r="Q25" s="16"/>
-    </row>
-    <row r="26" spans="1:17" ht="130.5">
-      <c r="A26" s="21">
+      <c r="G25" s="19"/>
+      <c r="H25" s="20"/>
+      <c r="I25" s="19"/>
+      <c r="J25" s="20"/>
+      <c r="K25" s="19"/>
+      <c r="L25" s="19"/>
+      <c r="M25" s="19"/>
+      <c r="N25" s="19"/>
+      <c r="O25" s="19"/>
+      <c r="P25" s="19"/>
+      <c r="Q25" s="19"/>
+    </row>
+    <row r="26" spans="1:17">
+      <c r="A26" s="16">
         <v>16</v>
       </c>
-      <c r="B26" s="21" t="s">
+      <c r="B26" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="C26" s="21" t="s">
+      <c r="C26" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="D26" s="22" t="s">
+      <c r="D26" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="E26" s="22" t="s">
+      <c r="E26" s="18" t="s">
         <v>76</v>
       </c>
       <c r="F26" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="G26" s="21"/>
-      <c r="H26" s="23">
+      <c r="G26" s="16"/>
+      <c r="H26" s="17">
         <v>2255000</v>
       </c>
-      <c r="I26" s="21"/>
-      <c r="J26" s="23">
+      <c r="I26" s="16"/>
+      <c r="J26" s="17">
         <v>2255000</v>
       </c>
-      <c r="K26" s="21"/>
-      <c r="L26" s="21"/>
-      <c r="M26" s="21"/>
-      <c r="N26" s="21"/>
-      <c r="O26" s="21"/>
-      <c r="P26" s="21"/>
-      <c r="Q26" s="21"/>
-    </row>
-    <row r="27" spans="1:17" ht="304.5">
-      <c r="A27" s="21"/>
-      <c r="B27" s="21"/>
-      <c r="C27" s="21"/>
-      <c r="D27" s="22"/>
-      <c r="E27" s="22"/>
+      <c r="K26" s="16"/>
+      <c r="L26" s="16"/>
+      <c r="M26" s="16"/>
+      <c r="N26" s="16"/>
+      <c r="O26" s="16"/>
+      <c r="P26" s="16"/>
+      <c r="Q26" s="16"/>
+    </row>
+    <row r="27" spans="1:17">
+      <c r="A27" s="16"/>
+      <c r="B27" s="16"/>
+      <c r="C27" s="16"/>
+      <c r="D27" s="18"/>
+      <c r="E27" s="18"/>
       <c r="F27" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="G27" s="21"/>
-      <c r="H27" s="23"/>
-      <c r="I27" s="21"/>
-      <c r="J27" s="23"/>
-      <c r="K27" s="21"/>
-      <c r="L27" s="21"/>
-      <c r="M27" s="21"/>
-      <c r="N27" s="21"/>
-      <c r="O27" s="21"/>
-      <c r="P27" s="21"/>
-      <c r="Q27" s="21"/>
-    </row>
-    <row r="28" spans="1:17" ht="116">
-      <c r="A28" s="16">
+      <c r="G27" s="16"/>
+      <c r="H27" s="17"/>
+      <c r="I27" s="16"/>
+      <c r="J27" s="17"/>
+      <c r="K27" s="16"/>
+      <c r="L27" s="16"/>
+      <c r="M27" s="16"/>
+      <c r="N27" s="16"/>
+      <c r="O27" s="16"/>
+      <c r="P27" s="16"/>
+      <c r="Q27" s="16"/>
+    </row>
+    <row r="28" spans="1:17">
+      <c r="A28" s="19">
         <v>17</v>
       </c>
-      <c r="B28" s="16" t="s">
+      <c r="B28" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="C28" s="16" t="s">
+      <c r="C28" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="D28" s="17" t="s">
+      <c r="D28" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="E28" s="17" t="s">
+      <c r="E28" s="21" t="s">
         <v>80</v>
       </c>
       <c r="F28" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="G28" s="16"/>
-      <c r="H28" s="18">
+      <c r="G28" s="19"/>
+      <c r="H28" s="20">
         <v>110000</v>
       </c>
-      <c r="I28" s="16"/>
-      <c r="J28" s="18">
+      <c r="I28" s="19"/>
+      <c r="J28" s="20">
         <v>110000</v>
       </c>
-      <c r="K28" s="16"/>
-      <c r="L28" s="16"/>
-      <c r="M28" s="16"/>
-      <c r="N28" s="16"/>
-      <c r="O28" s="16"/>
-      <c r="P28" s="16"/>
-      <c r="Q28" s="16"/>
-    </row>
-    <row r="29" spans="1:17" ht="145">
-      <c r="A29" s="16"/>
-      <c r="B29" s="16"/>
-      <c r="C29" s="16"/>
-      <c r="D29" s="17"/>
-      <c r="E29" s="17"/>
+      <c r="K28" s="19"/>
+      <c r="L28" s="19"/>
+      <c r="M28" s="19"/>
+      <c r="N28" s="19"/>
+      <c r="O28" s="19"/>
+      <c r="P28" s="19"/>
+      <c r="Q28" s="19"/>
+    </row>
+    <row r="29" spans="1:17">
+      <c r="A29" s="19"/>
+      <c r="B29" s="19"/>
+      <c r="C29" s="19"/>
+      <c r="D29" s="21"/>
+      <c r="E29" s="21"/>
       <c r="F29" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="G29" s="16"/>
-      <c r="H29" s="18"/>
-      <c r="I29" s="16"/>
-      <c r="J29" s="18"/>
-      <c r="K29" s="16"/>
-      <c r="L29" s="16"/>
-      <c r="M29" s="16"/>
-      <c r="N29" s="16"/>
-      <c r="O29" s="16"/>
-      <c r="P29" s="16"/>
-      <c r="Q29" s="16"/>
+      <c r="G29" s="19"/>
+      <c r="H29" s="20"/>
+      <c r="I29" s="19"/>
+      <c r="J29" s="20"/>
+      <c r="K29" s="19"/>
+      <c r="L29" s="19"/>
+      <c r="M29" s="19"/>
+      <c r="N29" s="19"/>
+      <c r="O29" s="19"/>
+      <c r="P29" s="19"/>
+      <c r="Q29" s="19"/>
     </row>
     <row r="30" spans="1:17">
       <c r="A30" s="7">
@@ -1863,61 +1863,61 @@
       <c r="P30" s="7"/>
       <c r="Q30" s="7"/>
     </row>
-    <row r="31" spans="1:17" ht="130.5">
-      <c r="A31" s="16">
+    <row r="31" spans="1:17">
+      <c r="A31" s="19">
         <v>19</v>
       </c>
-      <c r="B31" s="16" t="s">
+      <c r="B31" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="C31" s="16" t="s">
+      <c r="C31" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="D31" s="17" t="s">
+      <c r="D31" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="E31" s="17" t="s">
+      <c r="E31" s="21" t="s">
         <v>88</v>
       </c>
       <c r="F31" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="G31" s="16"/>
-      <c r="H31" s="18">
+      <c r="G31" s="19"/>
+      <c r="H31" s="20">
         <v>28000</v>
       </c>
-      <c r="I31" s="16"/>
-      <c r="J31" s="18">
+      <c r="I31" s="19"/>
+      <c r="J31" s="20">
         <v>28000</v>
       </c>
-      <c r="K31" s="16"/>
-      <c r="L31" s="16"/>
-      <c r="M31" s="16"/>
-      <c r="N31" s="16"/>
-      <c r="O31" s="16"/>
-      <c r="P31" s="16"/>
-      <c r="Q31" s="16"/>
-    </row>
-    <row r="32" spans="1:17" ht="188.5">
-      <c r="A32" s="16"/>
-      <c r="B32" s="16"/>
-      <c r="C32" s="16"/>
-      <c r="D32" s="17"/>
-      <c r="E32" s="17"/>
+      <c r="K31" s="19"/>
+      <c r="L31" s="19"/>
+      <c r="M31" s="19"/>
+      <c r="N31" s="19"/>
+      <c r="O31" s="19"/>
+      <c r="P31" s="19"/>
+      <c r="Q31" s="19"/>
+    </row>
+    <row r="32" spans="1:17">
+      <c r="A32" s="19"/>
+      <c r="B32" s="19"/>
+      <c r="C32" s="19"/>
+      <c r="D32" s="21"/>
+      <c r="E32" s="21"/>
       <c r="F32" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="G32" s="16"/>
-      <c r="H32" s="18"/>
-      <c r="I32" s="16"/>
-      <c r="J32" s="18"/>
-      <c r="K32" s="16"/>
-      <c r="L32" s="16"/>
-      <c r="M32" s="16"/>
-      <c r="N32" s="16"/>
-      <c r="O32" s="16"/>
-      <c r="P32" s="16"/>
-      <c r="Q32" s="16"/>
+      <c r="G32" s="19"/>
+      <c r="H32" s="20"/>
+      <c r="I32" s="19"/>
+      <c r="J32" s="20"/>
+      <c r="K32" s="19"/>
+      <c r="L32" s="19"/>
+      <c r="M32" s="19"/>
+      <c r="N32" s="19"/>
+      <c r="O32" s="19"/>
+      <c r="P32" s="19"/>
+      <c r="Q32" s="19"/>
     </row>
     <row r="33" spans="1:17">
       <c r="A33" s="7">
@@ -1989,63 +1989,63 @@
       <c r="P34" s="2"/>
       <c r="Q34" s="2"/>
     </row>
-    <row r="35" spans="1:17" ht="174">
-      <c r="A35" s="21">
+    <row r="35" spans="1:17">
+      <c r="A35" s="16">
         <v>22</v>
       </c>
-      <c r="B35" s="21" t="s">
+      <c r="B35" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="C35" s="21" t="s">
+      <c r="C35" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="D35" s="22" t="s">
+      <c r="D35" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="E35" s="22" t="s">
+      <c r="E35" s="18" t="s">
         <v>97</v>
       </c>
       <c r="F35" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="G35" s="21" t="s">
+      <c r="G35" s="16" t="s">
         <v>100</v>
       </c>
-      <c r="H35" s="23">
+      <c r="H35" s="17">
         <v>80000</v>
       </c>
-      <c r="I35" s="21"/>
-      <c r="J35" s="23">
+      <c r="I35" s="16"/>
+      <c r="J35" s="17">
         <v>80000</v>
       </c>
-      <c r="K35" s="21"/>
-      <c r="L35" s="21"/>
-      <c r="M35" s="21"/>
-      <c r="N35" s="21"/>
-      <c r="O35" s="21"/>
-      <c r="P35" s="21"/>
-      <c r="Q35" s="21"/>
-    </row>
-    <row r="36" spans="1:17" ht="159.5">
-      <c r="A36" s="21"/>
-      <c r="B36" s="21"/>
-      <c r="C36" s="21"/>
-      <c r="D36" s="22"/>
-      <c r="E36" s="22"/>
+      <c r="K35" s="16"/>
+      <c r="L35" s="16"/>
+      <c r="M35" s="16"/>
+      <c r="N35" s="16"/>
+      <c r="O35" s="16"/>
+      <c r="P35" s="16"/>
+      <c r="Q35" s="16"/>
+    </row>
+    <row r="36" spans="1:17">
+      <c r="A36" s="16"/>
+      <c r="B36" s="16"/>
+      <c r="C36" s="16"/>
+      <c r="D36" s="18"/>
+      <c r="E36" s="18"/>
       <c r="F36" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="G36" s="21"/>
-      <c r="H36" s="23"/>
-      <c r="I36" s="21"/>
-      <c r="J36" s="23"/>
-      <c r="K36" s="21"/>
-      <c r="L36" s="21"/>
-      <c r="M36" s="21"/>
-      <c r="N36" s="21"/>
-      <c r="O36" s="21"/>
-      <c r="P36" s="21"/>
-      <c r="Q36" s="21"/>
+      <c r="G36" s="16"/>
+      <c r="H36" s="17"/>
+      <c r="I36" s="16"/>
+      <c r="J36" s="17"/>
+      <c r="K36" s="16"/>
+      <c r="L36" s="16"/>
+      <c r="M36" s="16"/>
+      <c r="N36" s="16"/>
+      <c r="O36" s="16"/>
+      <c r="P36" s="16"/>
+      <c r="Q36" s="16"/>
     </row>
     <row r="37" spans="1:17">
       <c r="A37" s="2">
@@ -2082,61 +2082,61 @@
       <c r="P37" s="2"/>
       <c r="Q37" s="2"/>
     </row>
-    <row r="38" spans="1:17" ht="145">
-      <c r="A38" s="21">
+    <row r="38" spans="1:17">
+      <c r="A38" s="16">
         <v>24</v>
       </c>
-      <c r="B38" s="21" t="s">
+      <c r="B38" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="C38" s="21" t="s">
+      <c r="C38" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="D38" s="22" t="s">
+      <c r="D38" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="E38" s="22" t="s">
+      <c r="E38" s="18" t="s">
         <v>50</v>
       </c>
       <c r="F38" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="G38" s="21"/>
-      <c r="H38" s="23">
+      <c r="G38" s="16"/>
+      <c r="H38" s="17">
         <v>982000</v>
       </c>
-      <c r="I38" s="21"/>
-      <c r="J38" s="23">
+      <c r="I38" s="16"/>
+      <c r="J38" s="17">
         <v>982000</v>
       </c>
-      <c r="K38" s="21"/>
-      <c r="L38" s="21"/>
-      <c r="M38" s="21"/>
-      <c r="N38" s="21"/>
-      <c r="O38" s="21"/>
-      <c r="P38" s="21"/>
-      <c r="Q38" s="21"/>
-    </row>
-    <row r="39" spans="1:17" ht="319">
-      <c r="A39" s="21"/>
-      <c r="B39" s="21"/>
-      <c r="C39" s="21"/>
-      <c r="D39" s="22"/>
-      <c r="E39" s="22"/>
+      <c r="K38" s="16"/>
+      <c r="L38" s="16"/>
+      <c r="M38" s="16"/>
+      <c r="N38" s="16"/>
+      <c r="O38" s="16"/>
+      <c r="P38" s="16"/>
+      <c r="Q38" s="16"/>
+    </row>
+    <row r="39" spans="1:17" ht="29">
+      <c r="A39" s="16"/>
+      <c r="B39" s="16"/>
+      <c r="C39" s="16"/>
+      <c r="D39" s="18"/>
+      <c r="E39" s="18"/>
       <c r="F39" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="G39" s="21"/>
-      <c r="H39" s="23"/>
-      <c r="I39" s="21"/>
-      <c r="J39" s="23"/>
-      <c r="K39" s="21"/>
-      <c r="L39" s="21"/>
-      <c r="M39" s="21"/>
-      <c r="N39" s="21"/>
-      <c r="O39" s="21"/>
-      <c r="P39" s="21"/>
-      <c r="Q39" s="21"/>
+      <c r="G39" s="16"/>
+      <c r="H39" s="17"/>
+      <c r="I39" s="16"/>
+      <c r="J39" s="17"/>
+      <c r="K39" s="16"/>
+      <c r="L39" s="16"/>
+      <c r="M39" s="16"/>
+      <c r="N39" s="16"/>
+      <c r="O39" s="16"/>
+      <c r="P39" s="16"/>
+      <c r="Q39" s="16"/>
     </row>
     <row r="40" spans="1:17">
       <c r="A40" s="2">
@@ -2619,208 +2619,6 @@
     </row>
   </sheetData>
   <mergeCells count="224">
-    <mergeCell ref="N38:N39"/>
-    <mergeCell ref="O38:O39"/>
-    <mergeCell ref="P38:P39"/>
-    <mergeCell ref="Q38:Q39"/>
-    <mergeCell ref="H38:H39"/>
-    <mergeCell ref="I38:I39"/>
-    <mergeCell ref="J38:J39"/>
-    <mergeCell ref="K38:K39"/>
-    <mergeCell ref="L38:L39"/>
-    <mergeCell ref="M38:M39"/>
-    <mergeCell ref="N35:N36"/>
-    <mergeCell ref="O35:O36"/>
-    <mergeCell ref="P35:P36"/>
-    <mergeCell ref="Q35:Q36"/>
-    <mergeCell ref="A38:A39"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="C38:C39"/>
-    <mergeCell ref="D38:D39"/>
-    <mergeCell ref="E38:E39"/>
-    <mergeCell ref="G38:G39"/>
-    <mergeCell ref="H35:H36"/>
-    <mergeCell ref="I35:I36"/>
-    <mergeCell ref="J35:J36"/>
-    <mergeCell ref="K35:K36"/>
-    <mergeCell ref="L35:L36"/>
-    <mergeCell ref="M35:M36"/>
-    <mergeCell ref="N31:N32"/>
-    <mergeCell ref="O31:O32"/>
-    <mergeCell ref="P31:P32"/>
-    <mergeCell ref="Q31:Q32"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="B35:B36"/>
-    <mergeCell ref="C35:C36"/>
-    <mergeCell ref="D35:D36"/>
-    <mergeCell ref="E35:E36"/>
-    <mergeCell ref="G35:G36"/>
-    <mergeCell ref="H31:H32"/>
-    <mergeCell ref="I31:I32"/>
-    <mergeCell ref="J31:J32"/>
-    <mergeCell ref="K31:K32"/>
-    <mergeCell ref="L31:L32"/>
-    <mergeCell ref="M31:M32"/>
-    <mergeCell ref="N28:N29"/>
-    <mergeCell ref="O28:O29"/>
-    <mergeCell ref="P28:P29"/>
-    <mergeCell ref="Q28:Q29"/>
-    <mergeCell ref="A31:A32"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="C31:C32"/>
-    <mergeCell ref="D31:D32"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="G31:G32"/>
-    <mergeCell ref="H28:H29"/>
-    <mergeCell ref="I28:I29"/>
-    <mergeCell ref="J28:J29"/>
-    <mergeCell ref="K28:K29"/>
-    <mergeCell ref="L28:L29"/>
-    <mergeCell ref="M28:M29"/>
-    <mergeCell ref="N26:N27"/>
-    <mergeCell ref="O26:O27"/>
-    <mergeCell ref="P26:P27"/>
-    <mergeCell ref="Q26:Q27"/>
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="B28:B29"/>
-    <mergeCell ref="C28:C29"/>
-    <mergeCell ref="D28:D29"/>
-    <mergeCell ref="E28:E29"/>
-    <mergeCell ref="G28:G29"/>
-    <mergeCell ref="H26:H27"/>
-    <mergeCell ref="I26:I27"/>
-    <mergeCell ref="J26:J27"/>
-    <mergeCell ref="K26:K27"/>
-    <mergeCell ref="L26:L27"/>
-    <mergeCell ref="M26:M27"/>
-    <mergeCell ref="N24:N25"/>
-    <mergeCell ref="O24:O25"/>
-    <mergeCell ref="P24:P25"/>
-    <mergeCell ref="Q24:Q25"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="C26:C27"/>
-    <mergeCell ref="D26:D27"/>
-    <mergeCell ref="E26:E27"/>
-    <mergeCell ref="G26:G27"/>
-    <mergeCell ref="H24:H25"/>
-    <mergeCell ref="I24:I25"/>
-    <mergeCell ref="J24:J25"/>
-    <mergeCell ref="K24:K25"/>
-    <mergeCell ref="L24:L25"/>
-    <mergeCell ref="M24:M25"/>
-    <mergeCell ref="N22:N23"/>
-    <mergeCell ref="O22:O23"/>
-    <mergeCell ref="P22:P23"/>
-    <mergeCell ref="Q22:Q23"/>
-    <mergeCell ref="A24:A25"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="E24:E25"/>
-    <mergeCell ref="G24:G25"/>
-    <mergeCell ref="H22:H23"/>
-    <mergeCell ref="I22:I23"/>
-    <mergeCell ref="J22:J23"/>
-    <mergeCell ref="K22:K23"/>
-    <mergeCell ref="L22:L23"/>
-    <mergeCell ref="M22:M23"/>
-    <mergeCell ref="N19:N20"/>
-    <mergeCell ref="O19:O20"/>
-    <mergeCell ref="P19:P20"/>
-    <mergeCell ref="Q19:Q20"/>
-    <mergeCell ref="A22:A23"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="D22:D23"/>
-    <mergeCell ref="E22:E23"/>
-    <mergeCell ref="G22:G23"/>
-    <mergeCell ref="H19:H20"/>
-    <mergeCell ref="I19:I20"/>
-    <mergeCell ref="J19:J20"/>
-    <mergeCell ref="K19:K20"/>
-    <mergeCell ref="L19:L20"/>
-    <mergeCell ref="M19:M20"/>
-    <mergeCell ref="N16:N17"/>
-    <mergeCell ref="O16:O17"/>
-    <mergeCell ref="P16:P17"/>
-    <mergeCell ref="Q16:Q17"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="G19:G20"/>
-    <mergeCell ref="H16:H17"/>
-    <mergeCell ref="I16:I17"/>
-    <mergeCell ref="J16:J17"/>
-    <mergeCell ref="K16:K17"/>
-    <mergeCell ref="L16:L17"/>
-    <mergeCell ref="M16:M17"/>
-    <mergeCell ref="N14:N15"/>
-    <mergeCell ref="O14:O15"/>
-    <mergeCell ref="P14:P15"/>
-    <mergeCell ref="Q14:Q15"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="E16:E17"/>
-    <mergeCell ref="G16:G17"/>
-    <mergeCell ref="H14:H15"/>
-    <mergeCell ref="I14:I15"/>
-    <mergeCell ref="J14:J15"/>
-    <mergeCell ref="K14:K15"/>
-    <mergeCell ref="L14:L15"/>
-    <mergeCell ref="M14:M15"/>
-    <mergeCell ref="N11:N12"/>
-    <mergeCell ref="O11:O12"/>
-    <mergeCell ref="P11:P12"/>
-    <mergeCell ref="Q11:Q12"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="E14:E15"/>
-    <mergeCell ref="G14:G15"/>
-    <mergeCell ref="H11:H12"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="K11:K12"/>
-    <mergeCell ref="L11:L12"/>
-    <mergeCell ref="M11:M12"/>
-    <mergeCell ref="N9:N10"/>
-    <mergeCell ref="O9:O10"/>
-    <mergeCell ref="P9:P10"/>
-    <mergeCell ref="Q9:Q10"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="G11:G12"/>
-    <mergeCell ref="H9:H10"/>
-    <mergeCell ref="I9:I10"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="K9:K10"/>
-    <mergeCell ref="L9:L10"/>
-    <mergeCell ref="M9:M10"/>
-    <mergeCell ref="N4:N5"/>
-    <mergeCell ref="O4:O5"/>
-    <mergeCell ref="P4:P5"/>
-    <mergeCell ref="Q4:Q5"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="G9:G10"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="I4:I5"/>
-    <mergeCell ref="J4:J5"/>
-    <mergeCell ref="K4:K5"/>
-    <mergeCell ref="L4:L5"/>
-    <mergeCell ref="M4:M5"/>
     <mergeCell ref="N2:N3"/>
     <mergeCell ref="O2:O3"/>
     <mergeCell ref="P2:P3"/>
@@ -2843,6 +2641,208 @@
     <mergeCell ref="D2:D3"/>
     <mergeCell ref="E2:E3"/>
     <mergeCell ref="G2:G3"/>
+    <mergeCell ref="N4:N5"/>
+    <mergeCell ref="O4:O5"/>
+    <mergeCell ref="P4:P5"/>
+    <mergeCell ref="Q4:Q5"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="I4:I5"/>
+    <mergeCell ref="J4:J5"/>
+    <mergeCell ref="K4:K5"/>
+    <mergeCell ref="L4:L5"/>
+    <mergeCell ref="M4:M5"/>
+    <mergeCell ref="N9:N10"/>
+    <mergeCell ref="O9:O10"/>
+    <mergeCell ref="P9:P10"/>
+    <mergeCell ref="Q9:Q10"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="G11:G12"/>
+    <mergeCell ref="H9:H10"/>
+    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="K9:K10"/>
+    <mergeCell ref="L9:L10"/>
+    <mergeCell ref="M9:M10"/>
+    <mergeCell ref="N11:N12"/>
+    <mergeCell ref="O11:O12"/>
+    <mergeCell ref="P11:P12"/>
+    <mergeCell ref="Q11:Q12"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="E14:E15"/>
+    <mergeCell ref="G14:G15"/>
+    <mergeCell ref="H11:H12"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="K11:K12"/>
+    <mergeCell ref="L11:L12"/>
+    <mergeCell ref="M11:M12"/>
+    <mergeCell ref="N14:N15"/>
+    <mergeCell ref="O14:O15"/>
+    <mergeCell ref="P14:P15"/>
+    <mergeCell ref="Q14:Q15"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="E16:E17"/>
+    <mergeCell ref="G16:G17"/>
+    <mergeCell ref="H14:H15"/>
+    <mergeCell ref="I14:I15"/>
+    <mergeCell ref="J14:J15"/>
+    <mergeCell ref="K14:K15"/>
+    <mergeCell ref="L14:L15"/>
+    <mergeCell ref="M14:M15"/>
+    <mergeCell ref="N16:N17"/>
+    <mergeCell ref="O16:O17"/>
+    <mergeCell ref="P16:P17"/>
+    <mergeCell ref="Q16:Q17"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="G19:G20"/>
+    <mergeCell ref="H16:H17"/>
+    <mergeCell ref="I16:I17"/>
+    <mergeCell ref="J16:J17"/>
+    <mergeCell ref="K16:K17"/>
+    <mergeCell ref="L16:L17"/>
+    <mergeCell ref="M16:M17"/>
+    <mergeCell ref="N19:N20"/>
+    <mergeCell ref="O19:O20"/>
+    <mergeCell ref="P19:P20"/>
+    <mergeCell ref="Q19:Q20"/>
+    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="D22:D23"/>
+    <mergeCell ref="E22:E23"/>
+    <mergeCell ref="G22:G23"/>
+    <mergeCell ref="H19:H20"/>
+    <mergeCell ref="I19:I20"/>
+    <mergeCell ref="J19:J20"/>
+    <mergeCell ref="K19:K20"/>
+    <mergeCell ref="L19:L20"/>
+    <mergeCell ref="M19:M20"/>
+    <mergeCell ref="N22:N23"/>
+    <mergeCell ref="O22:O23"/>
+    <mergeCell ref="P22:P23"/>
+    <mergeCell ref="Q22:Q23"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="E24:E25"/>
+    <mergeCell ref="G24:G25"/>
+    <mergeCell ref="H22:H23"/>
+    <mergeCell ref="I22:I23"/>
+    <mergeCell ref="J22:J23"/>
+    <mergeCell ref="K22:K23"/>
+    <mergeCell ref="L22:L23"/>
+    <mergeCell ref="M22:M23"/>
+    <mergeCell ref="N24:N25"/>
+    <mergeCell ref="O24:O25"/>
+    <mergeCell ref="P24:P25"/>
+    <mergeCell ref="Q24:Q25"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="C26:C27"/>
+    <mergeCell ref="D26:D27"/>
+    <mergeCell ref="E26:E27"/>
+    <mergeCell ref="G26:G27"/>
+    <mergeCell ref="H24:H25"/>
+    <mergeCell ref="I24:I25"/>
+    <mergeCell ref="J24:J25"/>
+    <mergeCell ref="K24:K25"/>
+    <mergeCell ref="L24:L25"/>
+    <mergeCell ref="M24:M25"/>
+    <mergeCell ref="N26:N27"/>
+    <mergeCell ref="O26:O27"/>
+    <mergeCell ref="P26:P27"/>
+    <mergeCell ref="Q26:Q27"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="C28:C29"/>
+    <mergeCell ref="D28:D29"/>
+    <mergeCell ref="E28:E29"/>
+    <mergeCell ref="G28:G29"/>
+    <mergeCell ref="H26:H27"/>
+    <mergeCell ref="I26:I27"/>
+    <mergeCell ref="J26:J27"/>
+    <mergeCell ref="K26:K27"/>
+    <mergeCell ref="L26:L27"/>
+    <mergeCell ref="M26:M27"/>
+    <mergeCell ref="N28:N29"/>
+    <mergeCell ref="O28:O29"/>
+    <mergeCell ref="P28:P29"/>
+    <mergeCell ref="Q28:Q29"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="C31:C32"/>
+    <mergeCell ref="D31:D32"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="G31:G32"/>
+    <mergeCell ref="H28:H29"/>
+    <mergeCell ref="I28:I29"/>
+    <mergeCell ref="J28:J29"/>
+    <mergeCell ref="K28:K29"/>
+    <mergeCell ref="L28:L29"/>
+    <mergeCell ref="M28:M29"/>
+    <mergeCell ref="N31:N32"/>
+    <mergeCell ref="O31:O32"/>
+    <mergeCell ref="P31:P32"/>
+    <mergeCell ref="Q31:Q32"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="C35:C36"/>
+    <mergeCell ref="D35:D36"/>
+    <mergeCell ref="E35:E36"/>
+    <mergeCell ref="G35:G36"/>
+    <mergeCell ref="H31:H32"/>
+    <mergeCell ref="I31:I32"/>
+    <mergeCell ref="J31:J32"/>
+    <mergeCell ref="K31:K32"/>
+    <mergeCell ref="L31:L32"/>
+    <mergeCell ref="M31:M32"/>
+    <mergeCell ref="N35:N36"/>
+    <mergeCell ref="O35:O36"/>
+    <mergeCell ref="P35:P36"/>
+    <mergeCell ref="Q35:Q36"/>
+    <mergeCell ref="A38:A39"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="D38:D39"/>
+    <mergeCell ref="E38:E39"/>
+    <mergeCell ref="G38:G39"/>
+    <mergeCell ref="H35:H36"/>
+    <mergeCell ref="I35:I36"/>
+    <mergeCell ref="J35:J36"/>
+    <mergeCell ref="K35:K36"/>
+    <mergeCell ref="L35:L36"/>
+    <mergeCell ref="M35:M36"/>
+    <mergeCell ref="N38:N39"/>
+    <mergeCell ref="O38:O39"/>
+    <mergeCell ref="P38:P39"/>
+    <mergeCell ref="Q38:Q39"/>
+    <mergeCell ref="H38:H39"/>
+    <mergeCell ref="I38:I39"/>
+    <mergeCell ref="J38:J39"/>
+    <mergeCell ref="K38:K39"/>
+    <mergeCell ref="L38:L39"/>
+    <mergeCell ref="M38:M39"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="N6" r:id="rId1" display="https://mitrphol-my.sharepoint.com/:i:/r/personal/waiyawatc_mitrphol_com/Documents/Investment_Report/Image/%E0%B8%87%E0%B8%B2%E0%B8%99%E0%B9%84%E0%B8%A5%E0%B8%99%E0%B9%8C%E0%B8%97%E0%B9%88%E0%B8%AD%E0%B9%81%E0%B8%AD%E0%B8%A5%E0%B8%81%E0%B8%AD%E0%B8%AE%E0%B8%AD%E0%B8%A5%E0%B9%8C.jpg?csf=1&amp;web=1&amp;e=Rcs21T"/>

</xml_diff>

<commit_message>
Update Excel and Code 2/4/2026
</commit_message>
<xml_diff>
--- a/Investment_Budget_69.xlsx
+++ b/Investment_Budget_69.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="127">
   <si>
     <t>No.</t>
   </si>
@@ -402,6 +402,9 @@
   </si>
   <si>
     <t>ศูนย์กลาง(HUB)วีนัส สถานีขนถ่ายทุ่งหลวง</t>
+  </si>
+  <si>
+    <t>On Process</t>
   </si>
 </sst>
 </file>
@@ -495,7 +498,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -513,9 +516,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -544,6 +544,36 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -898,1843 +928,2113 @@
       </c>
     </row>
     <row r="2" spans="1:17">
-      <c r="A2" s="11">
+      <c r="A2" s="19">
         <v>1</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="20" t="s">
         <v>20</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="G2" s="11" t="s">
+      <c r="G2" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="H2" s="12">
+      <c r="H2" s="21">
         <v>350000</v>
       </c>
-      <c r="I2" s="12">
+      <c r="I2" s="21">
         <v>350000</v>
       </c>
-      <c r="J2" s="11">
+      <c r="J2" s="19">
         <v>0</v>
       </c>
-      <c r="K2" s="11">
+      <c r="K2" s="19">
         <v>50</v>
       </c>
-      <c r="L2" s="11" t="s">
+      <c r="L2" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="M2" s="15">
+      <c r="M2" s="22">
         <v>46113</v>
       </c>
-      <c r="N2" s="11"/>
-      <c r="O2" s="11"/>
-      <c r="P2" s="16"/>
-      <c r="Q2" s="11"/>
+      <c r="N2" s="10"/>
+      <c r="O2" s="10"/>
+      <c r="P2" s="15"/>
+      <c r="Q2" s="10"/>
     </row>
     <row r="3" spans="1:17">
-      <c r="A3" s="11"/>
-      <c r="B3" s="11"/>
-      <c r="C3" s="11"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
+      <c r="A3" s="19"/>
+      <c r="B3" s="19"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
       <c r="F3" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="G3" s="11"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="11"/>
-      <c r="K3" s="11"/>
-      <c r="L3" s="11"/>
-      <c r="M3" s="15"/>
-      <c r="N3" s="11"/>
-      <c r="O3" s="11"/>
-      <c r="P3" s="16"/>
-      <c r="Q3" s="11"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="21"/>
+      <c r="I3" s="21"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="19"/>
+      <c r="L3" s="19"/>
+      <c r="M3" s="22"/>
+      <c r="N3" s="10"/>
+      <c r="O3" s="10"/>
+      <c r="P3" s="15"/>
+      <c r="Q3" s="10"/>
     </row>
     <row r="4" spans="1:17">
-      <c r="A4" s="8">
+      <c r="A4" s="23">
         <v>2</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="E4" s="24" t="s">
         <v>27</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="G4" s="8"/>
-      <c r="H4" s="9">
+      <c r="G4" s="23"/>
+      <c r="H4" s="25">
         <v>460000</v>
       </c>
-      <c r="I4" s="9">
+      <c r="I4" s="25">
         <v>410995.5</v>
       </c>
-      <c r="J4" s="9">
+      <c r="J4" s="25">
         <v>49004.5</v>
       </c>
-      <c r="K4" s="8">
+      <c r="K4" s="23">
         <v>20</v>
       </c>
-      <c r="L4" s="8" t="s">
+      <c r="L4" s="23" t="s">
         <v>24</v>
       </c>
-      <c r="M4" s="14">
+      <c r="M4" s="26">
         <v>46113</v>
       </c>
-      <c r="N4" s="8"/>
-      <c r="O4" s="8"/>
-      <c r="P4" s="8"/>
-      <c r="Q4" s="8"/>
+      <c r="N4" s="7"/>
+      <c r="O4" s="7"/>
+      <c r="P4" s="7"/>
+      <c r="Q4" s="7"/>
     </row>
     <row r="5" spans="1:17">
-      <c r="A5" s="8"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
+      <c r="A5" s="23"/>
+      <c r="B5" s="23"/>
+      <c r="C5" s="23"/>
+      <c r="D5" s="24"/>
+      <c r="E5" s="24"/>
       <c r="F5" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="G5" s="8"/>
-      <c r="H5" s="9"/>
-      <c r="I5" s="9"/>
-      <c r="J5" s="9"/>
-      <c r="K5" s="8"/>
-      <c r="L5" s="8"/>
-      <c r="M5" s="14"/>
-      <c r="N5" s="8"/>
-      <c r="O5" s="8"/>
-      <c r="P5" s="8"/>
-      <c r="Q5" s="8"/>
+      <c r="G5" s="23"/>
+      <c r="H5" s="25"/>
+      <c r="I5" s="25"/>
+      <c r="J5" s="25"/>
+      <c r="K5" s="23"/>
+      <c r="L5" s="23"/>
+      <c r="M5" s="26"/>
+      <c r="N5" s="7"/>
+      <c r="O5" s="7"/>
+      <c r="P5" s="7"/>
+      <c r="Q5" s="7"/>
     </row>
     <row r="6" spans="1:17" ht="58">
-      <c r="A6" s="11">
+      <c r="A6" s="10">
         <v>3</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="F6" s="13" t="s">
+      <c r="F6" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="G6" s="11"/>
-      <c r="H6" s="12">
+      <c r="G6" s="10"/>
+      <c r="H6" s="11">
         <v>130000</v>
       </c>
-      <c r="I6" s="12">
+      <c r="I6" s="11">
         <v>120000</v>
       </c>
-      <c r="J6" s="12">
+      <c r="J6" s="11">
         <v>10000</v>
       </c>
-      <c r="K6" s="11">
+      <c r="K6" s="10">
         <v>100</v>
       </c>
-      <c r="L6" s="11" t="s">
+      <c r="L6" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="M6" s="15">
+      <c r="M6" s="14">
         <v>46113</v>
       </c>
       <c r="N6" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="O6" s="11"/>
-      <c r="P6" s="11"/>
-      <c r="Q6" s="11"/>
+      <c r="O6" s="10"/>
+      <c r="P6" s="10"/>
+      <c r="Q6" s="10"/>
     </row>
     <row r="7" spans="1:17">
-      <c r="A7" s="8">
+      <c r="A7" s="7">
         <v>4</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="E7" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="F7" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="G7" s="8"/>
-      <c r="H7" s="9">
+      <c r="G7" s="7"/>
+      <c r="H7" s="8">
         <v>300000</v>
       </c>
-      <c r="I7" s="9">
+      <c r="I7" s="8">
         <v>280000</v>
       </c>
-      <c r="J7" s="9">
+      <c r="J7" s="8">
         <v>20000</v>
       </c>
-      <c r="K7" s="8">
+      <c r="K7" s="7">
         <v>100</v>
       </c>
-      <c r="L7" s="8" t="s">
+      <c r="L7" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="M7" s="14">
+      <c r="M7" s="13">
         <v>46113</v>
       </c>
-      <c r="N7" s="8"/>
-      <c r="O7" s="8"/>
-      <c r="P7" s="8"/>
-      <c r="Q7" s="8"/>
+      <c r="N7" s="7"/>
+      <c r="O7" s="7"/>
+      <c r="P7" s="7"/>
+      <c r="Q7" s="7"/>
     </row>
     <row r="8" spans="1:17">
-      <c r="A8" s="11">
+      <c r="A8" s="10">
         <v>5</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="C8" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="E8" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="F8" s="13" t="s">
+      <c r="F8" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="G8" s="11"/>
-      <c r="H8" s="12">
+      <c r="G8" s="10"/>
+      <c r="H8" s="11">
         <v>20000</v>
       </c>
-      <c r="I8" s="12">
+      <c r="I8" s="11">
         <v>18614.400000000001</v>
       </c>
-      <c r="J8" s="12">
+      <c r="J8" s="11">
         <v>1385.6</v>
       </c>
-      <c r="K8" s="11">
+      <c r="K8" s="10">
         <v>100</v>
       </c>
-      <c r="L8" s="11" t="s">
+      <c r="L8" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="M8" s="15">
+      <c r="M8" s="14">
         <v>46113</v>
       </c>
       <c r="N8" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="O8" s="11"/>
-      <c r="P8" s="11"/>
-      <c r="Q8" s="11"/>
+      <c r="O8" s="10"/>
+      <c r="P8" s="10"/>
+      <c r="Q8" s="10"/>
     </row>
     <row r="9" spans="1:17">
-      <c r="A9" s="8">
+      <c r="A9" s="23">
         <v>6</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="E9" s="24" t="s">
         <v>44</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="G9" s="8"/>
-      <c r="H9" s="9">
+      <c r="G9" s="23"/>
+      <c r="H9" s="25">
         <v>160000</v>
       </c>
-      <c r="I9" s="9">
+      <c r="I9" s="25">
         <v>160000</v>
       </c>
-      <c r="J9" s="8">
+      <c r="J9" s="23">
         <v>0</v>
       </c>
-      <c r="K9" s="8">
+      <c r="K9" s="23">
         <v>50</v>
       </c>
-      <c r="L9" s="8" t="s">
+      <c r="L9" s="23" t="s">
         <v>24</v>
       </c>
-      <c r="M9" s="14">
+      <c r="M9" s="26">
         <v>46113</v>
       </c>
-      <c r="N9" s="8"/>
-      <c r="O9" s="8"/>
-      <c r="P9" s="8"/>
-      <c r="Q9" s="8"/>
+      <c r="N9" s="7"/>
+      <c r="O9" s="7"/>
+      <c r="P9" s="7"/>
+      <c r="Q9" s="7"/>
     </row>
     <row r="10" spans="1:17">
-      <c r="A10" s="8"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
+      <c r="A10" s="23"/>
+      <c r="B10" s="23"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
       <c r="F10" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="G10" s="8"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="9"/>
-      <c r="J10" s="8"/>
-      <c r="K10" s="8"/>
-      <c r="L10" s="8"/>
-      <c r="M10" s="14"/>
-      <c r="N10" s="8"/>
-      <c r="O10" s="8"/>
-      <c r="P10" s="8"/>
-      <c r="Q10" s="8"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="25"/>
+      <c r="I10" s="25"/>
+      <c r="J10" s="23"/>
+      <c r="K10" s="23"/>
+      <c r="L10" s="23"/>
+      <c r="M10" s="26"/>
+      <c r="N10" s="7"/>
+      <c r="O10" s="7"/>
+      <c r="P10" s="7"/>
+      <c r="Q10" s="7"/>
     </row>
     <row r="11" spans="1:17">
-      <c r="A11" s="11">
+      <c r="A11" s="19">
         <v>7</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="D11" s="13" t="s">
+      <c r="D11" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="E11" s="13" t="s">
+      <c r="E11" s="20" t="s">
         <v>49</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G11" s="11"/>
-      <c r="H11" s="12">
+      <c r="G11" s="19"/>
+      <c r="H11" s="21">
         <v>1490000</v>
       </c>
-      <c r="I11" s="12">
+      <c r="I11" s="21">
         <v>1033230</v>
       </c>
-      <c r="J11" s="12">
+      <c r="J11" s="21">
         <v>456770</v>
       </c>
-      <c r="K11" s="11">
+      <c r="K11" s="19">
         <v>15</v>
       </c>
-      <c r="L11" s="11" t="s">
+      <c r="L11" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="M11" s="15">
+      <c r="M11" s="22">
         <v>46113</v>
       </c>
-      <c r="N11" s="11"/>
-      <c r="O11" s="11"/>
-      <c r="P11" s="11"/>
-      <c r="Q11" s="11"/>
+      <c r="N11" s="10"/>
+      <c r="O11" s="10"/>
+      <c r="P11" s="10"/>
+      <c r="Q11" s="10"/>
     </row>
     <row r="12" spans="1:17" ht="29">
-      <c r="A12" s="11"/>
-      <c r="B12" s="11"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="13"/>
-      <c r="E12" s="13"/>
+      <c r="A12" s="19"/>
+      <c r="B12" s="19"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="20"/>
+      <c r="E12" s="20"/>
       <c r="F12" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="G12" s="11"/>
-      <c r="H12" s="12"/>
-      <c r="I12" s="12"/>
-      <c r="J12" s="12"/>
-      <c r="K12" s="11"/>
-      <c r="L12" s="11"/>
-      <c r="M12" s="15"/>
-      <c r="N12" s="11"/>
-      <c r="O12" s="11"/>
-      <c r="P12" s="11"/>
-      <c r="Q12" s="11"/>
+      <c r="G12" s="19"/>
+      <c r="H12" s="21"/>
+      <c r="I12" s="21"/>
+      <c r="J12" s="21"/>
+      <c r="K12" s="19"/>
+      <c r="L12" s="19"/>
+      <c r="M12" s="22"/>
+      <c r="N12" s="10"/>
+      <c r="O12" s="10"/>
+      <c r="P12" s="10"/>
+      <c r="Q12" s="10"/>
     </row>
     <row r="13" spans="1:17">
-      <c r="A13" s="8">
+      <c r="A13" s="7">
         <v>8</v>
       </c>
-      <c r="B13" s="8" t="s">
+      <c r="B13" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="E13" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="F13" s="10" t="s">
+      <c r="F13" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="G13" s="8"/>
-      <c r="H13" s="9">
+      <c r="G13" s="7"/>
+      <c r="H13" s="8">
         <v>400000</v>
       </c>
-      <c r="I13" s="9">
+      <c r="I13" s="8">
         <v>399690</v>
       </c>
-      <c r="J13" s="8">
+      <c r="J13" s="7">
         <v>310</v>
       </c>
-      <c r="K13" s="8">
+      <c r="K13" s="7">
         <v>10</v>
       </c>
-      <c r="L13" s="8" t="s">
+      <c r="L13" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="M13" s="14">
+      <c r="M13" s="13">
         <v>46113</v>
       </c>
-      <c r="N13" s="8"/>
-      <c r="O13" s="8"/>
-      <c r="P13" s="8"/>
-      <c r="Q13" s="8"/>
+      <c r="N13" s="7"/>
+      <c r="O13" s="7"/>
+      <c r="P13" s="7"/>
+      <c r="Q13" s="7"/>
     </row>
     <row r="14" spans="1:17">
-      <c r="A14" s="11">
+      <c r="A14" s="19">
         <v>9</v>
       </c>
-      <c r="B14" s="11" t="s">
+      <c r="B14" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="C14" s="11" t="s">
+      <c r="C14" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="D14" s="13" t="s">
+      <c r="D14" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="E14" s="13" t="s">
+      <c r="E14" s="20" t="s">
         <v>57</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="G14" s="11"/>
-      <c r="H14" s="12">
+      <c r="G14" s="19"/>
+      <c r="H14" s="21">
         <v>1200000</v>
       </c>
-      <c r="I14" s="12">
+      <c r="I14" s="21">
         <v>1100000</v>
       </c>
-      <c r="J14" s="12">
+      <c r="J14" s="21">
         <v>100000</v>
       </c>
-      <c r="K14" s="11">
+      <c r="K14" s="19">
         <v>10</v>
       </c>
-      <c r="L14" s="11" t="s">
+      <c r="L14" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="M14" s="15">
+      <c r="M14" s="22">
         <v>46104</v>
       </c>
-      <c r="N14" s="11"/>
-      <c r="O14" s="11"/>
-      <c r="P14" s="11"/>
-      <c r="Q14" s="11"/>
+      <c r="N14" s="10"/>
+      <c r="O14" s="10"/>
+      <c r="P14" s="10"/>
+      <c r="Q14" s="10"/>
     </row>
     <row r="15" spans="1:17">
-      <c r="A15" s="11"/>
-      <c r="B15" s="11"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
+      <c r="A15" s="19"/>
+      <c r="B15" s="19"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="20"/>
       <c r="F15" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="G15" s="11"/>
-      <c r="H15" s="12"/>
-      <c r="I15" s="12"/>
-      <c r="J15" s="12"/>
-      <c r="K15" s="11"/>
-      <c r="L15" s="11"/>
-      <c r="M15" s="15"/>
-      <c r="N15" s="11"/>
-      <c r="O15" s="11"/>
-      <c r="P15" s="11"/>
-      <c r="Q15" s="11"/>
+      <c r="G15" s="19"/>
+      <c r="H15" s="21"/>
+      <c r="I15" s="21"/>
+      <c r="J15" s="21"/>
+      <c r="K15" s="19"/>
+      <c r="L15" s="19"/>
+      <c r="M15" s="22"/>
+      <c r="N15" s="10"/>
+      <c r="O15" s="10"/>
+      <c r="P15" s="10"/>
+      <c r="Q15" s="10"/>
     </row>
     <row r="16" spans="1:17">
-      <c r="A16" s="8">
+      <c r="A16" s="23">
         <v>10</v>
       </c>
-      <c r="B16" s="8" t="s">
+      <c r="B16" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C16" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="D16" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="E16" s="10" t="s">
+      <c r="E16" s="24" t="s">
         <v>49</v>
       </c>
       <c r="F16" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="G16" s="8"/>
-      <c r="H16" s="9">
+      <c r="G16" s="23"/>
+      <c r="H16" s="25">
         <v>1430000</v>
       </c>
-      <c r="I16" s="8"/>
-      <c r="J16" s="9">
+      <c r="I16" s="23"/>
+      <c r="J16" s="25">
         <v>1430000</v>
       </c>
-      <c r="K16" s="8">
+      <c r="K16" s="23">
         <v>5</v>
       </c>
-      <c r="L16" s="8" t="s">
+      <c r="L16" s="23" t="s">
         <v>60</v>
       </c>
-      <c r="M16" s="14">
+      <c r="M16" s="26">
         <v>46104</v>
       </c>
-      <c r="N16" s="8"/>
-      <c r="O16" s="8"/>
-      <c r="P16" s="8"/>
-      <c r="Q16" s="8"/>
+      <c r="N16" s="7"/>
+      <c r="O16" s="7"/>
+      <c r="P16" s="7"/>
+      <c r="Q16" s="7"/>
     </row>
     <row r="17" spans="1:17" ht="29">
-      <c r="A17" s="8"/>
-      <c r="B17" s="8"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
+      <c r="A17" s="23"/>
+      <c r="B17" s="23"/>
+      <c r="C17" s="23"/>
+      <c r="D17" s="24"/>
+      <c r="E17" s="24"/>
       <c r="F17" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="G17" s="8"/>
-      <c r="H17" s="9"/>
-      <c r="I17" s="8"/>
-      <c r="J17" s="9"/>
-      <c r="K17" s="8"/>
-      <c r="L17" s="8"/>
-      <c r="M17" s="14"/>
-      <c r="N17" s="8"/>
-      <c r="O17" s="8"/>
-      <c r="P17" s="8"/>
-      <c r="Q17" s="8"/>
+      <c r="G17" s="23"/>
+      <c r="H17" s="25"/>
+      <c r="I17" s="23"/>
+      <c r="J17" s="25"/>
+      <c r="K17" s="23"/>
+      <c r="L17" s="23"/>
+      <c r="M17" s="26"/>
+      <c r="N17" s="7"/>
+      <c r="O17" s="7"/>
+      <c r="P17" s="7"/>
+      <c r="Q17" s="7"/>
     </row>
     <row r="18" spans="1:17">
-      <c r="A18" s="11">
+      <c r="A18" s="10">
         <v>11</v>
       </c>
-      <c r="B18" s="11" t="s">
+      <c r="B18" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="C18" s="11" t="s">
+      <c r="C18" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="D18" s="13" t="s">
+      <c r="D18" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="E18" s="13" t="s">
+      <c r="E18" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="F18" s="13" t="s">
+      <c r="F18" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="G18" s="11"/>
-      <c r="H18" s="12">
+      <c r="G18" s="10"/>
+      <c r="H18" s="11">
         <v>450000</v>
       </c>
-      <c r="I18" s="11"/>
-      <c r="J18" s="12">
+      <c r="I18" s="10"/>
+      <c r="J18" s="11">
         <v>450000</v>
       </c>
-      <c r="K18" s="11"/>
-      <c r="L18" s="11"/>
-      <c r="M18" s="15">
+      <c r="K18" s="10"/>
+      <c r="L18" s="10"/>
+      <c r="M18" s="14">
         <v>46104</v>
       </c>
-      <c r="N18" s="11"/>
-      <c r="O18" s="11"/>
-      <c r="P18" s="11"/>
-      <c r="Q18" s="11" t="s">
+      <c r="N18" s="10"/>
+      <c r="O18" s="10"/>
+      <c r="P18" s="10"/>
+      <c r="Q18" s="10" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="19" spans="1:17">
-      <c r="A19" s="8">
+      <c r="A19" s="23">
         <v>12</v>
       </c>
-      <c r="B19" s="8" t="s">
+      <c r="B19" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="C19" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="D19" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="E19" s="10" t="s">
+      <c r="E19" s="24" t="s">
         <v>49</v>
       </c>
       <c r="F19" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="G19" s="8"/>
-      <c r="H19" s="9">
+      <c r="G19" s="23"/>
+      <c r="H19" s="25">
         <v>920000</v>
       </c>
-      <c r="I19" s="8"/>
-      <c r="J19" s="9">
+      <c r="I19" s="23"/>
+      <c r="J19" s="25">
         <v>920000</v>
       </c>
-      <c r="K19" s="8">
+      <c r="K19" s="23">
         <v>5</v>
       </c>
-      <c r="L19" s="8" t="s">
+      <c r="L19" s="23" t="s">
         <v>60</v>
       </c>
-      <c r="M19" s="14">
+      <c r="M19" s="26">
         <v>46104</v>
       </c>
-      <c r="N19" s="8"/>
-      <c r="O19" s="8"/>
-      <c r="P19" s="8"/>
-      <c r="Q19" s="8"/>
+      <c r="N19" s="7"/>
+      <c r="O19" s="7"/>
+      <c r="P19" s="7"/>
+      <c r="Q19" s="7"/>
     </row>
     <row r="20" spans="1:17" ht="29">
-      <c r="A20" s="8"/>
-      <c r="B20" s="8"/>
-      <c r="C20" s="8"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="10"/>
+      <c r="A20" s="23"/>
+      <c r="B20" s="23"/>
+      <c r="C20" s="23"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="24"/>
       <c r="F20" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="G20" s="8"/>
-      <c r="H20" s="9"/>
-      <c r="I20" s="8"/>
-      <c r="J20" s="9"/>
-      <c r="K20" s="8"/>
-      <c r="L20" s="8"/>
-      <c r="M20" s="14"/>
-      <c r="N20" s="8"/>
-      <c r="O20" s="8"/>
-      <c r="P20" s="8"/>
-      <c r="Q20" s="8"/>
+      <c r="G20" s="23"/>
+      <c r="H20" s="25"/>
+      <c r="I20" s="23"/>
+      <c r="J20" s="25"/>
+      <c r="K20" s="23"/>
+      <c r="L20" s="23"/>
+      <c r="M20" s="26"/>
+      <c r="N20" s="7"/>
+      <c r="O20" s="7"/>
+      <c r="P20" s="7"/>
+      <c r="Q20" s="7"/>
     </row>
     <row r="21" spans="1:17">
-      <c r="A21" s="11">
+      <c r="A21" s="10">
         <v>13</v>
       </c>
-      <c r="B21" s="11" t="s">
+      <c r="B21" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="C21" s="11" t="s">
+      <c r="C21" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="D21" s="13" t="s">
+      <c r="D21" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="E21" s="13" t="s">
+      <c r="E21" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="F21" s="13" t="s">
+      <c r="F21" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="G21" s="11"/>
-      <c r="H21" s="12">
+      <c r="G21" s="10"/>
+      <c r="H21" s="11">
         <v>945000</v>
       </c>
-      <c r="I21" s="11"/>
-      <c r="J21" s="12">
+      <c r="I21" s="10"/>
+      <c r="J21" s="11">
         <v>945000</v>
       </c>
-      <c r="K21" s="11"/>
-      <c r="L21" s="11"/>
-      <c r="M21" s="15">
+      <c r="K21" s="10"/>
+      <c r="L21" s="10"/>
+      <c r="M21" s="14">
         <v>46104</v>
       </c>
-      <c r="N21" s="11"/>
-      <c r="O21" s="11"/>
-      <c r="P21" s="11"/>
-      <c r="Q21" s="11" t="s">
+      <c r="N21" s="10"/>
+      <c r="O21" s="10"/>
+      <c r="P21" s="10"/>
+      <c r="Q21" s="10" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="22" spans="1:17">
-      <c r="A22" s="8">
+      <c r="A22" s="23">
         <v>14</v>
       </c>
-      <c r="B22" s="8" t="s">
+      <c r="B22" s="23" t="s">
         <v>63</v>
       </c>
-      <c r="C22" s="8" t="s">
+      <c r="C22" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="D22" s="24" t="s">
         <v>64</v>
       </c>
-      <c r="E22" s="10" t="s">
+      <c r="E22" s="24" t="s">
         <v>65</v>
       </c>
       <c r="F22" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="G22" s="8" t="s">
+      <c r="G22" s="23" t="s">
         <v>68</v>
       </c>
-      <c r="H22" s="9">
+      <c r="H22" s="25">
         <v>100000</v>
       </c>
-      <c r="I22" s="8"/>
-      <c r="J22" s="9">
+      <c r="I22" s="25">
         <v>100000</v>
       </c>
-      <c r="K22" s="8"/>
-      <c r="L22" s="8"/>
-      <c r="M22" s="8"/>
-      <c r="N22" s="8"/>
-      <c r="O22" s="8"/>
-      <c r="P22" s="8"/>
-      <c r="Q22" s="8"/>
+      <c r="J22" s="23">
+        <v>0</v>
+      </c>
+      <c r="K22" s="23">
+        <v>10</v>
+      </c>
+      <c r="L22" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="M22" s="26">
+        <v>46114</v>
+      </c>
+      <c r="N22" s="7"/>
+      <c r="O22" s="7"/>
+      <c r="P22" s="7"/>
+      <c r="Q22" s="7"/>
     </row>
     <row r="23" spans="1:17">
-      <c r="A23" s="8"/>
-      <c r="B23" s="8"/>
-      <c r="C23" s="8"/>
-      <c r="D23" s="10"/>
-      <c r="E23" s="10"/>
+      <c r="A23" s="23"/>
+      <c r="B23" s="23"/>
+      <c r="C23" s="23"/>
+      <c r="D23" s="24"/>
+      <c r="E23" s="24"/>
       <c r="F23" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="G23" s="8"/>
-      <c r="H23" s="9"/>
-      <c r="I23" s="8"/>
-      <c r="J23" s="9"/>
-      <c r="K23" s="8"/>
-      <c r="L23" s="8"/>
-      <c r="M23" s="8"/>
-      <c r="N23" s="8"/>
-      <c r="O23" s="8"/>
-      <c r="P23" s="8"/>
-      <c r="Q23" s="8"/>
+      <c r="G23" s="23"/>
+      <c r="H23" s="25"/>
+      <c r="I23" s="25"/>
+      <c r="J23" s="23"/>
+      <c r="K23" s="23"/>
+      <c r="L23" s="23"/>
+      <c r="M23" s="26"/>
+      <c r="N23" s="7"/>
+      <c r="O23" s="7"/>
+      <c r="P23" s="7"/>
+      <c r="Q23" s="7"/>
     </row>
     <row r="24" spans="1:17">
-      <c r="A24" s="11">
+      <c r="A24" s="19">
         <v>15</v>
       </c>
-      <c r="B24" s="11" t="s">
+      <c r="B24" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="C24" s="11" t="s">
+      <c r="C24" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="D24" s="13" t="s">
+      <c r="D24" s="20" t="s">
         <v>69</v>
       </c>
-      <c r="E24" s="13" t="s">
+      <c r="E24" s="20" t="s">
         <v>70</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="G24" s="11" t="s">
+      <c r="G24" s="19" t="s">
         <v>73</v>
       </c>
-      <c r="H24" s="12">
+      <c r="H24" s="21">
         <v>370000</v>
       </c>
-      <c r="I24" s="11"/>
-      <c r="J24" s="12">
+      <c r="I24" s="21">
         <v>370000</v>
       </c>
-      <c r="K24" s="11"/>
-      <c r="L24" s="11"/>
-      <c r="M24" s="11"/>
-      <c r="N24" s="11"/>
-      <c r="O24" s="11"/>
-      <c r="P24" s="11"/>
-      <c r="Q24" s="11"/>
+      <c r="J24" s="19">
+        <v>0</v>
+      </c>
+      <c r="K24" s="19">
+        <v>70</v>
+      </c>
+      <c r="L24" s="19" t="s">
+        <v>126</v>
+      </c>
+      <c r="M24" s="22">
+        <v>46114</v>
+      </c>
+      <c r="N24" s="10"/>
+      <c r="O24" s="10"/>
+      <c r="P24" s="10"/>
+      <c r="Q24" s="10"/>
     </row>
     <row r="25" spans="1:17">
-      <c r="A25" s="11"/>
-      <c r="B25" s="11"/>
-      <c r="C25" s="11"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="13"/>
+      <c r="A25" s="19"/>
+      <c r="B25" s="19"/>
+      <c r="C25" s="19"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="20"/>
       <c r="F25" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="G25" s="11"/>
-      <c r="H25" s="12"/>
-      <c r="I25" s="11"/>
-      <c r="J25" s="12"/>
-      <c r="K25" s="11"/>
-      <c r="L25" s="11"/>
-      <c r="M25" s="11"/>
-      <c r="N25" s="11"/>
-      <c r="O25" s="11"/>
-      <c r="P25" s="11"/>
-      <c r="Q25" s="11"/>
+      <c r="G25" s="19"/>
+      <c r="H25" s="21"/>
+      <c r="I25" s="21"/>
+      <c r="J25" s="19"/>
+      <c r="K25" s="19"/>
+      <c r="L25" s="19"/>
+      <c r="M25" s="22"/>
+      <c r="N25" s="10"/>
+      <c r="O25" s="10"/>
+      <c r="P25" s="10"/>
+      <c r="Q25" s="10"/>
     </row>
     <row r="26" spans="1:17">
-      <c r="A26" s="8">
+      <c r="A26" s="23">
         <v>16</v>
       </c>
-      <c r="B26" s="8" t="s">
+      <c r="B26" s="23" t="s">
         <v>63</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="C26" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="D26" s="10" t="s">
+      <c r="D26" s="24" t="s">
         <v>74</v>
       </c>
-      <c r="E26" s="10" t="s">
+      <c r="E26" s="24" t="s">
         <v>75</v>
       </c>
       <c r="F26" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="G26" s="8"/>
-      <c r="H26" s="9">
+      <c r="G26" s="23"/>
+      <c r="H26" s="25">
         <v>2255000</v>
       </c>
-      <c r="I26" s="8"/>
-      <c r="J26" s="9">
-        <v>2255000</v>
-      </c>
-      <c r="K26" s="8"/>
-      <c r="L26" s="8"/>
-      <c r="M26" s="8"/>
-      <c r="N26" s="8"/>
-      <c r="O26" s="8"/>
-      <c r="P26" s="8"/>
-      <c r="Q26" s="8"/>
+      <c r="I26" s="25">
+        <v>2005050</v>
+      </c>
+      <c r="J26" s="25">
+        <v>249950</v>
+      </c>
+      <c r="K26" s="23">
+        <v>10</v>
+      </c>
+      <c r="L26" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="M26" s="26">
+        <v>46114</v>
+      </c>
+      <c r="N26" s="7"/>
+      <c r="O26" s="7"/>
+      <c r="P26" s="7"/>
+      <c r="Q26" s="7"/>
     </row>
     <row r="27" spans="1:17">
-      <c r="A27" s="8"/>
-      <c r="B27" s="8"/>
-      <c r="C27" s="8"/>
-      <c r="D27" s="10"/>
-      <c r="E27" s="10"/>
+      <c r="A27" s="23"/>
+      <c r="B27" s="23"/>
+      <c r="C27" s="23"/>
+      <c r="D27" s="24"/>
+      <c r="E27" s="24"/>
       <c r="F27" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="G27" s="8"/>
-      <c r="H27" s="9"/>
-      <c r="I27" s="8"/>
-      <c r="J27" s="9"/>
-      <c r="K27" s="8"/>
-      <c r="L27" s="8"/>
-      <c r="M27" s="8"/>
-      <c r="N27" s="8"/>
-      <c r="O27" s="8"/>
-      <c r="P27" s="8"/>
-      <c r="Q27" s="8"/>
+      <c r="G27" s="23"/>
+      <c r="H27" s="25"/>
+      <c r="I27" s="25"/>
+      <c r="J27" s="25"/>
+      <c r="K27" s="23"/>
+      <c r="L27" s="23"/>
+      <c r="M27" s="26"/>
+      <c r="N27" s="7"/>
+      <c r="O27" s="7"/>
+      <c r="P27" s="7"/>
+      <c r="Q27" s="7"/>
     </row>
     <row r="28" spans="1:17">
-      <c r="A28" s="11">
+      <c r="A28" s="19">
         <v>17</v>
       </c>
-      <c r="B28" s="11" t="s">
+      <c r="B28" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="C28" s="11" t="s">
+      <c r="C28" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="D28" s="13" t="s">
+      <c r="D28" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="E28" s="13" t="s">
+      <c r="E28" s="20" t="s">
         <v>79</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="G28" s="11"/>
-      <c r="H28" s="12">
+      <c r="G28" s="19"/>
+      <c r="H28" s="21">
         <v>110000</v>
       </c>
-      <c r="I28" s="11"/>
-      <c r="J28" s="12">
+      <c r="I28" s="19">
+        <v>0</v>
+      </c>
+      <c r="J28" s="21">
         <v>110000</v>
       </c>
-      <c r="K28" s="11"/>
-      <c r="L28" s="11"/>
-      <c r="M28" s="11"/>
-      <c r="N28" s="11"/>
-      <c r="O28" s="11"/>
-      <c r="P28" s="11"/>
-      <c r="Q28" s="11"/>
+      <c r="K28" s="19">
+        <v>5</v>
+      </c>
+      <c r="L28" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="M28" s="22">
+        <v>46114</v>
+      </c>
+      <c r="N28" s="10"/>
+      <c r="O28" s="10"/>
+      <c r="P28" s="10"/>
+      <c r="Q28" s="10"/>
     </row>
     <row r="29" spans="1:17">
-      <c r="A29" s="11"/>
-      <c r="B29" s="11"/>
-      <c r="C29" s="11"/>
-      <c r="D29" s="13"/>
-      <c r="E29" s="13"/>
+      <c r="A29" s="19"/>
+      <c r="B29" s="19"/>
+      <c r="C29" s="19"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="20"/>
       <c r="F29" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="G29" s="11"/>
-      <c r="H29" s="12"/>
-      <c r="I29" s="11"/>
-      <c r="J29" s="12"/>
-      <c r="K29" s="11"/>
-      <c r="L29" s="11"/>
-      <c r="M29" s="11"/>
-      <c r="N29" s="11"/>
-      <c r="O29" s="11"/>
-      <c r="P29" s="11"/>
-      <c r="Q29" s="11"/>
+      <c r="G29" s="19"/>
+      <c r="H29" s="21"/>
+      <c r="I29" s="19"/>
+      <c r="J29" s="21"/>
+      <c r="K29" s="19"/>
+      <c r="L29" s="19"/>
+      <c r="M29" s="22"/>
+      <c r="N29" s="10"/>
+      <c r="O29" s="10"/>
+      <c r="P29" s="10"/>
+      <c r="Q29" s="10"/>
     </row>
     <row r="30" spans="1:17">
-      <c r="A30" s="8">
+      <c r="A30" s="7">
         <v>18</v>
       </c>
-      <c r="B30" s="8" t="s">
+      <c r="B30" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="C30" s="8" t="s">
+      <c r="C30" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="D30" s="10" t="s">
+      <c r="D30" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="E30" s="10" t="s">
+      <c r="E30" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="F30" s="10" t="s">
+      <c r="F30" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="G30" s="8" t="s">
+      <c r="G30" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="H30" s="9">
+      <c r="H30" s="8">
         <v>1000000</v>
       </c>
-      <c r="I30" s="8"/>
-      <c r="J30" s="9">
-        <v>1000000</v>
-      </c>
-      <c r="K30" s="8"/>
-      <c r="L30" s="8"/>
-      <c r="M30" s="8"/>
-      <c r="N30" s="8"/>
-      <c r="O30" s="8"/>
-      <c r="P30" s="8"/>
-      <c r="Q30" s="8"/>
+      <c r="I30" s="8">
+        <v>950000</v>
+      </c>
+      <c r="J30" s="8">
+        <v>50000</v>
+      </c>
+      <c r="K30" s="7">
+        <v>10</v>
+      </c>
+      <c r="L30" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="M30" s="13">
+        <v>46114</v>
+      </c>
+      <c r="N30" s="7"/>
+      <c r="O30" s="7"/>
+      <c r="P30" s="7"/>
+      <c r="Q30" s="7"/>
     </row>
     <row r="31" spans="1:17">
-      <c r="A31" s="11">
+      <c r="A31" s="19">
         <v>19</v>
       </c>
-      <c r="B31" s="11" t="s">
+      <c r="B31" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="C31" s="11" t="s">
+      <c r="C31" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="D31" s="13" t="s">
+      <c r="D31" s="20" t="s">
         <v>86</v>
       </c>
-      <c r="E31" s="13" t="s">
+      <c r="E31" s="20" t="s">
         <v>87</v>
       </c>
       <c r="F31" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="G31" s="11"/>
-      <c r="H31" s="12">
+      <c r="G31" s="19"/>
+      <c r="H31" s="21">
         <v>28000</v>
       </c>
-      <c r="I31" s="11"/>
-      <c r="J31" s="12">
-        <v>28000</v>
-      </c>
-      <c r="K31" s="11"/>
-      <c r="L31" s="11"/>
-      <c r="M31" s="11"/>
-      <c r="N31" s="11"/>
-      <c r="O31" s="11"/>
-      <c r="P31" s="11"/>
-      <c r="Q31" s="11"/>
+      <c r="I31" s="21">
+        <v>20250</v>
+      </c>
+      <c r="J31" s="21">
+        <v>7750</v>
+      </c>
+      <c r="K31" s="19">
+        <v>10</v>
+      </c>
+      <c r="L31" s="19" t="s">
+        <v>24</v>
+      </c>
+      <c r="M31" s="22">
+        <v>46114</v>
+      </c>
+      <c r="N31" s="10"/>
+      <c r="O31" s="10"/>
+      <c r="P31" s="10"/>
+      <c r="Q31" s="10"/>
     </row>
     <row r="32" spans="1:17">
-      <c r="A32" s="11"/>
-      <c r="B32" s="11"/>
-      <c r="C32" s="11"/>
-      <c r="D32" s="13"/>
-      <c r="E32" s="13"/>
+      <c r="A32" s="19"/>
+      <c r="B32" s="19"/>
+      <c r="C32" s="19"/>
+      <c r="D32" s="20"/>
+      <c r="E32" s="20"/>
       <c r="F32" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="G32" s="11"/>
-      <c r="H32" s="12"/>
-      <c r="I32" s="11"/>
-      <c r="J32" s="12"/>
-      <c r="K32" s="11"/>
-      <c r="L32" s="11"/>
-      <c r="M32" s="11"/>
-      <c r="N32" s="11"/>
-      <c r="O32" s="11"/>
-      <c r="P32" s="11"/>
-      <c r="Q32" s="11"/>
+      <c r="G32" s="19"/>
+      <c r="H32" s="21"/>
+      <c r="I32" s="21"/>
+      <c r="J32" s="21"/>
+      <c r="K32" s="19"/>
+      <c r="L32" s="19"/>
+      <c r="M32" s="22"/>
+      <c r="N32" s="10"/>
+      <c r="O32" s="10"/>
+      <c r="P32" s="10"/>
+      <c r="Q32" s="10"/>
     </row>
     <row r="33" spans="1:17">
-      <c r="A33" s="8">
+      <c r="A33" s="7">
         <v>20</v>
       </c>
-      <c r="B33" s="8" t="s">
+      <c r="B33" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="C33" s="8" t="s">
+      <c r="C33" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="D33" s="10" t="s">
+      <c r="D33" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="E33" s="10" t="s">
+      <c r="E33" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="F33" s="10" t="s">
+      <c r="F33" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="G33" s="8"/>
-      <c r="H33" s="9">
+      <c r="G33" s="7"/>
+      <c r="H33" s="8">
         <v>140000</v>
       </c>
-      <c r="I33" s="8"/>
-      <c r="J33" s="9">
-        <v>140000</v>
-      </c>
-      <c r="K33" s="8"/>
-      <c r="L33" s="8"/>
-      <c r="M33" s="8"/>
-      <c r="N33" s="8"/>
-      <c r="O33" s="8"/>
-      <c r="P33" s="8"/>
-      <c r="Q33" s="8"/>
+      <c r="I33" s="8">
+        <v>115000</v>
+      </c>
+      <c r="J33" s="8">
+        <v>25000</v>
+      </c>
+      <c r="K33" s="7">
+        <v>80</v>
+      </c>
+      <c r="L33" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="M33" s="13">
+        <v>46114</v>
+      </c>
+      <c r="N33" s="7"/>
+      <c r="O33" s="7"/>
+      <c r="P33" s="7"/>
+      <c r="Q33" s="7"/>
     </row>
     <row r="34" spans="1:17">
-      <c r="A34" s="11">
+      <c r="A34" s="10">
         <v>21</v>
       </c>
-      <c r="B34" s="11" t="s">
+      <c r="B34" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="C34" s="11" t="s">
+      <c r="C34" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="D34" s="13" t="s">
+      <c r="D34" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="E34" s="13" t="s">
+      <c r="E34" s="12" t="s">
         <v>94</v>
       </c>
-      <c r="F34" s="13" t="s">
+      <c r="F34" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="G34" s="11"/>
-      <c r="H34" s="12">
+      <c r="G34" s="10"/>
+      <c r="H34" s="11">
         <v>20000</v>
       </c>
-      <c r="I34" s="11"/>
-      <c r="J34" s="12">
-        <v>20000</v>
-      </c>
-      <c r="K34" s="11"/>
-      <c r="L34" s="11"/>
-      <c r="M34" s="11"/>
-      <c r="N34" s="11"/>
-      <c r="O34" s="11"/>
-      <c r="P34" s="11"/>
-      <c r="Q34" s="11"/>
+      <c r="I34" s="11">
+        <v>18614</v>
+      </c>
+      <c r="J34" s="11">
+        <v>1386</v>
+      </c>
+      <c r="K34" s="10">
+        <v>100</v>
+      </c>
+      <c r="L34" s="10"/>
+      <c r="M34" s="10"/>
+      <c r="N34" s="10"/>
+      <c r="O34" s="10"/>
+      <c r="P34" s="10"/>
+      <c r="Q34" s="10"/>
     </row>
     <row r="35" spans="1:17">
-      <c r="A35" s="8">
+      <c r="A35" s="23">
         <v>22</v>
       </c>
-      <c r="B35" s="8" t="s">
+      <c r="B35" s="23" t="s">
         <v>63</v>
       </c>
-      <c r="C35" s="8" t="s">
+      <c r="C35" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="D35" s="10" t="s">
+      <c r="D35" s="24" t="s">
         <v>95</v>
       </c>
-      <c r="E35" s="10" t="s">
+      <c r="E35" s="24" t="s">
         <v>96</v>
       </c>
       <c r="F35" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="G35" s="8" t="s">
+      <c r="G35" s="23" t="s">
         <v>99</v>
       </c>
-      <c r="H35" s="9">
+      <c r="H35" s="25">
         <v>80000</v>
       </c>
-      <c r="I35" s="8"/>
-      <c r="J35" s="9">
+      <c r="I35" s="23"/>
+      <c r="J35" s="25">
         <v>80000</v>
       </c>
-      <c r="K35" s="8"/>
-      <c r="L35" s="8"/>
-      <c r="M35" s="8"/>
-      <c r="N35" s="8"/>
-      <c r="O35" s="8"/>
-      <c r="P35" s="8"/>
-      <c r="Q35" s="8"/>
+      <c r="K35" s="23"/>
+      <c r="L35" s="23"/>
+      <c r="M35" s="23"/>
+      <c r="N35" s="7"/>
+      <c r="O35" s="7"/>
+      <c r="P35" s="7"/>
+      <c r="Q35" s="7"/>
     </row>
     <row r="36" spans="1:17">
-      <c r="A36" s="8"/>
-      <c r="B36" s="8"/>
-      <c r="C36" s="8"/>
-      <c r="D36" s="10"/>
-      <c r="E36" s="10"/>
+      <c r="A36" s="23"/>
+      <c r="B36" s="23"/>
+      <c r="C36" s="23"/>
+      <c r="D36" s="24"/>
+      <c r="E36" s="24"/>
       <c r="F36" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="G36" s="8"/>
-      <c r="H36" s="9"/>
-      <c r="I36" s="8"/>
-      <c r="J36" s="9"/>
-      <c r="K36" s="8"/>
-      <c r="L36" s="8"/>
-      <c r="M36" s="8"/>
-      <c r="N36" s="8"/>
-      <c r="O36" s="8"/>
-      <c r="P36" s="8"/>
-      <c r="Q36" s="8"/>
+      <c r="G36" s="23"/>
+      <c r="H36" s="25"/>
+      <c r="I36" s="23"/>
+      <c r="J36" s="25"/>
+      <c r="K36" s="23"/>
+      <c r="L36" s="23"/>
+      <c r="M36" s="23"/>
+      <c r="N36" s="7"/>
+      <c r="O36" s="7"/>
+      <c r="P36" s="7"/>
+      <c r="Q36" s="7"/>
     </row>
     <row r="37" spans="1:17">
-      <c r="A37" s="11">
+      <c r="A37" s="10">
         <v>23</v>
       </c>
-      <c r="B37" s="11" t="s">
+      <c r="B37" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="C37" s="11" t="s">
+      <c r="C37" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="D37" s="13" t="s">
+      <c r="D37" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="E37" s="13" t="s">
+      <c r="E37" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="F37" s="13" t="s">
+      <c r="F37" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="G37" s="11"/>
-      <c r="H37" s="12">
+      <c r="G37" s="10"/>
+      <c r="H37" s="11">
         <v>20000</v>
       </c>
-      <c r="I37" s="11"/>
-      <c r="J37" s="12">
+      <c r="I37" s="10"/>
+      <c r="J37" s="11">
         <v>20000</v>
       </c>
-      <c r="K37" s="11"/>
-      <c r="L37" s="11"/>
-      <c r="M37" s="11"/>
-      <c r="N37" s="11"/>
-      <c r="O37" s="11"/>
-      <c r="P37" s="11"/>
-      <c r="Q37" s="11"/>
+      <c r="K37" s="10"/>
+      <c r="L37" s="10"/>
+      <c r="M37" s="10"/>
+      <c r="N37" s="10"/>
+      <c r="O37" s="10"/>
+      <c r="P37" s="10"/>
+      <c r="Q37" s="10"/>
     </row>
     <row r="38" spans="1:17">
-      <c r="A38" s="8">
+      <c r="A38" s="23">
         <v>24</v>
       </c>
-      <c r="B38" s="8" t="s">
+      <c r="B38" s="23" t="s">
         <v>63</v>
       </c>
-      <c r="C38" s="8" t="s">
+      <c r="C38" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="D38" s="10" t="s">
+      <c r="D38" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="E38" s="10" t="s">
+      <c r="E38" s="24" t="s">
         <v>49</v>
       </c>
       <c r="F38" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="G38" s="8"/>
-      <c r="H38" s="9">
+      <c r="G38" s="23"/>
+      <c r="H38" s="25">
         <v>982000</v>
       </c>
-      <c r="I38" s="8"/>
-      <c r="J38" s="9">
+      <c r="I38" s="23"/>
+      <c r="J38" s="25">
         <v>982000</v>
       </c>
-      <c r="K38" s="8"/>
-      <c r="L38" s="8"/>
-      <c r="M38" s="8"/>
-      <c r="N38" s="8"/>
-      <c r="O38" s="8"/>
-      <c r="P38" s="8"/>
-      <c r="Q38" s="8"/>
+      <c r="K38" s="23"/>
+      <c r="L38" s="23"/>
+      <c r="M38" s="23"/>
+      <c r="N38" s="7"/>
+      <c r="O38" s="7"/>
+      <c r="P38" s="7"/>
+      <c r="Q38" s="7"/>
     </row>
     <row r="39" spans="1:17" ht="29">
-      <c r="A39" s="8"/>
-      <c r="B39" s="8"/>
-      <c r="C39" s="8"/>
-      <c r="D39" s="10"/>
-      <c r="E39" s="10"/>
+      <c r="A39" s="23"/>
+      <c r="B39" s="23"/>
+      <c r="C39" s="23"/>
+      <c r="D39" s="24"/>
+      <c r="E39" s="24"/>
       <c r="F39" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="G39" s="8"/>
-      <c r="H39" s="9"/>
-      <c r="I39" s="8"/>
-      <c r="J39" s="9"/>
-      <c r="K39" s="8"/>
-      <c r="L39" s="8"/>
-      <c r="M39" s="8"/>
-      <c r="N39" s="8"/>
-      <c r="O39" s="8"/>
-      <c r="P39" s="8"/>
-      <c r="Q39" s="8"/>
+      <c r="G39" s="23"/>
+      <c r="H39" s="25"/>
+      <c r="I39" s="23"/>
+      <c r="J39" s="25"/>
+      <c r="K39" s="23"/>
+      <c r="L39" s="23"/>
+      <c r="M39" s="23"/>
+      <c r="N39" s="7"/>
+      <c r="O39" s="7"/>
+      <c r="P39" s="7"/>
+      <c r="Q39" s="7"/>
     </row>
     <row r="40" spans="1:17">
-      <c r="A40" s="11">
+      <c r="A40" s="10">
         <v>25</v>
       </c>
-      <c r="B40" s="11" t="s">
+      <c r="B40" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="C40" s="11" t="s">
+      <c r="C40" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="D40" s="13" t="s">
+      <c r="D40" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="E40" s="13" t="s">
+      <c r="E40" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="F40" s="13" t="s">
+      <c r="F40" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="G40" s="11"/>
-      <c r="H40" s="12">
+      <c r="G40" s="10"/>
+      <c r="H40" s="11">
         <v>370000</v>
       </c>
-      <c r="I40" s="11"/>
-      <c r="J40" s="12">
+      <c r="I40" s="10"/>
+      <c r="J40" s="11">
         <v>370000</v>
       </c>
-      <c r="K40" s="11"/>
-      <c r="L40" s="11"/>
-      <c r="M40" s="11"/>
-      <c r="N40" s="11"/>
-      <c r="O40" s="11"/>
-      <c r="P40" s="11"/>
-      <c r="Q40" s="11"/>
+      <c r="K40" s="10"/>
+      <c r="L40" s="10"/>
+      <c r="M40" s="10"/>
+      <c r="N40" s="10"/>
+      <c r="O40" s="10"/>
+      <c r="P40" s="10"/>
+      <c r="Q40" s="10"/>
     </row>
     <row r="41" spans="1:17">
-      <c r="A41" s="8">
+      <c r="A41" s="7">
         <v>26</v>
       </c>
-      <c r="B41" s="8" t="s">
+      <c r="B41" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="C41" s="8" t="s">
+      <c r="C41" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="D41" s="10" t="s">
+      <c r="D41" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="E41" s="8"/>
-      <c r="F41" s="8"/>
-      <c r="G41" s="8"/>
-      <c r="H41" s="9">
+      <c r="E41" s="7"/>
+      <c r="F41" s="7"/>
+      <c r="G41" s="7"/>
+      <c r="H41" s="8">
         <v>2855104</v>
       </c>
-      <c r="I41" s="8"/>
-      <c r="J41" s="9">
+      <c r="I41" s="7"/>
+      <c r="J41" s="8">
         <v>2855104</v>
       </c>
-      <c r="K41" s="8"/>
-      <c r="L41" s="8"/>
-      <c r="M41" s="8"/>
-      <c r="N41" s="8"/>
-      <c r="O41" s="8"/>
-      <c r="P41" s="8"/>
-      <c r="Q41" s="8"/>
+      <c r="K41" s="7"/>
+      <c r="L41" s="7"/>
+      <c r="M41" s="7"/>
+      <c r="N41" s="7"/>
+      <c r="O41" s="7"/>
+      <c r="P41" s="7"/>
+      <c r="Q41" s="7"/>
     </row>
     <row r="42" spans="1:17">
-      <c r="A42" s="11">
+      <c r="A42" s="10">
         <v>27</v>
       </c>
-      <c r="B42" s="11" t="s">
+      <c r="B42" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="C42" s="11" t="s">
+      <c r="C42" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="D42" s="13" t="s">
+      <c r="D42" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="E42" s="11"/>
-      <c r="F42" s="11"/>
-      <c r="G42" s="11"/>
-      <c r="H42" s="12">
+      <c r="E42" s="10"/>
+      <c r="F42" s="10"/>
+      <c r="G42" s="10"/>
+      <c r="H42" s="11">
         <v>2610000</v>
       </c>
-      <c r="I42" s="11"/>
-      <c r="J42" s="12">
+      <c r="I42" s="10"/>
+      <c r="J42" s="11">
         <v>2610000</v>
       </c>
-      <c r="K42" s="11"/>
-      <c r="L42" s="11"/>
-      <c r="M42" s="11"/>
-      <c r="N42" s="11"/>
-      <c r="O42" s="11"/>
-      <c r="P42" s="11"/>
-      <c r="Q42" s="11"/>
+      <c r="K42" s="10"/>
+      <c r="L42" s="10"/>
+      <c r="M42" s="10"/>
+      <c r="N42" s="10"/>
+      <c r="O42" s="10"/>
+      <c r="P42" s="10"/>
+      <c r="Q42" s="10"/>
     </row>
     <row r="43" spans="1:17">
-      <c r="A43" s="8">
+      <c r="A43" s="7">
         <v>28</v>
       </c>
-      <c r="B43" s="8" t="s">
+      <c r="B43" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="C43" s="8" t="s">
+      <c r="C43" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="D43" s="10" t="s">
+      <c r="D43" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="E43" s="8"/>
-      <c r="F43" s="8"/>
-      <c r="G43" s="8"/>
-      <c r="H43" s="9">
+      <c r="E43" s="7"/>
+      <c r="F43" s="7"/>
+      <c r="G43" s="7"/>
+      <c r="H43" s="8">
         <v>3496000</v>
       </c>
-      <c r="I43" s="8"/>
-      <c r="J43" s="9">
+      <c r="I43" s="7"/>
+      <c r="J43" s="8">
         <v>3496000</v>
       </c>
-      <c r="K43" s="8"/>
-      <c r="L43" s="8"/>
-      <c r="M43" s="8"/>
-      <c r="N43" s="8"/>
-      <c r="O43" s="8"/>
-      <c r="P43" s="8"/>
-      <c r="Q43" s="8"/>
+      <c r="K43" s="7"/>
+      <c r="L43" s="7"/>
+      <c r="M43" s="7"/>
+      <c r="N43" s="7"/>
+      <c r="O43" s="7"/>
+      <c r="P43" s="7"/>
+      <c r="Q43" s="7"/>
     </row>
     <row r="44" spans="1:17">
-      <c r="A44" s="11">
+      <c r="A44" s="10">
         <v>29</v>
       </c>
-      <c r="B44" s="11" t="s">
+      <c r="B44" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="C44" s="11" t="s">
+      <c r="C44" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="D44" s="13" t="s">
+      <c r="D44" s="12" t="s">
         <v>107</v>
       </c>
-      <c r="E44" s="11"/>
-      <c r="F44" s="11"/>
-      <c r="G44" s="11"/>
-      <c r="H44" s="12">
+      <c r="E44" s="10"/>
+      <c r="F44" s="10"/>
+      <c r="G44" s="10"/>
+      <c r="H44" s="11">
         <v>600000</v>
       </c>
-      <c r="I44" s="11"/>
-      <c r="J44" s="12">
+      <c r="I44" s="10"/>
+      <c r="J44" s="11">
         <v>600000</v>
       </c>
-      <c r="K44" s="11"/>
-      <c r="L44" s="11"/>
-      <c r="M44" s="11"/>
-      <c r="N44" s="11"/>
-      <c r="O44" s="11"/>
-      <c r="P44" s="11"/>
-      <c r="Q44" s="11"/>
+      <c r="K44" s="10"/>
+      <c r="L44" s="10"/>
+      <c r="M44" s="10"/>
+      <c r="N44" s="10"/>
+      <c r="O44" s="10"/>
+      <c r="P44" s="10"/>
+      <c r="Q44" s="10"/>
     </row>
     <row r="45" spans="1:17">
-      <c r="A45" s="8">
+      <c r="A45" s="7">
         <v>30</v>
       </c>
-      <c r="B45" s="8" t="s">
+      <c r="B45" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="C45" s="8" t="s">
+      <c r="C45" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D45" s="10" t="s">
+      <c r="D45" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="E45" s="8"/>
-      <c r="F45" s="8"/>
-      <c r="G45" s="8"/>
-      <c r="H45" s="9">
+      <c r="E45" s="7"/>
+      <c r="F45" s="7"/>
+      <c r="G45" s="7"/>
+      <c r="H45" s="8">
         <v>640000</v>
       </c>
-      <c r="I45" s="8"/>
-      <c r="J45" s="9">
+      <c r="I45" s="7"/>
+      <c r="J45" s="8">
         <v>640000</v>
       </c>
-      <c r="K45" s="8"/>
-      <c r="L45" s="8"/>
-      <c r="M45" s="8"/>
-      <c r="N45" s="8"/>
-      <c r="O45" s="8"/>
-      <c r="P45" s="8"/>
-      <c r="Q45" s="8"/>
+      <c r="K45" s="7"/>
+      <c r="L45" s="7"/>
+      <c r="M45" s="7"/>
+      <c r="N45" s="7"/>
+      <c r="O45" s="7"/>
+      <c r="P45" s="7"/>
+      <c r="Q45" s="7"/>
     </row>
     <row r="46" spans="1:17">
-      <c r="A46" s="11">
+      <c r="A46" s="10">
         <v>31</v>
       </c>
-      <c r="B46" s="11" t="s">
+      <c r="B46" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="C46" s="11" t="s">
+      <c r="C46" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="D46" s="13" t="s">
+      <c r="D46" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="E46" s="11"/>
-      <c r="F46" s="11"/>
-      <c r="G46" s="11"/>
-      <c r="H46" s="12">
+      <c r="E46" s="10"/>
+      <c r="F46" s="10"/>
+      <c r="G46" s="10"/>
+      <c r="H46" s="11">
         <v>650000</v>
       </c>
-      <c r="I46" s="11"/>
-      <c r="J46" s="12">
+      <c r="I46" s="10"/>
+      <c r="J46" s="11">
         <v>650000</v>
       </c>
-      <c r="K46" s="11"/>
-      <c r="L46" s="11"/>
-      <c r="M46" s="11"/>
-      <c r="N46" s="11"/>
-      <c r="O46" s="11"/>
-      <c r="P46" s="11"/>
-      <c r="Q46" s="11"/>
+      <c r="K46" s="10"/>
+      <c r="L46" s="10"/>
+      <c r="M46" s="10"/>
+      <c r="N46" s="10"/>
+      <c r="O46" s="10"/>
+      <c r="P46" s="10"/>
+      <c r="Q46" s="10"/>
     </row>
     <row r="47" spans="1:17">
-      <c r="A47" s="8">
+      <c r="A47" s="7">
         <v>32</v>
       </c>
-      <c r="B47" s="8" t="s">
+      <c r="B47" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="C47" s="8" t="s">
+      <c r="C47" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="D47" s="10" t="s">
+      <c r="D47" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="E47" s="8"/>
-      <c r="F47" s="8"/>
-      <c r="G47" s="8"/>
-      <c r="H47" s="9">
+      <c r="E47" s="7"/>
+      <c r="F47" s="7"/>
+      <c r="G47" s="7"/>
+      <c r="H47" s="8">
         <v>120000</v>
       </c>
-      <c r="I47" s="8"/>
-      <c r="J47" s="9">
+      <c r="I47" s="7"/>
+      <c r="J47" s="8">
         <v>120000</v>
       </c>
-      <c r="K47" s="8"/>
-      <c r="L47" s="8"/>
-      <c r="M47" s="8"/>
-      <c r="N47" s="8"/>
-      <c r="O47" s="8"/>
-      <c r="P47" s="8"/>
-      <c r="Q47" s="8"/>
+      <c r="K47" s="7"/>
+      <c r="L47" s="7"/>
+      <c r="M47" s="7"/>
+      <c r="N47" s="7"/>
+      <c r="O47" s="7"/>
+      <c r="P47" s="7"/>
+      <c r="Q47" s="7"/>
     </row>
     <row r="48" spans="1:17">
-      <c r="A48" s="11">
+      <c r="A48" s="10">
         <v>33</v>
       </c>
-      <c r="B48" s="11" t="s">
+      <c r="B48" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="C48" s="11" t="s">
+      <c r="C48" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="D48" s="13" t="s">
+      <c r="D48" s="12" t="s">
         <v>111</v>
       </c>
-      <c r="E48" s="11"/>
-      <c r="F48" s="11"/>
-      <c r="G48" s="11"/>
-      <c r="H48" s="12">
+      <c r="E48" s="10"/>
+      <c r="F48" s="10"/>
+      <c r="G48" s="10"/>
+      <c r="H48" s="11">
         <v>222200</v>
       </c>
-      <c r="I48" s="11"/>
-      <c r="J48" s="12">
+      <c r="I48" s="10"/>
+      <c r="J48" s="11">
         <v>222200</v>
       </c>
-      <c r="K48" s="11"/>
-      <c r="L48" s="11"/>
-      <c r="M48" s="11"/>
-      <c r="N48" s="11"/>
-      <c r="O48" s="11"/>
-      <c r="P48" s="11"/>
-      <c r="Q48" s="11"/>
+      <c r="K48" s="10"/>
+      <c r="L48" s="10"/>
+      <c r="M48" s="10"/>
+      <c r="N48" s="10"/>
+      <c r="O48" s="10"/>
+      <c r="P48" s="10"/>
+      <c r="Q48" s="10"/>
     </row>
     <row r="49" spans="1:17">
-      <c r="A49" s="8">
+      <c r="A49" s="7">
         <v>34</v>
       </c>
-      <c r="B49" s="8" t="s">
+      <c r="B49" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="C49" s="8" t="s">
+      <c r="C49" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D49" s="10" t="s">
+      <c r="D49" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="E49" s="8"/>
-      <c r="F49" s="8"/>
-      <c r="G49" s="8"/>
-      <c r="H49" s="9">
+      <c r="E49" s="7"/>
+      <c r="F49" s="7"/>
+      <c r="G49" s="7"/>
+      <c r="H49" s="8">
         <v>900000</v>
       </c>
-      <c r="I49" s="8"/>
-      <c r="J49" s="9">
+      <c r="I49" s="7"/>
+      <c r="J49" s="8">
         <v>900000</v>
       </c>
-      <c r="K49" s="8"/>
-      <c r="L49" s="8"/>
-      <c r="M49" s="8"/>
-      <c r="N49" s="8"/>
-      <c r="O49" s="8"/>
-      <c r="P49" s="8"/>
-      <c r="Q49" s="8"/>
+      <c r="K49" s="7"/>
+      <c r="L49" s="7"/>
+      <c r="M49" s="7"/>
+      <c r="N49" s="7"/>
+      <c r="O49" s="7"/>
+      <c r="P49" s="7"/>
+      <c r="Q49" s="7"/>
     </row>
     <row r="50" spans="1:17">
-      <c r="A50" s="11">
+      <c r="A50" s="10">
         <v>35</v>
       </c>
-      <c r="B50" s="11" t="s">
+      <c r="B50" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="C50" s="11" t="s">
+      <c r="C50" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="D50" s="13" t="s">
+      <c r="D50" s="12" t="s">
         <v>113</v>
       </c>
-      <c r="E50" s="11"/>
-      <c r="F50" s="11"/>
-      <c r="G50" s="11"/>
-      <c r="H50" s="12">
+      <c r="E50" s="10"/>
+      <c r="F50" s="10"/>
+      <c r="G50" s="10"/>
+      <c r="H50" s="11">
         <v>278500</v>
       </c>
-      <c r="I50" s="11"/>
-      <c r="J50" s="12">
+      <c r="I50" s="10"/>
+      <c r="J50" s="11">
         <v>278500</v>
       </c>
-      <c r="K50" s="11"/>
-      <c r="L50" s="11"/>
-      <c r="M50" s="11"/>
-      <c r="N50" s="11"/>
-      <c r="O50" s="11"/>
-      <c r="P50" s="11"/>
-      <c r="Q50" s="11"/>
+      <c r="K50" s="10"/>
+      <c r="L50" s="10"/>
+      <c r="M50" s="10"/>
+      <c r="N50" s="10"/>
+      <c r="O50" s="10"/>
+      <c r="P50" s="10"/>
+      <c r="Q50" s="10"/>
     </row>
     <row r="51" spans="1:17">
-      <c r="A51" s="8">
+      <c r="A51" s="7">
         <v>36</v>
       </c>
-      <c r="B51" s="8" t="s">
+      <c r="B51" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="C51" s="8" t="s">
+      <c r="C51" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="D51" s="10" t="s">
+      <c r="D51" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="E51" s="8"/>
-      <c r="F51" s="8"/>
-      <c r="G51" s="8"/>
-      <c r="H51" s="9">
+      <c r="E51" s="7"/>
+      <c r="F51" s="7"/>
+      <c r="G51" s="7"/>
+      <c r="H51" s="8">
         <v>225000</v>
       </c>
-      <c r="I51" s="8"/>
-      <c r="J51" s="9">
+      <c r="I51" s="7"/>
+      <c r="J51" s="8">
         <v>225000</v>
       </c>
-      <c r="K51" s="8"/>
-      <c r="L51" s="8"/>
-      <c r="M51" s="8"/>
-      <c r="N51" s="8"/>
-      <c r="O51" s="8"/>
-      <c r="P51" s="8"/>
-      <c r="Q51" s="8"/>
+      <c r="K51" s="7"/>
+      <c r="L51" s="7"/>
+      <c r="M51" s="7"/>
+      <c r="N51" s="7"/>
+      <c r="O51" s="7"/>
+      <c r="P51" s="7"/>
+      <c r="Q51" s="7"/>
     </row>
     <row r="52" spans="1:17">
-      <c r="A52" s="11">
+      <c r="A52" s="10">
         <v>37</v>
       </c>
-      <c r="B52" s="11" t="s">
+      <c r="B52" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="C52" s="11" t="s">
+      <c r="C52" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="D52" s="13" t="s">
+      <c r="D52" s="12" t="s">
         <v>115</v>
       </c>
-      <c r="E52" s="11"/>
-      <c r="F52" s="11"/>
-      <c r="G52" s="11"/>
-      <c r="H52" s="12">
+      <c r="E52" s="10"/>
+      <c r="F52" s="10"/>
+      <c r="G52" s="10"/>
+      <c r="H52" s="11">
         <v>85000</v>
       </c>
-      <c r="I52" s="11"/>
-      <c r="J52" s="12">
+      <c r="I52" s="10"/>
+      <c r="J52" s="11">
         <v>85000</v>
       </c>
-      <c r="K52" s="11"/>
-      <c r="L52" s="11"/>
-      <c r="M52" s="11"/>
-      <c r="N52" s="11"/>
-      <c r="O52" s="11"/>
-      <c r="P52" s="11"/>
-      <c r="Q52" s="11"/>
+      <c r="K52" s="10"/>
+      <c r="L52" s="10"/>
+      <c r="M52" s="10"/>
+      <c r="N52" s="10"/>
+      <c r="O52" s="10"/>
+      <c r="P52" s="10"/>
+      <c r="Q52" s="10"/>
     </row>
     <row r="53" spans="1:17">
-      <c r="A53" s="8">
+      <c r="A53" s="7">
         <v>38</v>
       </c>
-      <c r="B53" s="8" t="s">
+      <c r="B53" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="C53" s="8" t="s">
+      <c r="C53" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="D53" s="10" t="s">
+      <c r="D53" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="E53" s="8" t="s">
+      <c r="E53" s="17" t="s">
         <v>118</v>
       </c>
-      <c r="F53" s="8"/>
-      <c r="G53" s="8"/>
-      <c r="H53" s="9">
+      <c r="F53" s="7"/>
+      <c r="G53" s="7"/>
+      <c r="H53" s="8">
         <v>1800000</v>
       </c>
-      <c r="I53" s="8"/>
-      <c r="J53" s="9">
+      <c r="I53" s="7"/>
+      <c r="J53" s="8">
         <v>1800000</v>
       </c>
-      <c r="K53" s="8"/>
-      <c r="L53" s="8"/>
-      <c r="M53" s="8"/>
-      <c r="N53" s="8"/>
-      <c r="O53" s="8"/>
-      <c r="P53" s="8"/>
-      <c r="Q53" s="8"/>
+      <c r="K53" s="7"/>
+      <c r="L53" s="7"/>
+      <c r="M53" s="7"/>
+      <c r="N53" s="7"/>
+      <c r="O53" s="7"/>
+      <c r="P53" s="7"/>
+      <c r="Q53" s="7"/>
     </row>
     <row r="54" spans="1:17">
-      <c r="A54" s="11">
+      <c r="A54" s="10">
         <v>39</v>
       </c>
-      <c r="B54" s="11" t="s">
+      <c r="B54" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="C54" s="11" t="s">
+      <c r="C54" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="D54" s="11" t="s">
+      <c r="D54" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="E54" s="11" t="s">
+      <c r="E54" s="18" t="s">
         <v>120</v>
       </c>
-      <c r="F54" s="11"/>
-      <c r="G54" s="11"/>
-      <c r="H54" s="12">
+      <c r="F54" s="10"/>
+      <c r="G54" s="10"/>
+      <c r="H54" s="11">
         <v>1120000</v>
       </c>
-      <c r="I54" s="11"/>
-      <c r="J54" s="12">
+      <c r="I54" s="10"/>
+      <c r="J54" s="11">
         <v>1120000</v>
       </c>
-      <c r="K54" s="11"/>
-      <c r="L54" s="11"/>
-      <c r="M54" s="11"/>
-      <c r="N54" s="11"/>
-      <c r="O54" s="11"/>
-      <c r="P54" s="11"/>
-      <c r="Q54" s="11"/>
+      <c r="K54" s="10"/>
+      <c r="L54" s="10"/>
+      <c r="M54" s="10"/>
+      <c r="N54" s="10"/>
+      <c r="O54" s="10"/>
+      <c r="P54" s="10"/>
+      <c r="Q54" s="10"/>
     </row>
     <row r="55" spans="1:17">
-      <c r="A55" s="8">
+      <c r="A55" s="7">
         <v>40</v>
       </c>
-      <c r="B55" s="8" t="s">
+      <c r="B55" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="C55" s="8" t="s">
+      <c r="C55" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="D55" s="8" t="s">
+      <c r="D55" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="E55" s="8" t="s">
+      <c r="E55" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="F55" s="8"/>
-      <c r="G55" s="8"/>
-      <c r="H55" s="9">
+      <c r="F55" s="7"/>
+      <c r="G55" s="7"/>
+      <c r="H55" s="8">
         <v>860000</v>
       </c>
-      <c r="I55" s="8"/>
-      <c r="J55" s="9">
+      <c r="I55" s="7"/>
+      <c r="J55" s="8">
         <v>860000</v>
       </c>
-      <c r="K55" s="8"/>
-      <c r="L55" s="8"/>
-      <c r="M55" s="8"/>
-      <c r="N55" s="8"/>
-      <c r="O55" s="8"/>
-      <c r="P55" s="8"/>
-      <c r="Q55" s="8"/>
+      <c r="K55" s="7"/>
+      <c r="L55" s="7"/>
+      <c r="M55" s="7"/>
+      <c r="N55" s="7"/>
+      <c r="O55" s="7"/>
+      <c r="P55" s="7"/>
+      <c r="Q55" s="7"/>
     </row>
     <row r="56" spans="1:17">
-      <c r="A56" s="6">
+      <c r="A56" s="10">
         <v>41</v>
       </c>
-      <c r="B56" s="6" t="s">
+      <c r="B56" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="C56" s="6" t="s">
+      <c r="C56" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="D56" s="6" t="s">
+      <c r="D56" s="12" t="s">
         <v>123</v>
       </c>
-      <c r="E56" s="6" t="s">
+      <c r="E56" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="F56" s="6"/>
-      <c r="G56" s="6"/>
-      <c r="H56" s="7">
+      <c r="F56" s="10"/>
+      <c r="G56" s="10"/>
+      <c r="H56" s="11">
         <v>500000</v>
       </c>
-      <c r="I56" s="7"/>
-      <c r="J56" s="7">
+      <c r="I56" s="10"/>
+      <c r="J56" s="11">
         <v>500000</v>
       </c>
-      <c r="K56" s="6"/>
-      <c r="L56" s="6"/>
-      <c r="M56" s="6"/>
+      <c r="K56" s="10"/>
+      <c r="L56" s="10"/>
+      <c r="M56" s="10"/>
       <c r="N56" s="6"/>
       <c r="O56" s="6"/>
       <c r="P56" s="6"/>
       <c r="Q56" s="6"/>
     </row>
     <row r="57" spans="1:17">
-      <c r="A57">
+      <c r="A57" s="7">
         <v>42</v>
       </c>
-      <c r="B57" t="s">
+      <c r="B57" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="C57" t="s">
+      <c r="C57" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="D57" t="s">
+      <c r="D57" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="H57" s="17">
+      <c r="E57" s="17"/>
+      <c r="F57" s="7"/>
+      <c r="G57" s="7"/>
+      <c r="H57" s="8">
         <v>380000</v>
       </c>
-      <c r="J57" s="17">
+      <c r="I57" s="7"/>
+      <c r="J57" s="8">
         <v>380000</v>
       </c>
+      <c r="K57" s="7"/>
+      <c r="L57" s="7"/>
+      <c r="M57" s="7"/>
     </row>
     <row r="58" spans="1:17">
-      <c r="A58">
+      <c r="A58" s="10">
         <v>43</v>
       </c>
-      <c r="J58">
+      <c r="B58" s="10"/>
+      <c r="C58" s="10"/>
+      <c r="D58" s="10"/>
+      <c r="E58" s="10"/>
+      <c r="F58" s="10"/>
+      <c r="G58" s="10"/>
+      <c r="H58" s="10"/>
+      <c r="I58" s="10"/>
+      <c r="J58" s="10">
         <v>0</v>
       </c>
+      <c r="K58" s="10"/>
+      <c r="L58" s="10"/>
+      <c r="M58" s="10"/>
     </row>
     <row r="59" spans="1:17">
-      <c r="A59">
+      <c r="A59" s="7">
         <v>44</v>
       </c>
-      <c r="J59">
+      <c r="B59" s="7"/>
+      <c r="C59" s="7"/>
+      <c r="D59" s="7"/>
+      <c r="E59" s="7"/>
+      <c r="F59" s="7"/>
+      <c r="G59" s="7"/>
+      <c r="H59" s="7"/>
+      <c r="I59" s="7"/>
+      <c r="J59" s="7">
         <v>0</v>
       </c>
+      <c r="K59" s="7"/>
+      <c r="L59" s="7"/>
+      <c r="M59" s="7"/>
     </row>
     <row r="60" spans="1:17">
-      <c r="A60">
+      <c r="A60" s="10">
         <v>45</v>
       </c>
-      <c r="J60">
+      <c r="B60" s="10"/>
+      <c r="C60" s="10"/>
+      <c r="D60" s="10"/>
+      <c r="E60" s="10"/>
+      <c r="F60" s="10"/>
+      <c r="G60" s="10"/>
+      <c r="H60" s="10"/>
+      <c r="I60" s="10"/>
+      <c r="J60" s="10">
         <v>0</v>
       </c>
+      <c r="K60" s="10"/>
+      <c r="L60" s="10"/>
+      <c r="M60" s="10"/>
     </row>
     <row r="61" spans="1:17">
       <c r="A61" t="s">
         <v>116</v>
       </c>
-      <c r="H61" s="17">
+      <c r="H61" s="16">
         <v>31071804</v>
       </c>
-      <c r="I61" s="17">
+      <c r="I61" s="16">
         <v>3872529.9</v>
       </c>
-      <c r="J61" s="17">
+      <c r="J61" s="16">
         <v>27199274.100000001</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="168">
+    <mergeCell ref="H38:H39"/>
+    <mergeCell ref="I38:I39"/>
+    <mergeCell ref="J38:J39"/>
+    <mergeCell ref="K38:K39"/>
+    <mergeCell ref="L38:L39"/>
+    <mergeCell ref="M38:M39"/>
+    <mergeCell ref="A38:A39"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="D38:D39"/>
+    <mergeCell ref="E38:E39"/>
+    <mergeCell ref="G38:G39"/>
+    <mergeCell ref="H35:H36"/>
+    <mergeCell ref="I35:I36"/>
+    <mergeCell ref="J35:J36"/>
+    <mergeCell ref="K35:K36"/>
+    <mergeCell ref="L35:L36"/>
+    <mergeCell ref="M35:M36"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="C35:C36"/>
+    <mergeCell ref="D35:D36"/>
+    <mergeCell ref="E35:E36"/>
+    <mergeCell ref="G35:G36"/>
+    <mergeCell ref="H31:H32"/>
+    <mergeCell ref="I31:I32"/>
+    <mergeCell ref="J31:J32"/>
+    <mergeCell ref="K31:K32"/>
+    <mergeCell ref="L31:L32"/>
+    <mergeCell ref="M31:M32"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="C31:C32"/>
+    <mergeCell ref="D31:D32"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="G31:G32"/>
+    <mergeCell ref="H28:H29"/>
+    <mergeCell ref="I28:I29"/>
+    <mergeCell ref="J28:J29"/>
+    <mergeCell ref="K28:K29"/>
+    <mergeCell ref="L28:L29"/>
+    <mergeCell ref="M28:M29"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="C28:C29"/>
+    <mergeCell ref="D28:D29"/>
+    <mergeCell ref="E28:E29"/>
+    <mergeCell ref="G28:G29"/>
+    <mergeCell ref="H26:H27"/>
+    <mergeCell ref="I26:I27"/>
+    <mergeCell ref="J26:J27"/>
+    <mergeCell ref="K26:K27"/>
+    <mergeCell ref="L26:L27"/>
+    <mergeCell ref="M26:M27"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="C26:C27"/>
+    <mergeCell ref="D26:D27"/>
+    <mergeCell ref="E26:E27"/>
+    <mergeCell ref="G26:G27"/>
+    <mergeCell ref="H24:H25"/>
+    <mergeCell ref="I24:I25"/>
+    <mergeCell ref="J24:J25"/>
+    <mergeCell ref="K24:K25"/>
+    <mergeCell ref="L24:L25"/>
+    <mergeCell ref="M24:M25"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="E24:E25"/>
+    <mergeCell ref="G24:G25"/>
+    <mergeCell ref="H22:H23"/>
+    <mergeCell ref="I22:I23"/>
+    <mergeCell ref="J22:J23"/>
+    <mergeCell ref="K22:K23"/>
+    <mergeCell ref="L22:L23"/>
+    <mergeCell ref="M22:M23"/>
+    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="D22:D23"/>
+    <mergeCell ref="E22:E23"/>
+    <mergeCell ref="G22:G23"/>
+    <mergeCell ref="H19:H20"/>
+    <mergeCell ref="I19:I20"/>
+    <mergeCell ref="J19:J20"/>
+    <mergeCell ref="K19:K20"/>
+    <mergeCell ref="L19:L20"/>
+    <mergeCell ref="M19:M20"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="G19:G20"/>
+    <mergeCell ref="H16:H17"/>
+    <mergeCell ref="I16:I17"/>
+    <mergeCell ref="J16:J17"/>
+    <mergeCell ref="K16:K17"/>
+    <mergeCell ref="L16:L17"/>
+    <mergeCell ref="M16:M17"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="E16:E17"/>
+    <mergeCell ref="G16:G17"/>
+    <mergeCell ref="H14:H15"/>
+    <mergeCell ref="I14:I15"/>
+    <mergeCell ref="J14:J15"/>
+    <mergeCell ref="K14:K15"/>
+    <mergeCell ref="L14:L15"/>
+    <mergeCell ref="M14:M15"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="E14:E15"/>
+    <mergeCell ref="G14:G15"/>
+    <mergeCell ref="H11:H12"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="K11:K12"/>
+    <mergeCell ref="L11:L12"/>
+    <mergeCell ref="M11:M12"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="G11:G12"/>
+    <mergeCell ref="H9:H10"/>
+    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="K9:K10"/>
+    <mergeCell ref="L9:L10"/>
+    <mergeCell ref="M9:M10"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="I4:I5"/>
+    <mergeCell ref="J4:J5"/>
+    <mergeCell ref="K4:K5"/>
+    <mergeCell ref="L4:L5"/>
+    <mergeCell ref="M4:M5"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="G4:G5"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="J2:J3"/>
+    <mergeCell ref="K2:K3"/>
+    <mergeCell ref="L2:L3"/>
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="G2:G3"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update image and excel 2/4/2026
</commit_message>
<xml_diff>
--- a/Investment_Budget_69.xlsx
+++ b/Investment_Budget_69.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="127">
   <si>
     <t>No.</t>
   </si>
@@ -498,7 +498,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -521,25 +521,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -570,6 +552,30 @@
     </xf>
     <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -928,107 +934,107 @@
       </c>
     </row>
     <row r="2" spans="1:17">
-      <c r="A2" s="19">
+      <c r="A2" s="25">
         <v>1</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="19" t="s">
+      <c r="C2" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="20" t="s">
+      <c r="D2" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="20" t="s">
+      <c r="E2" s="27" t="s">
         <v>20</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="G2" s="19" t="s">
+      <c r="G2" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="H2" s="21">
+      <c r="H2" s="24">
         <v>350000</v>
       </c>
-      <c r="I2" s="21">
+      <c r="I2" s="24">
         <v>350000</v>
       </c>
-      <c r="J2" s="19">
+      <c r="J2" s="25">
         <v>0</v>
       </c>
-      <c r="K2" s="19">
+      <c r="K2" s="25">
         <v>50</v>
       </c>
-      <c r="L2" s="19" t="s">
+      <c r="L2" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="M2" s="22">
+      <c r="M2" s="26">
         <v>46113</v>
       </c>
-      <c r="N2" s="10"/>
-      <c r="O2" s="10"/>
-      <c r="P2" s="15"/>
-      <c r="Q2" s="10"/>
+      <c r="N2" s="8"/>
+      <c r="O2" s="8"/>
+      <c r="P2" s="9"/>
+      <c r="Q2" s="8"/>
     </row>
     <row r="3" spans="1:17">
-      <c r="A3" s="19"/>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
+      <c r="A3" s="25"/>
+      <c r="B3" s="25"/>
+      <c r="C3" s="25"/>
+      <c r="D3" s="27"/>
+      <c r="E3" s="27"/>
       <c r="F3" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="G3" s="19"/>
-      <c r="H3" s="21"/>
-      <c r="I3" s="21"/>
-      <c r="J3" s="19"/>
-      <c r="K3" s="19"/>
-      <c r="L3" s="19"/>
-      <c r="M3" s="22"/>
-      <c r="N3" s="10"/>
-      <c r="O3" s="10"/>
-      <c r="P3" s="15"/>
-      <c r="Q3" s="10"/>
+      <c r="G3" s="25"/>
+      <c r="H3" s="24"/>
+      <c r="I3" s="24"/>
+      <c r="J3" s="25"/>
+      <c r="K3" s="25"/>
+      <c r="L3" s="25"/>
+      <c r="M3" s="26"/>
+      <c r="N3" s="8"/>
+      <c r="O3" s="8"/>
+      <c r="P3" s="9"/>
+      <c r="Q3" s="8"/>
     </row>
     <row r="4" spans="1:17">
-      <c r="A4" s="23">
+      <c r="A4" s="22">
         <v>2</v>
       </c>
-      <c r="B4" s="23" t="s">
+      <c r="B4" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="23" t="s">
+      <c r="C4" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="24" t="s">
+      <c r="D4" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="E4" s="24" t="s">
+      <c r="E4" s="23" t="s">
         <v>27</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="G4" s="23"/>
-      <c r="H4" s="25">
+      <c r="G4" s="22"/>
+      <c r="H4" s="21">
         <v>460000</v>
       </c>
-      <c r="I4" s="25">
+      <c r="I4" s="21">
         <v>410995.5</v>
       </c>
-      <c r="J4" s="25">
+      <c r="J4" s="21">
         <v>49004.5</v>
       </c>
-      <c r="K4" s="23">
+      <c r="K4" s="22">
         <v>20</v>
       </c>
-      <c r="L4" s="23" t="s">
+      <c r="L4" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="M4" s="26">
+      <c r="M4" s="28">
         <v>46113</v>
       </c>
       <c r="N4" s="7"/>
@@ -1037,107 +1043,107 @@
       <c r="Q4" s="7"/>
     </row>
     <row r="5" spans="1:17">
-      <c r="A5" s="23"/>
-      <c r="B5" s="23"/>
-      <c r="C5" s="23"/>
-      <c r="D5" s="24"/>
-      <c r="E5" s="24"/>
+      <c r="A5" s="22"/>
+      <c r="B5" s="22"/>
+      <c r="C5" s="22"/>
+      <c r="D5" s="23"/>
+      <c r="E5" s="23"/>
       <c r="F5" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="G5" s="23"/>
-      <c r="H5" s="25"/>
-      <c r="I5" s="25"/>
-      <c r="J5" s="25"/>
-      <c r="K5" s="23"/>
-      <c r="L5" s="23"/>
-      <c r="M5" s="26"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="21"/>
+      <c r="I5" s="21"/>
+      <c r="J5" s="21"/>
+      <c r="K5" s="22"/>
+      <c r="L5" s="22"/>
+      <c r="M5" s="28"/>
       <c r="N5" s="7"/>
       <c r="O5" s="7"/>
       <c r="P5" s="7"/>
       <c r="Q5" s="7"/>
     </row>
     <row r="6" spans="1:17" ht="58">
-      <c r="A6" s="10">
+      <c r="A6" s="13">
         <v>3</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="12" t="s">
+      <c r="D6" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="E6" s="12" t="s">
+      <c r="E6" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="F6" s="12" t="s">
+      <c r="F6" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="G6" s="10"/>
-      <c r="H6" s="11">
+      <c r="G6" s="13"/>
+      <c r="H6" s="15">
         <v>130000</v>
       </c>
-      <c r="I6" s="11">
+      <c r="I6" s="15">
         <v>120000</v>
       </c>
-      <c r="J6" s="11">
+      <c r="J6" s="15">
         <v>10000</v>
       </c>
-      <c r="K6" s="10">
+      <c r="K6" s="13">
         <v>100</v>
       </c>
-      <c r="L6" s="10" t="s">
+      <c r="L6" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="M6" s="14">
+      <c r="M6" s="16">
         <v>46113</v>
       </c>
       <c r="N6" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="O6" s="10"/>
-      <c r="P6" s="10"/>
-      <c r="Q6" s="10"/>
+      <c r="O6" s="8"/>
+      <c r="P6" s="8"/>
+      <c r="Q6" s="8"/>
     </row>
     <row r="7" spans="1:17">
-      <c r="A7" s="7">
+      <c r="A7" s="17">
         <v>4</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="D7" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="F7" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="G7" s="7"/>
-      <c r="H7" s="8">
+      <c r="G7" s="17"/>
+      <c r="H7" s="19">
         <v>300000</v>
       </c>
-      <c r="I7" s="8">
+      <c r="I7" s="19">
         <v>280000</v>
       </c>
-      <c r="J7" s="8">
+      <c r="J7" s="19">
         <v>20000</v>
       </c>
-      <c r="K7" s="7">
+      <c r="K7" s="17">
         <v>100</v>
       </c>
-      <c r="L7" s="7" t="s">
+      <c r="L7" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="M7" s="13">
+      <c r="M7" s="20">
         <v>46113</v>
       </c>
       <c r="N7" s="7"/>
@@ -1146,86 +1152,86 @@
       <c r="Q7" s="7"/>
     </row>
     <row r="8" spans="1:17">
-      <c r="A8" s="10">
+      <c r="A8" s="13">
         <v>5</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="12" t="s">
+      <c r="D8" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="E8" s="12" t="s">
+      <c r="E8" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="F8" s="12" t="s">
+      <c r="F8" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="G8" s="10"/>
-      <c r="H8" s="11">
+      <c r="G8" s="13"/>
+      <c r="H8" s="15">
         <v>20000</v>
       </c>
-      <c r="I8" s="11">
+      <c r="I8" s="15">
         <v>18614.400000000001</v>
       </c>
-      <c r="J8" s="11">
+      <c r="J8" s="15">
         <v>1385.6</v>
       </c>
-      <c r="K8" s="10">
+      <c r="K8" s="13">
         <v>100</v>
       </c>
-      <c r="L8" s="10" t="s">
+      <c r="L8" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="M8" s="14">
+      <c r="M8" s="16">
         <v>46113</v>
       </c>
       <c r="N8" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="O8" s="10"/>
-      <c r="P8" s="10"/>
-      <c r="Q8" s="10"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
+      <c r="Q8" s="8"/>
     </row>
     <row r="9" spans="1:17">
-      <c r="A9" s="23">
+      <c r="A9" s="22">
         <v>6</v>
       </c>
-      <c r="B9" s="23" t="s">
+      <c r="B9" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="23" t="s">
+      <c r="C9" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="D9" s="24" t="s">
+      <c r="D9" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="E9" s="24" t="s">
+      <c r="E9" s="23" t="s">
         <v>44</v>
       </c>
       <c r="F9" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="G9" s="23"/>
-      <c r="H9" s="25">
+      <c r="G9" s="22"/>
+      <c r="H9" s="21">
         <v>160000</v>
       </c>
-      <c r="I9" s="25">
+      <c r="I9" s="21">
         <v>160000</v>
       </c>
-      <c r="J9" s="23">
+      <c r="J9" s="22">
         <v>0</v>
       </c>
-      <c r="K9" s="23">
+      <c r="K9" s="22">
         <v>50</v>
       </c>
-      <c r="L9" s="23" t="s">
+      <c r="L9" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="M9" s="26">
+      <c r="M9" s="28">
         <v>46113</v>
       </c>
       <c r="N9" s="7"/>
@@ -1234,126 +1240,126 @@
       <c r="Q9" s="7"/>
     </row>
     <row r="10" spans="1:17">
-      <c r="A10" s="23"/>
-      <c r="B10" s="23"/>
-      <c r="C10" s="23"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
+      <c r="A10" s="22"/>
+      <c r="B10" s="22"/>
+      <c r="C10" s="22"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="23"/>
       <c r="F10" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="G10" s="23"/>
-      <c r="H10" s="25"/>
-      <c r="I10" s="25"/>
-      <c r="J10" s="23"/>
-      <c r="K10" s="23"/>
-      <c r="L10" s="23"/>
-      <c r="M10" s="26"/>
+      <c r="G10" s="22"/>
+      <c r="H10" s="21"/>
+      <c r="I10" s="21"/>
+      <c r="J10" s="22"/>
+      <c r="K10" s="22"/>
+      <c r="L10" s="22"/>
+      <c r="M10" s="28"/>
       <c r="N10" s="7"/>
       <c r="O10" s="7"/>
       <c r="P10" s="7"/>
       <c r="Q10" s="7"/>
     </row>
     <row r="11" spans="1:17">
-      <c r="A11" s="19">
+      <c r="A11" s="25">
         <v>7</v>
       </c>
-      <c r="B11" s="19" t="s">
+      <c r="B11" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="19" t="s">
+      <c r="C11" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="D11" s="20" t="s">
+      <c r="D11" s="27" t="s">
         <v>48</v>
       </c>
-      <c r="E11" s="20" t="s">
+      <c r="E11" s="27" t="s">
         <v>49</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G11" s="19"/>
-      <c r="H11" s="21">
+      <c r="G11" s="25"/>
+      <c r="H11" s="24">
         <v>1490000</v>
       </c>
-      <c r="I11" s="21">
+      <c r="I11" s="24">
         <v>1033230</v>
       </c>
-      <c r="J11" s="21">
+      <c r="J11" s="24">
         <v>456770</v>
       </c>
-      <c r="K11" s="19">
+      <c r="K11" s="25">
         <v>15</v>
       </c>
-      <c r="L11" s="19" t="s">
+      <c r="L11" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="M11" s="22">
+      <c r="M11" s="26">
         <v>46113</v>
       </c>
-      <c r="N11" s="10"/>
-      <c r="O11" s="10"/>
-      <c r="P11" s="10"/>
-      <c r="Q11" s="10"/>
+      <c r="N11" s="8"/>
+      <c r="O11" s="8"/>
+      <c r="P11" s="8"/>
+      <c r="Q11" s="8"/>
     </row>
     <row r="12" spans="1:17" ht="29">
-      <c r="A12" s="19"/>
-      <c r="B12" s="19"/>
-      <c r="C12" s="19"/>
-      <c r="D12" s="20"/>
-      <c r="E12" s="20"/>
+      <c r="A12" s="25"/>
+      <c r="B12" s="25"/>
+      <c r="C12" s="25"/>
+      <c r="D12" s="27"/>
+      <c r="E12" s="27"/>
       <c r="F12" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="G12" s="19"/>
-      <c r="H12" s="21"/>
-      <c r="I12" s="21"/>
-      <c r="J12" s="21"/>
-      <c r="K12" s="19"/>
-      <c r="L12" s="19"/>
-      <c r="M12" s="22"/>
-      <c r="N12" s="10"/>
-      <c r="O12" s="10"/>
-      <c r="P12" s="10"/>
-      <c r="Q12" s="10"/>
+      <c r="G12" s="25"/>
+      <c r="H12" s="24"/>
+      <c r="I12" s="24"/>
+      <c r="J12" s="24"/>
+      <c r="K12" s="25"/>
+      <c r="L12" s="25"/>
+      <c r="M12" s="26"/>
+      <c r="N12" s="8"/>
+      <c r="O12" s="8"/>
+      <c r="P12" s="8"/>
+      <c r="Q12" s="8"/>
     </row>
     <row r="13" spans="1:17">
-      <c r="A13" s="7">
+      <c r="A13" s="17">
         <v>8</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="D13" s="9" t="s">
+      <c r="D13" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="E13" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="F13" s="9" t="s">
+      <c r="F13" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="G13" s="7"/>
-      <c r="H13" s="8">
+      <c r="G13" s="17"/>
+      <c r="H13" s="19">
         <v>400000</v>
       </c>
-      <c r="I13" s="8">
+      <c r="I13" s="19">
         <v>399690</v>
       </c>
-      <c r="J13" s="7">
+      <c r="J13" s="17">
         <v>310</v>
       </c>
-      <c r="K13" s="7">
+      <c r="K13" s="17">
         <v>10</v>
       </c>
-      <c r="L13" s="7" t="s">
+      <c r="L13" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="M13" s="13">
+      <c r="M13" s="20">
         <v>46113</v>
       </c>
       <c r="N13" s="7"/>
@@ -1362,103 +1368,103 @@
       <c r="Q13" s="7"/>
     </row>
     <row r="14" spans="1:17">
-      <c r="A14" s="19">
+      <c r="A14" s="25">
         <v>9</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="C14" s="19" t="s">
+      <c r="C14" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="D14" s="20" t="s">
+      <c r="D14" s="27" t="s">
         <v>56</v>
       </c>
-      <c r="E14" s="20" t="s">
+      <c r="E14" s="27" t="s">
         <v>57</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="G14" s="19"/>
-      <c r="H14" s="21">
+      <c r="G14" s="25"/>
+      <c r="H14" s="24">
         <v>1200000</v>
       </c>
-      <c r="I14" s="21">
+      <c r="I14" s="24">
         <v>1100000</v>
       </c>
-      <c r="J14" s="21">
+      <c r="J14" s="24">
         <v>100000</v>
       </c>
-      <c r="K14" s="19">
+      <c r="K14" s="25">
         <v>10</v>
       </c>
-      <c r="L14" s="19" t="s">
+      <c r="L14" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="M14" s="22">
+      <c r="M14" s="26">
         <v>46104</v>
       </c>
-      <c r="N14" s="10"/>
-      <c r="O14" s="10"/>
-      <c r="P14" s="10"/>
-      <c r="Q14" s="10"/>
+      <c r="N14" s="8"/>
+      <c r="O14" s="8"/>
+      <c r="P14" s="8"/>
+      <c r="Q14" s="8"/>
     </row>
     <row r="15" spans="1:17">
-      <c r="A15" s="19"/>
-      <c r="B15" s="19"/>
-      <c r="C15" s="19"/>
-      <c r="D15" s="20"/>
-      <c r="E15" s="20"/>
+      <c r="A15" s="25"/>
+      <c r="B15" s="25"/>
+      <c r="C15" s="25"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="27"/>
       <c r="F15" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="G15" s="19"/>
-      <c r="H15" s="21"/>
-      <c r="I15" s="21"/>
-      <c r="J15" s="21"/>
-      <c r="K15" s="19"/>
-      <c r="L15" s="19"/>
-      <c r="M15" s="22"/>
-      <c r="N15" s="10"/>
-      <c r="O15" s="10"/>
-      <c r="P15" s="10"/>
-      <c r="Q15" s="10"/>
+      <c r="G15" s="25"/>
+      <c r="H15" s="24"/>
+      <c r="I15" s="24"/>
+      <c r="J15" s="24"/>
+      <c r="K15" s="25"/>
+      <c r="L15" s="25"/>
+      <c r="M15" s="26"/>
+      <c r="N15" s="8"/>
+      <c r="O15" s="8"/>
+      <c r="P15" s="8"/>
+      <c r="Q15" s="8"/>
     </row>
     <row r="16" spans="1:17">
-      <c r="A16" s="23">
+      <c r="A16" s="22">
         <v>10</v>
       </c>
-      <c r="B16" s="23" t="s">
+      <c r="B16" s="22" t="s">
         <v>55</v>
       </c>
-      <c r="C16" s="23" t="s">
+      <c r="C16" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="D16" s="24" t="s">
+      <c r="D16" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E16" s="24" t="s">
+      <c r="E16" s="23" t="s">
         <v>49</v>
       </c>
       <c r="F16" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="G16" s="23"/>
-      <c r="H16" s="25">
+      <c r="G16" s="22"/>
+      <c r="H16" s="21">
         <v>1430000</v>
       </c>
-      <c r="I16" s="23"/>
-      <c r="J16" s="25">
+      <c r="I16" s="22"/>
+      <c r="J16" s="21">
         <v>1430000</v>
       </c>
-      <c r="K16" s="23">
+      <c r="K16" s="22">
         <v>5</v>
       </c>
-      <c r="L16" s="23" t="s">
+      <c r="L16" s="22" t="s">
         <v>60</v>
       </c>
-      <c r="M16" s="26">
+      <c r="M16" s="28">
         <v>46104</v>
       </c>
       <c r="N16" s="7"/>
@@ -1467,99 +1473,99 @@
       <c r="Q16" s="7"/>
     </row>
     <row r="17" spans="1:17" ht="29">
-      <c r="A17" s="23"/>
-      <c r="B17" s="23"/>
-      <c r="C17" s="23"/>
-      <c r="D17" s="24"/>
-      <c r="E17" s="24"/>
+      <c r="A17" s="22"/>
+      <c r="B17" s="22"/>
+      <c r="C17" s="22"/>
+      <c r="D17" s="23"/>
+      <c r="E17" s="23"/>
       <c r="F17" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="G17" s="23"/>
-      <c r="H17" s="25"/>
-      <c r="I17" s="23"/>
-      <c r="J17" s="25"/>
-      <c r="K17" s="23"/>
-      <c r="L17" s="23"/>
-      <c r="M17" s="26"/>
+      <c r="G17" s="22"/>
+      <c r="H17" s="21"/>
+      <c r="I17" s="22"/>
+      <c r="J17" s="21"/>
+      <c r="K17" s="22"/>
+      <c r="L17" s="22"/>
+      <c r="M17" s="28"/>
       <c r="N17" s="7"/>
       <c r="O17" s="7"/>
       <c r="P17" s="7"/>
       <c r="Q17" s="7"/>
     </row>
     <row r="18" spans="1:17">
-      <c r="A18" s="10">
+      <c r="A18" s="13">
         <v>11</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="C18" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="D18" s="12" t="s">
+      <c r="D18" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="E18" s="12" t="s">
+      <c r="E18" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="F18" s="12" t="s">
+      <c r="F18" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="G18" s="10"/>
-      <c r="H18" s="11">
+      <c r="G18" s="13"/>
+      <c r="H18" s="15">
         <v>450000</v>
       </c>
-      <c r="I18" s="10"/>
-      <c r="J18" s="11">
+      <c r="I18" s="13"/>
+      <c r="J18" s="15">
         <v>450000</v>
       </c>
-      <c r="K18" s="10"/>
-      <c r="L18" s="10"/>
-      <c r="M18" s="14">
+      <c r="K18" s="13"/>
+      <c r="L18" s="13"/>
+      <c r="M18" s="16">
         <v>46104</v>
       </c>
-      <c r="N18" s="10"/>
-      <c r="O18" s="10"/>
-      <c r="P18" s="10"/>
-      <c r="Q18" s="10" t="s">
+      <c r="N18" s="8"/>
+      <c r="O18" s="8"/>
+      <c r="P18" s="8"/>
+      <c r="Q18" s="8" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="19" spans="1:17">
-      <c r="A19" s="23">
+      <c r="A19" s="22">
         <v>12</v>
       </c>
-      <c r="B19" s="23" t="s">
+      <c r="B19" s="22" t="s">
         <v>62</v>
       </c>
-      <c r="C19" s="23" t="s">
+      <c r="C19" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="D19" s="24" t="s">
+      <c r="D19" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E19" s="24" t="s">
+      <c r="E19" s="23" t="s">
         <v>49</v>
       </c>
       <c r="F19" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="G19" s="23"/>
-      <c r="H19" s="25">
+      <c r="G19" s="22"/>
+      <c r="H19" s="21">
         <v>920000</v>
       </c>
-      <c r="I19" s="23"/>
-      <c r="J19" s="25">
+      <c r="I19" s="22"/>
+      <c r="J19" s="21">
         <v>920000</v>
       </c>
-      <c r="K19" s="23">
+      <c r="K19" s="22">
         <v>5</v>
       </c>
-      <c r="L19" s="23" t="s">
+      <c r="L19" s="22" t="s">
         <v>60</v>
       </c>
-      <c r="M19" s="26">
+      <c r="M19" s="28">
         <v>46104</v>
       </c>
       <c r="N19" s="7"/>
@@ -1568,103 +1574,103 @@
       <c r="Q19" s="7"/>
     </row>
     <row r="20" spans="1:17" ht="29">
-      <c r="A20" s="23"/>
-      <c r="B20" s="23"/>
-      <c r="C20" s="23"/>
-      <c r="D20" s="24"/>
-      <c r="E20" s="24"/>
+      <c r="A20" s="22"/>
+      <c r="B20" s="22"/>
+      <c r="C20" s="22"/>
+      <c r="D20" s="23"/>
+      <c r="E20" s="23"/>
       <c r="F20" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="G20" s="23"/>
-      <c r="H20" s="25"/>
-      <c r="I20" s="23"/>
-      <c r="J20" s="25"/>
-      <c r="K20" s="23"/>
-      <c r="L20" s="23"/>
-      <c r="M20" s="26"/>
+      <c r="G20" s="22"/>
+      <c r="H20" s="21"/>
+      <c r="I20" s="22"/>
+      <c r="J20" s="21"/>
+      <c r="K20" s="22"/>
+      <c r="L20" s="22"/>
+      <c r="M20" s="28"/>
       <c r="N20" s="7"/>
       <c r="O20" s="7"/>
       <c r="P20" s="7"/>
       <c r="Q20" s="7"/>
     </row>
     <row r="21" spans="1:17">
-      <c r="A21" s="10">
+      <c r="A21" s="13">
         <v>13</v>
       </c>
-      <c r="B21" s="10" t="s">
+      <c r="B21" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="C21" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="D21" s="12" t="s">
+      <c r="D21" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="E21" s="12" t="s">
+      <c r="E21" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="F21" s="12" t="s">
+      <c r="F21" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="G21" s="10"/>
-      <c r="H21" s="11">
+      <c r="G21" s="13"/>
+      <c r="H21" s="15">
         <v>945000</v>
       </c>
-      <c r="I21" s="10"/>
-      <c r="J21" s="11">
+      <c r="I21" s="13"/>
+      <c r="J21" s="15">
         <v>945000</v>
       </c>
-      <c r="K21" s="10"/>
-      <c r="L21" s="10"/>
-      <c r="M21" s="14">
+      <c r="K21" s="13"/>
+      <c r="L21" s="13"/>
+      <c r="M21" s="16">
         <v>46104</v>
       </c>
-      <c r="N21" s="10"/>
-      <c r="O21" s="10"/>
-      <c r="P21" s="10"/>
-      <c r="Q21" s="10" t="s">
+      <c r="N21" s="8"/>
+      <c r="O21" s="8"/>
+      <c r="P21" s="8"/>
+      <c r="Q21" s="8" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="22" spans="1:17">
-      <c r="A22" s="23">
+      <c r="A22" s="22">
         <v>14</v>
       </c>
-      <c r="B22" s="23" t="s">
+      <c r="B22" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="C22" s="23" t="s">
+      <c r="C22" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="D22" s="24" t="s">
+      <c r="D22" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="E22" s="24" t="s">
+      <c r="E22" s="23" t="s">
         <v>65</v>
       </c>
       <c r="F22" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="G22" s="23" t="s">
+      <c r="G22" s="22" t="s">
         <v>68</v>
       </c>
-      <c r="H22" s="25">
+      <c r="H22" s="21">
         <v>100000</v>
       </c>
-      <c r="I22" s="25">
+      <c r="I22" s="21">
         <v>100000</v>
       </c>
-      <c r="J22" s="23">
+      <c r="J22" s="22">
         <v>0</v>
       </c>
-      <c r="K22" s="23">
+      <c r="K22" s="22">
         <v>10</v>
       </c>
-      <c r="L22" s="23" t="s">
+      <c r="L22" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="M22" s="26">
+      <c r="M22" s="28">
         <v>46114</v>
       </c>
       <c r="N22" s="7"/>
@@ -1673,128 +1679,128 @@
       <c r="Q22" s="7"/>
     </row>
     <row r="23" spans="1:17">
-      <c r="A23" s="23"/>
-      <c r="B23" s="23"/>
-      <c r="C23" s="23"/>
-      <c r="D23" s="24"/>
-      <c r="E23" s="24"/>
+      <c r="A23" s="22"/>
+      <c r="B23" s="22"/>
+      <c r="C23" s="22"/>
+      <c r="D23" s="23"/>
+      <c r="E23" s="23"/>
       <c r="F23" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="G23" s="23"/>
-      <c r="H23" s="25"/>
-      <c r="I23" s="25"/>
-      <c r="J23" s="23"/>
-      <c r="K23" s="23"/>
-      <c r="L23" s="23"/>
-      <c r="M23" s="26"/>
+      <c r="G23" s="22"/>
+      <c r="H23" s="21"/>
+      <c r="I23" s="21"/>
+      <c r="J23" s="22"/>
+      <c r="K23" s="22"/>
+      <c r="L23" s="22"/>
+      <c r="M23" s="28"/>
       <c r="N23" s="7"/>
       <c r="O23" s="7"/>
       <c r="P23" s="7"/>
       <c r="Q23" s="7"/>
     </row>
     <row r="24" spans="1:17">
-      <c r="A24" s="19">
+      <c r="A24" s="25">
         <v>15</v>
       </c>
-      <c r="B24" s="19" t="s">
+      <c r="B24" s="25" t="s">
         <v>63</v>
       </c>
-      <c r="C24" s="19" t="s">
+      <c r="C24" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="D24" s="20" t="s">
+      <c r="D24" s="27" t="s">
         <v>69</v>
       </c>
-      <c r="E24" s="20" t="s">
+      <c r="E24" s="27" t="s">
         <v>70</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="G24" s="19" t="s">
+      <c r="G24" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="H24" s="21">
+      <c r="H24" s="24">
         <v>370000</v>
       </c>
-      <c r="I24" s="21">
+      <c r="I24" s="24">
         <v>370000</v>
       </c>
-      <c r="J24" s="19">
+      <c r="J24" s="25">
         <v>0</v>
       </c>
-      <c r="K24" s="19">
+      <c r="K24" s="25">
         <v>70</v>
       </c>
-      <c r="L24" s="19" t="s">
+      <c r="L24" s="25" t="s">
         <v>126</v>
       </c>
-      <c r="M24" s="22">
+      <c r="M24" s="26">
         <v>46114</v>
       </c>
-      <c r="N24" s="10"/>
-      <c r="O24" s="10"/>
-      <c r="P24" s="10"/>
-      <c r="Q24" s="10"/>
+      <c r="N24" s="8"/>
+      <c r="O24" s="8"/>
+      <c r="P24" s="8"/>
+      <c r="Q24" s="8"/>
     </row>
     <row r="25" spans="1:17">
-      <c r="A25" s="19"/>
-      <c r="B25" s="19"/>
-      <c r="C25" s="19"/>
-      <c r="D25" s="20"/>
-      <c r="E25" s="20"/>
+      <c r="A25" s="25"/>
+      <c r="B25" s="25"/>
+      <c r="C25" s="25"/>
+      <c r="D25" s="27"/>
+      <c r="E25" s="27"/>
       <c r="F25" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="G25" s="19"/>
-      <c r="H25" s="21"/>
-      <c r="I25" s="21"/>
-      <c r="J25" s="19"/>
-      <c r="K25" s="19"/>
-      <c r="L25" s="19"/>
-      <c r="M25" s="22"/>
-      <c r="N25" s="10"/>
-      <c r="O25" s="10"/>
-      <c r="P25" s="10"/>
-      <c r="Q25" s="10"/>
+      <c r="G25" s="25"/>
+      <c r="H25" s="24"/>
+      <c r="I25" s="24"/>
+      <c r="J25" s="25"/>
+      <c r="K25" s="25"/>
+      <c r="L25" s="25"/>
+      <c r="M25" s="26"/>
+      <c r="N25" s="8"/>
+      <c r="O25" s="8"/>
+      <c r="P25" s="8"/>
+      <c r="Q25" s="8"/>
     </row>
     <row r="26" spans="1:17">
-      <c r="A26" s="23">
+      <c r="A26" s="22">
         <v>16</v>
       </c>
-      <c r="B26" s="23" t="s">
+      <c r="B26" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="C26" s="23" t="s">
+      <c r="C26" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="D26" s="24" t="s">
+      <c r="D26" s="23" t="s">
         <v>74</v>
       </c>
-      <c r="E26" s="24" t="s">
+      <c r="E26" s="23" t="s">
         <v>75</v>
       </c>
       <c r="F26" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="G26" s="23"/>
-      <c r="H26" s="25">
+      <c r="G26" s="22"/>
+      <c r="H26" s="21">
         <v>2255000</v>
       </c>
-      <c r="I26" s="25">
+      <c r="I26" s="21">
         <v>2005050</v>
       </c>
-      <c r="J26" s="25">
+      <c r="J26" s="21">
         <v>249950</v>
       </c>
-      <c r="K26" s="23">
+      <c r="K26" s="22">
         <v>10</v>
       </c>
-      <c r="L26" s="23" t="s">
+      <c r="L26" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="M26" s="26">
+      <c r="M26" s="28">
         <v>46114</v>
       </c>
       <c r="N26" s="7"/>
@@ -1803,128 +1809,128 @@
       <c r="Q26" s="7"/>
     </row>
     <row r="27" spans="1:17">
-      <c r="A27" s="23"/>
-      <c r="B27" s="23"/>
-      <c r="C27" s="23"/>
-      <c r="D27" s="24"/>
-      <c r="E27" s="24"/>
+      <c r="A27" s="22"/>
+      <c r="B27" s="22"/>
+      <c r="C27" s="22"/>
+      <c r="D27" s="23"/>
+      <c r="E27" s="23"/>
       <c r="F27" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="G27" s="23"/>
-      <c r="H27" s="25"/>
-      <c r="I27" s="25"/>
-      <c r="J27" s="25"/>
-      <c r="K27" s="23"/>
-      <c r="L27" s="23"/>
-      <c r="M27" s="26"/>
+      <c r="G27" s="22"/>
+      <c r="H27" s="21"/>
+      <c r="I27" s="21"/>
+      <c r="J27" s="21"/>
+      <c r="K27" s="22"/>
+      <c r="L27" s="22"/>
+      <c r="M27" s="28"/>
       <c r="N27" s="7"/>
       <c r="O27" s="7"/>
       <c r="P27" s="7"/>
       <c r="Q27" s="7"/>
     </row>
     <row r="28" spans="1:17">
-      <c r="A28" s="19">
+      <c r="A28" s="25">
         <v>17</v>
       </c>
-      <c r="B28" s="19" t="s">
+      <c r="B28" s="25" t="s">
         <v>63</v>
       </c>
-      <c r="C28" s="19" t="s">
+      <c r="C28" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="D28" s="20" t="s">
+      <c r="D28" s="27" t="s">
         <v>78</v>
       </c>
-      <c r="E28" s="20" t="s">
+      <c r="E28" s="27" t="s">
         <v>79</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="G28" s="19"/>
-      <c r="H28" s="21">
+      <c r="G28" s="25"/>
+      <c r="H28" s="24">
         <v>110000</v>
       </c>
-      <c r="I28" s="19">
+      <c r="I28" s="25">
         <v>0</v>
       </c>
-      <c r="J28" s="21">
+      <c r="J28" s="24">
         <v>110000</v>
       </c>
-      <c r="K28" s="19">
+      <c r="K28" s="25">
         <v>5</v>
       </c>
-      <c r="L28" s="19" t="s">
+      <c r="L28" s="25" t="s">
         <v>60</v>
       </c>
-      <c r="M28" s="22">
+      <c r="M28" s="26">
         <v>46114</v>
       </c>
-      <c r="N28" s="10"/>
-      <c r="O28" s="10"/>
-      <c r="P28" s="10"/>
-      <c r="Q28" s="10"/>
+      <c r="N28" s="8"/>
+      <c r="O28" s="8"/>
+      <c r="P28" s="8"/>
+      <c r="Q28" s="8"/>
     </row>
     <row r="29" spans="1:17">
-      <c r="A29" s="19"/>
-      <c r="B29" s="19"/>
-      <c r="C29" s="19"/>
-      <c r="D29" s="20"/>
-      <c r="E29" s="20"/>
+      <c r="A29" s="25"/>
+      <c r="B29" s="25"/>
+      <c r="C29" s="25"/>
+      <c r="D29" s="27"/>
+      <c r="E29" s="27"/>
       <c r="F29" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="G29" s="19"/>
-      <c r="H29" s="21"/>
-      <c r="I29" s="19"/>
-      <c r="J29" s="21"/>
-      <c r="K29" s="19"/>
-      <c r="L29" s="19"/>
-      <c r="M29" s="22"/>
-      <c r="N29" s="10"/>
-      <c r="O29" s="10"/>
-      <c r="P29" s="10"/>
-      <c r="Q29" s="10"/>
+      <c r="G29" s="25"/>
+      <c r="H29" s="24"/>
+      <c r="I29" s="25"/>
+      <c r="J29" s="24"/>
+      <c r="K29" s="25"/>
+      <c r="L29" s="25"/>
+      <c r="M29" s="26"/>
+      <c r="N29" s="8"/>
+      <c r="O29" s="8"/>
+      <c r="P29" s="8"/>
+      <c r="Q29" s="8"/>
     </row>
     <row r="30" spans="1:17">
-      <c r="A30" s="7">
+      <c r="A30" s="17">
         <v>18</v>
       </c>
-      <c r="B30" s="7" t="s">
+      <c r="B30" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="C30" s="7" t="s">
+      <c r="C30" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="D30" s="9" t="s">
+      <c r="D30" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="E30" s="9" t="s">
+      <c r="E30" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="F30" s="9" t="s">
+      <c r="F30" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="G30" s="7" t="s">
+      <c r="G30" s="17" t="s">
         <v>85</v>
       </c>
-      <c r="H30" s="8">
+      <c r="H30" s="19">
         <v>1000000</v>
       </c>
-      <c r="I30" s="8">
+      <c r="I30" s="19">
         <v>950000</v>
       </c>
-      <c r="J30" s="8">
+      <c r="J30" s="19">
         <v>50000</v>
       </c>
-      <c r="K30" s="7">
+      <c r="K30" s="17">
         <v>10</v>
       </c>
-      <c r="L30" s="7" t="s">
+      <c r="L30" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="M30" s="13">
+      <c r="M30" s="20">
         <v>46114</v>
       </c>
       <c r="N30" s="7"/>
@@ -1933,105 +1939,105 @@
       <c r="Q30" s="7"/>
     </row>
     <row r="31" spans="1:17">
-      <c r="A31" s="19">
+      <c r="A31" s="25">
         <v>19</v>
       </c>
-      <c r="B31" s="19" t="s">
+      <c r="B31" s="25" t="s">
         <v>63</v>
       </c>
-      <c r="C31" s="19" t="s">
+      <c r="C31" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D31" s="20" t="s">
+      <c r="D31" s="27" t="s">
         <v>86</v>
       </c>
-      <c r="E31" s="20" t="s">
+      <c r="E31" s="27" t="s">
         <v>87</v>
       </c>
       <c r="F31" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="G31" s="19"/>
-      <c r="H31" s="21">
+      <c r="G31" s="25"/>
+      <c r="H31" s="24">
         <v>28000</v>
       </c>
-      <c r="I31" s="21">
+      <c r="I31" s="24">
         <v>20250</v>
       </c>
-      <c r="J31" s="21">
+      <c r="J31" s="24">
         <v>7750</v>
       </c>
-      <c r="K31" s="19">
+      <c r="K31" s="25">
         <v>10</v>
       </c>
-      <c r="L31" s="19" t="s">
+      <c r="L31" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="M31" s="22">
+      <c r="M31" s="26">
         <v>46114</v>
       </c>
-      <c r="N31" s="10"/>
-      <c r="O31" s="10"/>
-      <c r="P31" s="10"/>
-      <c r="Q31" s="10"/>
+      <c r="N31" s="8"/>
+      <c r="O31" s="8"/>
+      <c r="P31" s="8"/>
+      <c r="Q31" s="8"/>
     </row>
     <row r="32" spans="1:17">
-      <c r="A32" s="19"/>
-      <c r="B32" s="19"/>
-      <c r="C32" s="19"/>
-      <c r="D32" s="20"/>
-      <c r="E32" s="20"/>
+      <c r="A32" s="25"/>
+      <c r="B32" s="25"/>
+      <c r="C32" s="25"/>
+      <c r="D32" s="27"/>
+      <c r="E32" s="27"/>
       <c r="F32" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="G32" s="19"/>
-      <c r="H32" s="21"/>
-      <c r="I32" s="21"/>
-      <c r="J32" s="21"/>
-      <c r="K32" s="19"/>
-      <c r="L32" s="19"/>
-      <c r="M32" s="22"/>
-      <c r="N32" s="10"/>
-      <c r="O32" s="10"/>
-      <c r="P32" s="10"/>
-      <c r="Q32" s="10"/>
+      <c r="G32" s="25"/>
+      <c r="H32" s="24"/>
+      <c r="I32" s="24"/>
+      <c r="J32" s="24"/>
+      <c r="K32" s="25"/>
+      <c r="L32" s="25"/>
+      <c r="M32" s="26"/>
+      <c r="N32" s="8"/>
+      <c r="O32" s="8"/>
+      <c r="P32" s="8"/>
+      <c r="Q32" s="8"/>
     </row>
     <row r="33" spans="1:17">
-      <c r="A33" s="7">
+      <c r="A33" s="17">
         <v>20</v>
       </c>
-      <c r="B33" s="7" t="s">
+      <c r="B33" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="C33" s="7" t="s">
+      <c r="C33" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="D33" s="9" t="s">
+      <c r="D33" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="E33" s="9" t="s">
+      <c r="E33" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="F33" s="9" t="s">
+      <c r="F33" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="G33" s="7"/>
-      <c r="H33" s="8">
+      <c r="G33" s="17"/>
+      <c r="H33" s="19">
         <v>140000</v>
       </c>
-      <c r="I33" s="8">
+      <c r="I33" s="19">
         <v>115000</v>
       </c>
-      <c r="J33" s="8">
+      <c r="J33" s="19">
         <v>25000</v>
       </c>
-      <c r="K33" s="7">
+      <c r="K33" s="17">
         <v>80</v>
       </c>
-      <c r="L33" s="7" t="s">
+      <c r="L33" s="17" t="s">
         <v>126</v>
       </c>
-      <c r="M33" s="13">
+      <c r="M33" s="20">
         <v>46114</v>
       </c>
       <c r="N33" s="7"/>
@@ -2040,832 +2046,1024 @@
       <c r="Q33" s="7"/>
     </row>
     <row r="34" spans="1:17">
-      <c r="A34" s="10">
+      <c r="A34" s="13">
         <v>21</v>
       </c>
-      <c r="B34" s="10" t="s">
+      <c r="B34" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="C34" s="10" t="s">
+      <c r="C34" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="D34" s="12" t="s">
+      <c r="D34" s="14" t="s">
         <v>93</v>
       </c>
-      <c r="E34" s="12" t="s">
+      <c r="E34" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="F34" s="12" t="s">
+      <c r="F34" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="G34" s="10"/>
-      <c r="H34" s="11">
+      <c r="G34" s="13"/>
+      <c r="H34" s="15">
         <v>20000</v>
       </c>
-      <c r="I34" s="11">
+      <c r="I34" s="15">
         <v>18614</v>
       </c>
-      <c r="J34" s="11">
+      <c r="J34" s="15">
         <v>1386</v>
       </c>
-      <c r="K34" s="10">
+      <c r="K34" s="13">
         <v>100</v>
       </c>
-      <c r="L34" s="10"/>
-      <c r="M34" s="10"/>
-      <c r="N34" s="10"/>
-      <c r="O34" s="10"/>
-      <c r="P34" s="10"/>
-      <c r="Q34" s="10"/>
+      <c r="L34" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="M34" s="16">
+        <v>46114</v>
+      </c>
+      <c r="N34" s="8"/>
+      <c r="O34" s="8"/>
+      <c r="P34" s="8"/>
+      <c r="Q34" s="8"/>
     </row>
     <row r="35" spans="1:17">
-      <c r="A35" s="23">
+      <c r="A35" s="22">
         <v>22</v>
       </c>
-      <c r="B35" s="23" t="s">
+      <c r="B35" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="C35" s="23" t="s">
+      <c r="C35" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="D35" s="24" t="s">
+      <c r="D35" s="23" t="s">
         <v>95</v>
       </c>
-      <c r="E35" s="24" t="s">
+      <c r="E35" s="23" t="s">
         <v>96</v>
       </c>
       <c r="F35" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="G35" s="23" t="s">
+      <c r="G35" s="22" t="s">
         <v>99</v>
       </c>
-      <c r="H35" s="25">
+      <c r="H35" s="21">
         <v>80000</v>
       </c>
-      <c r="I35" s="23"/>
-      <c r="J35" s="25">
-        <v>80000</v>
-      </c>
-      <c r="K35" s="23"/>
-      <c r="L35" s="23"/>
-      <c r="M35" s="23"/>
+      <c r="I35" s="21">
+        <v>74970</v>
+      </c>
+      <c r="J35" s="21">
+        <v>5030</v>
+      </c>
+      <c r="K35" s="22">
+        <v>10</v>
+      </c>
+      <c r="L35" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="M35" s="28">
+        <v>46114</v>
+      </c>
       <c r="N35" s="7"/>
       <c r="O35" s="7"/>
       <c r="P35" s="7"/>
       <c r="Q35" s="7"/>
     </row>
     <row r="36" spans="1:17">
-      <c r="A36" s="23"/>
-      <c r="B36" s="23"/>
-      <c r="C36" s="23"/>
-      <c r="D36" s="24"/>
-      <c r="E36" s="24"/>
+      <c r="A36" s="22"/>
+      <c r="B36" s="22"/>
+      <c r="C36" s="22"/>
+      <c r="D36" s="23"/>
+      <c r="E36" s="23"/>
       <c r="F36" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="G36" s="23"/>
-      <c r="H36" s="25"/>
-      <c r="I36" s="23"/>
-      <c r="J36" s="25"/>
-      <c r="K36" s="23"/>
-      <c r="L36" s="23"/>
-      <c r="M36" s="23"/>
+      <c r="G36" s="22"/>
+      <c r="H36" s="21"/>
+      <c r="I36" s="21"/>
+      <c r="J36" s="21"/>
+      <c r="K36" s="22"/>
+      <c r="L36" s="22"/>
+      <c r="M36" s="28"/>
       <c r="N36" s="7"/>
       <c r="O36" s="7"/>
       <c r="P36" s="7"/>
       <c r="Q36" s="7"/>
     </row>
     <row r="37" spans="1:17">
-      <c r="A37" s="10">
+      <c r="A37" s="13">
         <v>23</v>
       </c>
-      <c r="B37" s="10" t="s">
+      <c r="B37" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="C37" s="10" t="s">
+      <c r="C37" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="D37" s="12" t="s">
+      <c r="D37" s="14" t="s">
         <v>100</v>
       </c>
-      <c r="E37" s="12" t="s">
+      <c r="E37" s="14" t="s">
         <v>101</v>
       </c>
-      <c r="F37" s="12" t="s">
+      <c r="F37" s="14" t="s">
         <v>102</v>
       </c>
-      <c r="G37" s="10"/>
-      <c r="H37" s="11">
+      <c r="G37" s="13"/>
+      <c r="H37" s="15">
         <v>20000</v>
       </c>
-      <c r="I37" s="10"/>
-      <c r="J37" s="11">
-        <v>20000</v>
-      </c>
-      <c r="K37" s="10"/>
-      <c r="L37" s="10"/>
-      <c r="M37" s="10"/>
-      <c r="N37" s="10"/>
-      <c r="O37" s="10"/>
-      <c r="P37" s="10"/>
-      <c r="Q37" s="10"/>
+      <c r="I37" s="15">
+        <v>15580</v>
+      </c>
+      <c r="J37" s="15">
+        <v>4420</v>
+      </c>
+      <c r="K37" s="13">
+        <v>10</v>
+      </c>
+      <c r="L37" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="M37" s="16">
+        <v>46114</v>
+      </c>
+      <c r="N37" s="8"/>
+      <c r="O37" s="8"/>
+      <c r="P37" s="8"/>
+      <c r="Q37" s="8"/>
     </row>
     <row r="38" spans="1:17">
-      <c r="A38" s="23">
+      <c r="A38" s="22">
         <v>24</v>
       </c>
-      <c r="B38" s="23" t="s">
+      <c r="B38" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="C38" s="23" t="s">
+      <c r="C38" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="D38" s="24" t="s">
+      <c r="D38" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="E38" s="24" t="s">
+      <c r="E38" s="23" t="s">
         <v>49</v>
       </c>
       <c r="F38" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="G38" s="23"/>
-      <c r="H38" s="25">
+      <c r="G38" s="22"/>
+      <c r="H38" s="21">
         <v>982000</v>
       </c>
-      <c r="I38" s="23"/>
-      <c r="J38" s="25">
-        <v>982000</v>
-      </c>
-      <c r="K38" s="23"/>
-      <c r="L38" s="23"/>
-      <c r="M38" s="23"/>
+      <c r="I38" s="21">
+        <v>788000</v>
+      </c>
+      <c r="J38" s="21">
+        <v>194000</v>
+      </c>
+      <c r="K38" s="22">
+        <v>10</v>
+      </c>
+      <c r="L38" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="M38" s="28">
+        <v>46114</v>
+      </c>
       <c r="N38" s="7"/>
       <c r="O38" s="7"/>
       <c r="P38" s="7"/>
       <c r="Q38" s="7"/>
     </row>
     <row r="39" spans="1:17" ht="29">
-      <c r="A39" s="23"/>
-      <c r="B39" s="23"/>
-      <c r="C39" s="23"/>
-      <c r="D39" s="24"/>
-      <c r="E39" s="24"/>
+      <c r="A39" s="22"/>
+      <c r="B39" s="22"/>
+      <c r="C39" s="22"/>
+      <c r="D39" s="23"/>
+      <c r="E39" s="23"/>
       <c r="F39" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="G39" s="23"/>
-      <c r="H39" s="25"/>
-      <c r="I39" s="23"/>
-      <c r="J39" s="25"/>
-      <c r="K39" s="23"/>
-      <c r="L39" s="23"/>
-      <c r="M39" s="23"/>
+      <c r="G39" s="22"/>
+      <c r="H39" s="21"/>
+      <c r="I39" s="21"/>
+      <c r="J39" s="21"/>
+      <c r="K39" s="22"/>
+      <c r="L39" s="22"/>
+      <c r="M39" s="28"/>
       <c r="N39" s="7"/>
       <c r="O39" s="7"/>
       <c r="P39" s="7"/>
       <c r="Q39" s="7"/>
     </row>
     <row r="40" spans="1:17">
-      <c r="A40" s="10">
+      <c r="A40" s="13">
         <v>25</v>
       </c>
-      <c r="B40" s="10" t="s">
+      <c r="B40" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="C40" s="10" t="s">
+      <c r="C40" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="D40" s="12" t="s">
+      <c r="D40" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="E40" s="12" t="s">
+      <c r="E40" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="F40" s="12" t="s">
+      <c r="F40" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="G40" s="10"/>
-      <c r="H40" s="11">
+      <c r="G40" s="13"/>
+      <c r="H40" s="15">
         <v>370000</v>
       </c>
-      <c r="I40" s="10"/>
-      <c r="J40" s="11">
-        <v>370000</v>
-      </c>
-      <c r="K40" s="10"/>
-      <c r="L40" s="10"/>
-      <c r="M40" s="10"/>
-      <c r="N40" s="10"/>
-      <c r="O40" s="10"/>
-      <c r="P40" s="10"/>
-      <c r="Q40" s="10"/>
+      <c r="I40" s="15">
+        <v>225000</v>
+      </c>
+      <c r="J40" s="15">
+        <v>145000</v>
+      </c>
+      <c r="K40" s="13">
+        <v>10</v>
+      </c>
+      <c r="L40" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="M40" s="16">
+        <v>46114</v>
+      </c>
+      <c r="N40" s="8"/>
+      <c r="O40" s="8"/>
+      <c r="P40" s="8"/>
+      <c r="Q40" s="8"/>
     </row>
     <row r="41" spans="1:17">
-      <c r="A41" s="7">
+      <c r="A41" s="17">
         <v>26</v>
       </c>
-      <c r="B41" s="7" t="s">
+      <c r="B41" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="C41" s="7" t="s">
+      <c r="C41" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="D41" s="9" t="s">
+      <c r="D41" s="18" t="s">
         <v>104</v>
       </c>
-      <c r="E41" s="7"/>
-      <c r="F41" s="7"/>
-      <c r="G41" s="7"/>
-      <c r="H41" s="8">
+      <c r="E41" s="17"/>
+      <c r="F41" s="17"/>
+      <c r="G41" s="17"/>
+      <c r="H41" s="19">
         <v>2855104</v>
       </c>
-      <c r="I41" s="7"/>
-      <c r="J41" s="8">
+      <c r="I41" s="17"/>
+      <c r="J41" s="19">
         <v>2855104</v>
       </c>
-      <c r="K41" s="7"/>
-      <c r="L41" s="7"/>
-      <c r="M41" s="7"/>
+      <c r="K41" s="17"/>
+      <c r="L41" s="17"/>
+      <c r="M41" s="17"/>
       <c r="N41" s="7"/>
       <c r="O41" s="7"/>
       <c r="P41" s="7"/>
       <c r="Q41" s="7"/>
     </row>
     <row r="42" spans="1:17">
-      <c r="A42" s="10">
+      <c r="A42" s="13">
         <v>27</v>
       </c>
-      <c r="B42" s="10" t="s">
+      <c r="B42" s="13" t="s">
         <v>103</v>
       </c>
-      <c r="C42" s="10" t="s">
+      <c r="C42" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="D42" s="12" t="s">
+      <c r="D42" s="14" t="s">
         <v>105</v>
       </c>
-      <c r="E42" s="10"/>
-      <c r="F42" s="10"/>
-      <c r="G42" s="10"/>
-      <c r="H42" s="11">
+      <c r="E42" s="13"/>
+      <c r="F42" s="13"/>
+      <c r="G42" s="13"/>
+      <c r="H42" s="15">
         <v>2610000</v>
       </c>
-      <c r="I42" s="10"/>
-      <c r="J42" s="11">
+      <c r="I42" s="13"/>
+      <c r="J42" s="15">
         <v>2610000</v>
       </c>
-      <c r="K42" s="10"/>
-      <c r="L42" s="10"/>
-      <c r="M42" s="10"/>
-      <c r="N42" s="10"/>
-      <c r="O42" s="10"/>
-      <c r="P42" s="10"/>
-      <c r="Q42" s="10"/>
+      <c r="K42" s="13"/>
+      <c r="L42" s="13"/>
+      <c r="M42" s="13"/>
+      <c r="N42" s="8"/>
+      <c r="O42" s="8"/>
+      <c r="P42" s="8"/>
+      <c r="Q42" s="8"/>
     </row>
     <row r="43" spans="1:17">
-      <c r="A43" s="7">
+      <c r="A43" s="17">
         <v>28</v>
       </c>
-      <c r="B43" s="7" t="s">
+      <c r="B43" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="C43" s="7" t="s">
+      <c r="C43" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="D43" s="9" t="s">
+      <c r="D43" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="E43" s="7"/>
-      <c r="F43" s="7"/>
-      <c r="G43" s="7"/>
-      <c r="H43" s="8">
+      <c r="E43" s="17"/>
+      <c r="F43" s="17"/>
+      <c r="G43" s="17"/>
+      <c r="H43" s="19">
         <v>3496000</v>
       </c>
-      <c r="I43" s="7"/>
-      <c r="J43" s="8">
+      <c r="I43" s="17"/>
+      <c r="J43" s="19">
         <v>3496000</v>
       </c>
-      <c r="K43" s="7"/>
-      <c r="L43" s="7"/>
-      <c r="M43" s="7"/>
+      <c r="K43" s="17"/>
+      <c r="L43" s="17"/>
+      <c r="M43" s="17"/>
       <c r="N43" s="7"/>
       <c r="O43" s="7"/>
       <c r="P43" s="7"/>
       <c r="Q43" s="7"/>
     </row>
     <row r="44" spans="1:17">
-      <c r="A44" s="10">
+      <c r="A44" s="13">
         <v>29</v>
       </c>
-      <c r="B44" s="10" t="s">
+      <c r="B44" s="13" t="s">
         <v>103</v>
       </c>
-      <c r="C44" s="10" t="s">
+      <c r="C44" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="D44" s="12" t="s">
+      <c r="D44" s="14" t="s">
         <v>107</v>
       </c>
-      <c r="E44" s="10"/>
-      <c r="F44" s="10"/>
-      <c r="G44" s="10"/>
-      <c r="H44" s="11">
+      <c r="E44" s="13"/>
+      <c r="F44" s="13"/>
+      <c r="G44" s="13"/>
+      <c r="H44" s="15">
         <v>600000</v>
       </c>
-      <c r="I44" s="10"/>
-      <c r="J44" s="11">
+      <c r="I44" s="13"/>
+      <c r="J44" s="15">
         <v>600000</v>
       </c>
-      <c r="K44" s="10"/>
-      <c r="L44" s="10"/>
-      <c r="M44" s="10"/>
-      <c r="N44" s="10"/>
-      <c r="O44" s="10"/>
-      <c r="P44" s="10"/>
-      <c r="Q44" s="10"/>
+      <c r="K44" s="13"/>
+      <c r="L44" s="13"/>
+      <c r="M44" s="13"/>
+      <c r="N44" s="8"/>
+      <c r="O44" s="8"/>
+      <c r="P44" s="8"/>
+      <c r="Q44" s="8"/>
     </row>
     <row r="45" spans="1:17">
-      <c r="A45" s="7">
+      <c r="A45" s="17">
         <v>30</v>
       </c>
-      <c r="B45" s="7" t="s">
+      <c r="B45" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="C45" s="7" t="s">
+      <c r="C45" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="D45" s="9" t="s">
+      <c r="D45" s="18" t="s">
         <v>108</v>
       </c>
-      <c r="E45" s="7"/>
-      <c r="F45" s="7"/>
-      <c r="G45" s="7"/>
-      <c r="H45" s="8">
+      <c r="E45" s="17"/>
+      <c r="F45" s="17"/>
+      <c r="G45" s="17"/>
+      <c r="H45" s="19">
         <v>640000</v>
       </c>
-      <c r="I45" s="7"/>
-      <c r="J45" s="8">
+      <c r="I45" s="17"/>
+      <c r="J45" s="19">
         <v>640000</v>
       </c>
-      <c r="K45" s="7"/>
-      <c r="L45" s="7"/>
-      <c r="M45" s="7"/>
+      <c r="K45" s="17"/>
+      <c r="L45" s="17"/>
+      <c r="M45" s="17"/>
       <c r="N45" s="7"/>
       <c r="O45" s="7"/>
       <c r="P45" s="7"/>
       <c r="Q45" s="7"/>
     </row>
     <row r="46" spans="1:17">
-      <c r="A46" s="10">
+      <c r="A46" s="13">
         <v>31</v>
       </c>
-      <c r="B46" s="10" t="s">
+      <c r="B46" s="13" t="s">
         <v>103</v>
       </c>
-      <c r="C46" s="10" t="s">
+      <c r="C46" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="D46" s="12" t="s">
+      <c r="D46" s="14" t="s">
         <v>109</v>
       </c>
-      <c r="E46" s="10"/>
-      <c r="F46" s="10"/>
-      <c r="G46" s="10"/>
-      <c r="H46" s="11">
+      <c r="E46" s="13"/>
+      <c r="F46" s="13"/>
+      <c r="G46" s="13"/>
+      <c r="H46" s="15">
         <v>650000</v>
       </c>
-      <c r="I46" s="10"/>
-      <c r="J46" s="11">
+      <c r="I46" s="13"/>
+      <c r="J46" s="15">
         <v>650000</v>
       </c>
-      <c r="K46" s="10"/>
-      <c r="L46" s="10"/>
-      <c r="M46" s="10"/>
-      <c r="N46" s="10"/>
-      <c r="O46" s="10"/>
-      <c r="P46" s="10"/>
-      <c r="Q46" s="10"/>
+      <c r="K46" s="13"/>
+      <c r="L46" s="13"/>
+      <c r="M46" s="13"/>
+      <c r="N46" s="8"/>
+      <c r="O46" s="8"/>
+      <c r="P46" s="8"/>
+      <c r="Q46" s="8"/>
     </row>
     <row r="47" spans="1:17">
-      <c r="A47" s="7">
+      <c r="A47" s="17">
         <v>32</v>
       </c>
-      <c r="B47" s="7" t="s">
+      <c r="B47" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="C47" s="7" t="s">
+      <c r="C47" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="D47" s="9" t="s">
+      <c r="D47" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="E47" s="7"/>
-      <c r="F47" s="7"/>
-      <c r="G47" s="7"/>
-      <c r="H47" s="8">
+      <c r="E47" s="17"/>
+      <c r="F47" s="17"/>
+      <c r="G47" s="17"/>
+      <c r="H47" s="19">
         <v>120000</v>
       </c>
-      <c r="I47" s="7"/>
-      <c r="J47" s="8">
+      <c r="I47" s="17"/>
+      <c r="J47" s="19">
         <v>120000</v>
       </c>
-      <c r="K47" s="7"/>
-      <c r="L47" s="7"/>
-      <c r="M47" s="7"/>
+      <c r="K47" s="17"/>
+      <c r="L47" s="17"/>
+      <c r="M47" s="17"/>
       <c r="N47" s="7"/>
       <c r="O47" s="7"/>
       <c r="P47" s="7"/>
       <c r="Q47" s="7"/>
     </row>
     <row r="48" spans="1:17">
-      <c r="A48" s="10">
+      <c r="A48" s="13">
         <v>33</v>
       </c>
-      <c r="B48" s="10" t="s">
+      <c r="B48" s="13" t="s">
         <v>103</v>
       </c>
-      <c r="C48" s="10" t="s">
+      <c r="C48" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="D48" s="12" t="s">
+      <c r="D48" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="E48" s="10"/>
-      <c r="F48" s="10"/>
-      <c r="G48" s="10"/>
-      <c r="H48" s="11">
+      <c r="E48" s="13"/>
+      <c r="F48" s="13"/>
+      <c r="G48" s="13"/>
+      <c r="H48" s="15">
         <v>222200</v>
       </c>
-      <c r="I48" s="10"/>
-      <c r="J48" s="11">
+      <c r="I48" s="13"/>
+      <c r="J48" s="15">
         <v>222200</v>
       </c>
-      <c r="K48" s="10"/>
-      <c r="L48" s="10"/>
-      <c r="M48" s="10"/>
-      <c r="N48" s="10"/>
-      <c r="O48" s="10"/>
-      <c r="P48" s="10"/>
-      <c r="Q48" s="10"/>
+      <c r="K48" s="13"/>
+      <c r="L48" s="13"/>
+      <c r="M48" s="13"/>
+      <c r="N48" s="8"/>
+      <c r="O48" s="8"/>
+      <c r="P48" s="8"/>
+      <c r="Q48" s="8"/>
     </row>
     <row r="49" spans="1:17">
-      <c r="A49" s="7">
+      <c r="A49" s="17">
         <v>34</v>
       </c>
-      <c r="B49" s="7" t="s">
+      <c r="B49" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="C49" s="7" t="s">
+      <c r="C49" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="D49" s="9" t="s">
+      <c r="D49" s="18" t="s">
         <v>112</v>
       </c>
-      <c r="E49" s="7"/>
-      <c r="F49" s="7"/>
-      <c r="G49" s="7"/>
-      <c r="H49" s="8">
+      <c r="E49" s="17"/>
+      <c r="F49" s="17"/>
+      <c r="G49" s="17"/>
+      <c r="H49" s="19">
         <v>900000</v>
       </c>
-      <c r="I49" s="7"/>
-      <c r="J49" s="8">
+      <c r="I49" s="17"/>
+      <c r="J49" s="19">
         <v>900000</v>
       </c>
-      <c r="K49" s="7"/>
-      <c r="L49" s="7"/>
-      <c r="M49" s="7"/>
+      <c r="K49" s="17"/>
+      <c r="L49" s="17"/>
+      <c r="M49" s="17"/>
       <c r="N49" s="7"/>
       <c r="O49" s="7"/>
       <c r="P49" s="7"/>
       <c r="Q49" s="7"/>
     </row>
     <row r="50" spans="1:17">
-      <c r="A50" s="10">
+      <c r="A50" s="13">
         <v>35</v>
       </c>
-      <c r="B50" s="10" t="s">
+      <c r="B50" s="13" t="s">
         <v>103</v>
       </c>
-      <c r="C50" s="10" t="s">
+      <c r="C50" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="D50" s="12" t="s">
+      <c r="D50" s="14" t="s">
         <v>113</v>
       </c>
-      <c r="E50" s="10"/>
-      <c r="F50" s="10"/>
-      <c r="G50" s="10"/>
-      <c r="H50" s="11">
+      <c r="E50" s="13"/>
+      <c r="F50" s="13"/>
+      <c r="G50" s="13"/>
+      <c r="H50" s="15">
         <v>278500</v>
       </c>
-      <c r="I50" s="10"/>
-      <c r="J50" s="11">
+      <c r="I50" s="13"/>
+      <c r="J50" s="15">
         <v>278500</v>
       </c>
-      <c r="K50" s="10"/>
-      <c r="L50" s="10"/>
-      <c r="M50" s="10"/>
-      <c r="N50" s="10"/>
-      <c r="O50" s="10"/>
-      <c r="P50" s="10"/>
-      <c r="Q50" s="10"/>
+      <c r="K50" s="13"/>
+      <c r="L50" s="13"/>
+      <c r="M50" s="13"/>
+      <c r="N50" s="8"/>
+      <c r="O50" s="8"/>
+      <c r="P50" s="8"/>
+      <c r="Q50" s="8"/>
     </row>
     <row r="51" spans="1:17">
-      <c r="A51" s="7">
+      <c r="A51" s="17">
         <v>36</v>
       </c>
-      <c r="B51" s="7" t="s">
+      <c r="B51" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="C51" s="7" t="s">
+      <c r="C51" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="D51" s="9" t="s">
+      <c r="D51" s="18" t="s">
         <v>114</v>
       </c>
-      <c r="E51" s="7"/>
-      <c r="F51" s="7"/>
-      <c r="G51" s="7"/>
-      <c r="H51" s="8">
+      <c r="E51" s="17"/>
+      <c r="F51" s="17"/>
+      <c r="G51" s="17"/>
+      <c r="H51" s="19">
         <v>225000</v>
       </c>
-      <c r="I51" s="7"/>
-      <c r="J51" s="8">
+      <c r="I51" s="17"/>
+      <c r="J51" s="19">
         <v>225000</v>
       </c>
-      <c r="K51" s="7"/>
-      <c r="L51" s="7"/>
-      <c r="M51" s="7"/>
+      <c r="K51" s="17"/>
+      <c r="L51" s="17"/>
+      <c r="M51" s="17"/>
       <c r="N51" s="7"/>
       <c r="O51" s="7"/>
       <c r="P51" s="7"/>
       <c r="Q51" s="7"/>
     </row>
     <row r="52" spans="1:17">
-      <c r="A52" s="10">
+      <c r="A52" s="13">
         <v>37</v>
       </c>
-      <c r="B52" s="10" t="s">
+      <c r="B52" s="13" t="s">
         <v>103</v>
       </c>
-      <c r="C52" s="10" t="s">
+      <c r="C52" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="D52" s="12" t="s">
+      <c r="D52" s="14" t="s">
         <v>115</v>
       </c>
-      <c r="E52" s="10"/>
-      <c r="F52" s="10"/>
-      <c r="G52" s="10"/>
-      <c r="H52" s="11">
+      <c r="E52" s="13"/>
+      <c r="F52" s="13"/>
+      <c r="G52" s="13"/>
+      <c r="H52" s="15">
         <v>85000</v>
       </c>
-      <c r="I52" s="10"/>
-      <c r="J52" s="11">
+      <c r="I52" s="13"/>
+      <c r="J52" s="15">
         <v>85000</v>
       </c>
-      <c r="K52" s="10"/>
-      <c r="L52" s="10"/>
-      <c r="M52" s="10"/>
-      <c r="N52" s="10"/>
-      <c r="O52" s="10"/>
-      <c r="P52" s="10"/>
-      <c r="Q52" s="10"/>
+      <c r="K52" s="13"/>
+      <c r="L52" s="13"/>
+      <c r="M52" s="13"/>
+      <c r="N52" s="8"/>
+      <c r="O52" s="8"/>
+      <c r="P52" s="8"/>
+      <c r="Q52" s="8"/>
     </row>
     <row r="53" spans="1:17">
-      <c r="A53" s="7">
+      <c r="A53" s="17">
         <v>38</v>
       </c>
-      <c r="B53" s="7" t="s">
+      <c r="B53" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="C53" s="7" t="s">
+      <c r="C53" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="D53" s="9" t="s">
+      <c r="D53" s="18" t="s">
         <v>117</v>
       </c>
-      <c r="E53" s="17" t="s">
+      <c r="E53" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="F53" s="7"/>
-      <c r="G53" s="7"/>
-      <c r="H53" s="8">
+      <c r="F53" s="17"/>
+      <c r="G53" s="17"/>
+      <c r="H53" s="19">
         <v>1800000</v>
       </c>
-      <c r="I53" s="7"/>
-      <c r="J53" s="8">
+      <c r="I53" s="17"/>
+      <c r="J53" s="19">
         <v>1800000</v>
       </c>
-      <c r="K53" s="7"/>
-      <c r="L53" s="7"/>
-      <c r="M53" s="7"/>
+      <c r="K53" s="17"/>
+      <c r="L53" s="17"/>
+      <c r="M53" s="17"/>
       <c r="N53" s="7"/>
       <c r="O53" s="7"/>
       <c r="P53" s="7"/>
       <c r="Q53" s="7"/>
     </row>
     <row r="54" spans="1:17">
-      <c r="A54" s="10">
+      <c r="A54" s="13">
         <v>39</v>
       </c>
-      <c r="B54" s="10" t="s">
+      <c r="B54" s="13" t="s">
         <v>103</v>
       </c>
-      <c r="C54" s="10" t="s">
+      <c r="C54" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="D54" s="12" t="s">
+      <c r="D54" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="E54" s="18" t="s">
+      <c r="E54" s="12" t="s">
         <v>120</v>
       </c>
-      <c r="F54" s="10"/>
-      <c r="G54" s="10"/>
-      <c r="H54" s="11">
+      <c r="F54" s="13"/>
+      <c r="G54" s="13"/>
+      <c r="H54" s="15">
         <v>1120000</v>
       </c>
-      <c r="I54" s="10"/>
-      <c r="J54" s="11">
+      <c r="I54" s="13"/>
+      <c r="J54" s="15">
         <v>1120000</v>
       </c>
-      <c r="K54" s="10"/>
-      <c r="L54" s="10"/>
-      <c r="M54" s="10"/>
-      <c r="N54" s="10"/>
-      <c r="O54" s="10"/>
-      <c r="P54" s="10"/>
-      <c r="Q54" s="10"/>
+      <c r="K54" s="13"/>
+      <c r="L54" s="13"/>
+      <c r="M54" s="13"/>
+      <c r="N54" s="8"/>
+      <c r="O54" s="8"/>
+      <c r="P54" s="8"/>
+      <c r="Q54" s="8"/>
     </row>
     <row r="55" spans="1:17">
-      <c r="A55" s="7">
+      <c r="A55" s="17">
         <v>40</v>
       </c>
-      <c r="B55" s="7" t="s">
+      <c r="B55" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="C55" s="7" t="s">
+      <c r="C55" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="D55" s="9" t="s">
+      <c r="D55" s="18" t="s">
         <v>121</v>
       </c>
-      <c r="E55" s="17" t="s">
+      <c r="E55" s="11" t="s">
         <v>122</v>
       </c>
-      <c r="F55" s="7"/>
-      <c r="G55" s="7"/>
-      <c r="H55" s="8">
+      <c r="F55" s="17"/>
+      <c r="G55" s="17"/>
+      <c r="H55" s="19">
         <v>860000</v>
       </c>
-      <c r="I55" s="7"/>
-      <c r="J55" s="8">
+      <c r="I55" s="17"/>
+      <c r="J55" s="19">
         <v>860000</v>
       </c>
-      <c r="K55" s="7"/>
-      <c r="L55" s="7"/>
-      <c r="M55" s="7"/>
+      <c r="K55" s="17"/>
+      <c r="L55" s="17"/>
+      <c r="M55" s="17"/>
       <c r="N55" s="7"/>
       <c r="O55" s="7"/>
       <c r="P55" s="7"/>
       <c r="Q55" s="7"/>
     </row>
     <row r="56" spans="1:17">
-      <c r="A56" s="10">
+      <c r="A56" s="13">
         <v>41</v>
       </c>
-      <c r="B56" s="10" t="s">
+      <c r="B56" s="13" t="s">
         <v>103</v>
       </c>
-      <c r="C56" s="10" t="s">
+      <c r="C56" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="D56" s="12" t="s">
+      <c r="D56" s="14" t="s">
         <v>123</v>
       </c>
-      <c r="E56" s="18" t="s">
+      <c r="E56" s="12" t="s">
         <v>124</v>
       </c>
-      <c r="F56" s="10"/>
-      <c r="G56" s="10"/>
-      <c r="H56" s="11">
+      <c r="F56" s="13"/>
+      <c r="G56" s="13"/>
+      <c r="H56" s="15">
         <v>500000</v>
       </c>
-      <c r="I56" s="10"/>
-      <c r="J56" s="11">
+      <c r="I56" s="13"/>
+      <c r="J56" s="15">
         <v>500000</v>
       </c>
-      <c r="K56" s="10"/>
-      <c r="L56" s="10"/>
-      <c r="M56" s="10"/>
+      <c r="K56" s="13"/>
+      <c r="L56" s="13"/>
+      <c r="M56" s="13"/>
       <c r="N56" s="6"/>
       <c r="O56" s="6"/>
       <c r="P56" s="6"/>
       <c r="Q56" s="6"/>
     </row>
     <row r="57" spans="1:17">
-      <c r="A57" s="7">
+      <c r="A57" s="17">
         <v>42</v>
       </c>
-      <c r="B57" s="7" t="s">
+      <c r="B57" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="C57" s="7" t="s">
+      <c r="C57" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="D57" s="9" t="s">
+      <c r="D57" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="E57" s="17"/>
-      <c r="F57" s="7"/>
-      <c r="G57" s="7"/>
-      <c r="H57" s="8">
+      <c r="E57" s="11"/>
+      <c r="F57" s="17"/>
+      <c r="G57" s="17"/>
+      <c r="H57" s="19">
         <v>380000</v>
       </c>
-      <c r="I57" s="7"/>
-      <c r="J57" s="8">
+      <c r="I57" s="17"/>
+      <c r="J57" s="19">
         <v>380000</v>
       </c>
-      <c r="K57" s="7"/>
-      <c r="L57" s="7"/>
-      <c r="M57" s="7"/>
+      <c r="K57" s="17"/>
+      <c r="L57" s="17"/>
+      <c r="M57" s="17"/>
     </row>
     <row r="58" spans="1:17">
-      <c r="A58" s="10">
+      <c r="A58" s="13">
         <v>43</v>
       </c>
-      <c r="B58" s="10"/>
-      <c r="C58" s="10"/>
-      <c r="D58" s="10"/>
-      <c r="E58" s="10"/>
-      <c r="F58" s="10"/>
-      <c r="G58" s="10"/>
-      <c r="H58" s="10"/>
-      <c r="I58" s="10"/>
-      <c r="J58" s="10">
+      <c r="B58" s="13"/>
+      <c r="C58" s="13"/>
+      <c r="D58" s="13"/>
+      <c r="E58" s="13"/>
+      <c r="F58" s="13"/>
+      <c r="G58" s="13"/>
+      <c r="H58" s="13"/>
+      <c r="I58" s="13"/>
+      <c r="J58" s="13">
         <v>0</v>
       </c>
-      <c r="K58" s="10"/>
-      <c r="L58" s="10"/>
-      <c r="M58" s="10"/>
+      <c r="K58" s="13"/>
+      <c r="L58" s="13"/>
+      <c r="M58" s="13"/>
     </row>
     <row r="59" spans="1:17">
-      <c r="A59" s="7">
+      <c r="A59" s="17">
         <v>44</v>
       </c>
-      <c r="B59" s="7"/>
-      <c r="C59" s="7"/>
-      <c r="D59" s="7"/>
-      <c r="E59" s="7"/>
-      <c r="F59" s="7"/>
-      <c r="G59" s="7"/>
-      <c r="H59" s="7"/>
-      <c r="I59" s="7"/>
-      <c r="J59" s="7">
+      <c r="B59" s="17"/>
+      <c r="C59" s="17"/>
+      <c r="D59" s="17"/>
+      <c r="E59" s="17"/>
+      <c r="F59" s="17"/>
+      <c r="G59" s="17"/>
+      <c r="H59" s="17"/>
+      <c r="I59" s="17"/>
+      <c r="J59" s="17">
         <v>0</v>
       </c>
-      <c r="K59" s="7"/>
-      <c r="L59" s="7"/>
-      <c r="M59" s="7"/>
+      <c r="K59" s="17"/>
+      <c r="L59" s="17"/>
+      <c r="M59" s="17"/>
     </row>
     <row r="60" spans="1:17">
-      <c r="A60" s="10">
+      <c r="A60" s="13">
         <v>45</v>
       </c>
-      <c r="B60" s="10"/>
-      <c r="C60" s="10"/>
-      <c r="D60" s="10"/>
-      <c r="E60" s="10"/>
-      <c r="F60" s="10"/>
-      <c r="G60" s="10"/>
-      <c r="H60" s="10"/>
-      <c r="I60" s="10"/>
-      <c r="J60" s="10">
+      <c r="B60" s="13"/>
+      <c r="C60" s="13"/>
+      <c r="D60" s="13"/>
+      <c r="E60" s="13"/>
+      <c r="F60" s="13"/>
+      <c r="G60" s="13"/>
+      <c r="H60" s="13"/>
+      <c r="I60" s="13"/>
+      <c r="J60" s="13">
         <v>0</v>
       </c>
-      <c r="K60" s="10"/>
-      <c r="L60" s="10"/>
-      <c r="M60" s="10"/>
+      <c r="K60" s="13"/>
+      <c r="L60" s="13"/>
+      <c r="M60" s="13"/>
     </row>
     <row r="61" spans="1:17">
       <c r="A61" t="s">
         <v>116</v>
       </c>
-      <c r="H61" s="16">
+      <c r="H61" s="10">
         <v>31071804</v>
       </c>
-      <c r="I61" s="16">
+      <c r="I61" s="10">
         <v>3872529.9</v>
       </c>
-      <c r="J61" s="16">
+      <c r="J61" s="10">
         <v>27199274.100000001</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="168">
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="J2:J3"/>
+    <mergeCell ref="K2:K3"/>
+    <mergeCell ref="L2:L3"/>
+    <mergeCell ref="M2:M3"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="I4:I5"/>
+    <mergeCell ref="J4:J5"/>
+    <mergeCell ref="K4:K5"/>
+    <mergeCell ref="L4:L5"/>
+    <mergeCell ref="M4:M5"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="G4:G5"/>
+    <mergeCell ref="H9:H10"/>
+    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="K9:K10"/>
+    <mergeCell ref="L9:L10"/>
+    <mergeCell ref="M9:M10"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="H11:H12"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="K11:K12"/>
+    <mergeCell ref="L11:L12"/>
+    <mergeCell ref="M11:M12"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="G11:G12"/>
+    <mergeCell ref="H14:H15"/>
+    <mergeCell ref="I14:I15"/>
+    <mergeCell ref="J14:J15"/>
+    <mergeCell ref="K14:K15"/>
+    <mergeCell ref="L14:L15"/>
+    <mergeCell ref="M14:M15"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="E14:E15"/>
+    <mergeCell ref="G14:G15"/>
+    <mergeCell ref="H16:H17"/>
+    <mergeCell ref="I16:I17"/>
+    <mergeCell ref="J16:J17"/>
+    <mergeCell ref="K16:K17"/>
+    <mergeCell ref="L16:L17"/>
+    <mergeCell ref="M16:M17"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="E16:E17"/>
+    <mergeCell ref="G16:G17"/>
+    <mergeCell ref="H19:H20"/>
+    <mergeCell ref="I19:I20"/>
+    <mergeCell ref="J19:J20"/>
+    <mergeCell ref="K19:K20"/>
+    <mergeCell ref="L19:L20"/>
+    <mergeCell ref="M19:M20"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="G19:G20"/>
+    <mergeCell ref="H22:H23"/>
+    <mergeCell ref="I22:I23"/>
+    <mergeCell ref="J22:J23"/>
+    <mergeCell ref="K22:K23"/>
+    <mergeCell ref="L22:L23"/>
+    <mergeCell ref="M22:M23"/>
+    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="D22:D23"/>
+    <mergeCell ref="E22:E23"/>
+    <mergeCell ref="G22:G23"/>
+    <mergeCell ref="H24:H25"/>
+    <mergeCell ref="I24:I25"/>
+    <mergeCell ref="J24:J25"/>
+    <mergeCell ref="K24:K25"/>
+    <mergeCell ref="L24:L25"/>
+    <mergeCell ref="M24:M25"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="E24:E25"/>
+    <mergeCell ref="G24:G25"/>
+    <mergeCell ref="H26:H27"/>
+    <mergeCell ref="I26:I27"/>
+    <mergeCell ref="J26:J27"/>
+    <mergeCell ref="K26:K27"/>
+    <mergeCell ref="L26:L27"/>
+    <mergeCell ref="M26:M27"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="C26:C27"/>
+    <mergeCell ref="D26:D27"/>
+    <mergeCell ref="E26:E27"/>
+    <mergeCell ref="G26:G27"/>
+    <mergeCell ref="H28:H29"/>
+    <mergeCell ref="I28:I29"/>
+    <mergeCell ref="J28:J29"/>
+    <mergeCell ref="K28:K29"/>
+    <mergeCell ref="L28:L29"/>
+    <mergeCell ref="M28:M29"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="C28:C29"/>
+    <mergeCell ref="D28:D29"/>
+    <mergeCell ref="E28:E29"/>
+    <mergeCell ref="G28:G29"/>
+    <mergeCell ref="H31:H32"/>
+    <mergeCell ref="I31:I32"/>
+    <mergeCell ref="J31:J32"/>
+    <mergeCell ref="K31:K32"/>
+    <mergeCell ref="L31:L32"/>
+    <mergeCell ref="M31:M32"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="C31:C32"/>
+    <mergeCell ref="D31:D32"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="G31:G32"/>
+    <mergeCell ref="H35:H36"/>
+    <mergeCell ref="I35:I36"/>
+    <mergeCell ref="J35:J36"/>
+    <mergeCell ref="K35:K36"/>
+    <mergeCell ref="L35:L36"/>
+    <mergeCell ref="M35:M36"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="C35:C36"/>
+    <mergeCell ref="D35:D36"/>
+    <mergeCell ref="E35:E36"/>
+    <mergeCell ref="G35:G36"/>
     <mergeCell ref="H38:H39"/>
     <mergeCell ref="I38:I39"/>
     <mergeCell ref="J38:J39"/>
@@ -2878,162 +3076,6 @@
     <mergeCell ref="D38:D39"/>
     <mergeCell ref="E38:E39"/>
     <mergeCell ref="G38:G39"/>
-    <mergeCell ref="H35:H36"/>
-    <mergeCell ref="I35:I36"/>
-    <mergeCell ref="J35:J36"/>
-    <mergeCell ref="K35:K36"/>
-    <mergeCell ref="L35:L36"/>
-    <mergeCell ref="M35:M36"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="B35:B36"/>
-    <mergeCell ref="C35:C36"/>
-    <mergeCell ref="D35:D36"/>
-    <mergeCell ref="E35:E36"/>
-    <mergeCell ref="G35:G36"/>
-    <mergeCell ref="H31:H32"/>
-    <mergeCell ref="I31:I32"/>
-    <mergeCell ref="J31:J32"/>
-    <mergeCell ref="K31:K32"/>
-    <mergeCell ref="L31:L32"/>
-    <mergeCell ref="M31:M32"/>
-    <mergeCell ref="A31:A32"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="C31:C32"/>
-    <mergeCell ref="D31:D32"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="G31:G32"/>
-    <mergeCell ref="H28:H29"/>
-    <mergeCell ref="I28:I29"/>
-    <mergeCell ref="J28:J29"/>
-    <mergeCell ref="K28:K29"/>
-    <mergeCell ref="L28:L29"/>
-    <mergeCell ref="M28:M29"/>
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="B28:B29"/>
-    <mergeCell ref="C28:C29"/>
-    <mergeCell ref="D28:D29"/>
-    <mergeCell ref="E28:E29"/>
-    <mergeCell ref="G28:G29"/>
-    <mergeCell ref="H26:H27"/>
-    <mergeCell ref="I26:I27"/>
-    <mergeCell ref="J26:J27"/>
-    <mergeCell ref="K26:K27"/>
-    <mergeCell ref="L26:L27"/>
-    <mergeCell ref="M26:M27"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="C26:C27"/>
-    <mergeCell ref="D26:D27"/>
-    <mergeCell ref="E26:E27"/>
-    <mergeCell ref="G26:G27"/>
-    <mergeCell ref="H24:H25"/>
-    <mergeCell ref="I24:I25"/>
-    <mergeCell ref="J24:J25"/>
-    <mergeCell ref="K24:K25"/>
-    <mergeCell ref="L24:L25"/>
-    <mergeCell ref="M24:M25"/>
-    <mergeCell ref="A24:A25"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="E24:E25"/>
-    <mergeCell ref="G24:G25"/>
-    <mergeCell ref="H22:H23"/>
-    <mergeCell ref="I22:I23"/>
-    <mergeCell ref="J22:J23"/>
-    <mergeCell ref="K22:K23"/>
-    <mergeCell ref="L22:L23"/>
-    <mergeCell ref="M22:M23"/>
-    <mergeCell ref="A22:A23"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="D22:D23"/>
-    <mergeCell ref="E22:E23"/>
-    <mergeCell ref="G22:G23"/>
-    <mergeCell ref="H19:H20"/>
-    <mergeCell ref="I19:I20"/>
-    <mergeCell ref="J19:J20"/>
-    <mergeCell ref="K19:K20"/>
-    <mergeCell ref="L19:L20"/>
-    <mergeCell ref="M19:M20"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="G19:G20"/>
-    <mergeCell ref="H16:H17"/>
-    <mergeCell ref="I16:I17"/>
-    <mergeCell ref="J16:J17"/>
-    <mergeCell ref="K16:K17"/>
-    <mergeCell ref="L16:L17"/>
-    <mergeCell ref="M16:M17"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="E16:E17"/>
-    <mergeCell ref="G16:G17"/>
-    <mergeCell ref="H14:H15"/>
-    <mergeCell ref="I14:I15"/>
-    <mergeCell ref="J14:J15"/>
-    <mergeCell ref="K14:K15"/>
-    <mergeCell ref="L14:L15"/>
-    <mergeCell ref="M14:M15"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="E14:E15"/>
-    <mergeCell ref="G14:G15"/>
-    <mergeCell ref="H11:H12"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="K11:K12"/>
-    <mergeCell ref="L11:L12"/>
-    <mergeCell ref="M11:M12"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="G11:G12"/>
-    <mergeCell ref="H9:H10"/>
-    <mergeCell ref="I9:I10"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="K9:K10"/>
-    <mergeCell ref="L9:L10"/>
-    <mergeCell ref="M9:M10"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="G9:G10"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="I4:I5"/>
-    <mergeCell ref="J4:J5"/>
-    <mergeCell ref="K4:K5"/>
-    <mergeCell ref="L4:L5"/>
-    <mergeCell ref="M4:M5"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="G4:G5"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="J2:J3"/>
-    <mergeCell ref="K2:K3"/>
-    <mergeCell ref="L2:L3"/>
-    <mergeCell ref="M2:M3"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="G2:G3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update code and excel 4/4/2026
</commit_message>
<xml_diff>
--- a/Investment_Budget_69.xlsx
+++ b/Investment_Budget_69.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="132">
   <si>
     <t>No.</t>
   </si>
@@ -405,13 +405,28 @@
   </si>
   <si>
     <t>On Process</t>
+  </si>
+  <si>
+    <t>https://mitrphol-my.sharepoint.com/:i:/p/waiyawatc/IQB0TkwiEe9LQbMIXhAinnNsAVjhfvVR84xbvcOGJHKHPhk?e=X7cnw6</t>
+  </si>
+  <si>
+    <t>https://mitrphol-my.sharepoint.com/:i:/p/waiyawatc/IQDj7qFw-5IRSbFuORiw8lobAaY82Uoxwx5vknlrFIn6MWo?e=R3PIMH</t>
+  </si>
+  <si>
+    <t>40.71% / 0.98 MB / 2Y</t>
+  </si>
+  <si>
+    <t>62% / 1.97MB / 2Y</t>
+  </si>
+  <si>
+    <t>89% / 0.98MB / 2Y</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -441,15 +456,6 @@
       <u/>
       <sz val="11"/>
       <color rgb="FF0563C1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="222"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="222"/>
@@ -496,9 +502,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -509,52 +515,18 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -578,6 +550,44 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -934,70 +944,70 @@
       </c>
     </row>
     <row r="2" spans="1:17">
-      <c r="A2" s="25">
+      <c r="A2" s="18">
         <v>1</v>
       </c>
-      <c r="B2" s="25" t="s">
+      <c r="B2" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="25" t="s">
+      <c r="C2" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="27" t="s">
+      <c r="D2" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="27" t="s">
+      <c r="E2" s="20" t="s">
         <v>20</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="G2" s="25" t="s">
+      <c r="G2" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="H2" s="24">
+      <c r="H2" s="17">
         <v>350000</v>
       </c>
-      <c r="I2" s="24">
+      <c r="I2" s="17">
         <v>350000</v>
       </c>
-      <c r="J2" s="25">
+      <c r="J2" s="18">
         <v>0</v>
       </c>
-      <c r="K2" s="25">
+      <c r="K2" s="18">
         <v>50</v>
       </c>
-      <c r="L2" s="25" t="s">
+      <c r="L2" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M2" s="26">
+      <c r="M2" s="19">
         <v>46113</v>
       </c>
-      <c r="N2" s="8"/>
-      <c r="O2" s="8"/>
-      <c r="P2" s="9"/>
-      <c r="Q2" s="8"/>
+      <c r="N2" s="18"/>
+      <c r="O2" s="18"/>
+      <c r="P2" s="25"/>
+      <c r="Q2" s="18"/>
     </row>
     <row r="3" spans="1:17">
-      <c r="A3" s="25"/>
-      <c r="B3" s="25"/>
-      <c r="C3" s="25"/>
-      <c r="D3" s="27"/>
-      <c r="E3" s="27"/>
+      <c r="A3" s="18"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
       <c r="F3" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="G3" s="25"/>
-      <c r="H3" s="24"/>
-      <c r="I3" s="24"/>
-      <c r="J3" s="25"/>
-      <c r="K3" s="25"/>
-      <c r="L3" s="25"/>
-      <c r="M3" s="26"/>
-      <c r="N3" s="8"/>
-      <c r="O3" s="8"/>
-      <c r="P3" s="9"/>
-      <c r="Q3" s="8"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="17"/>
+      <c r="I3" s="17"/>
+      <c r="J3" s="18"/>
+      <c r="K3" s="18"/>
+      <c r="L3" s="18"/>
+      <c r="M3" s="19"/>
+      <c r="N3" s="18"/>
+      <c r="O3" s="18"/>
+      <c r="P3" s="25"/>
+      <c r="Q3" s="18"/>
     </row>
     <row r="4" spans="1:17">
       <c r="A4" s="22">
@@ -1009,10 +1019,10 @@
       <c r="C4" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="23" t="s">
+      <c r="D4" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="E4" s="23" t="s">
+      <c r="E4" s="24" t="s">
         <v>27</v>
       </c>
       <c r="F4" s="3" t="s">
@@ -1034,20 +1044,20 @@
       <c r="L4" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="M4" s="28">
+      <c r="M4" s="23">
         <v>46113</v>
       </c>
-      <c r="N4" s="7"/>
-      <c r="O4" s="7"/>
-      <c r="P4" s="7"/>
-      <c r="Q4" s="7"/>
+      <c r="N4" s="22"/>
+      <c r="O4" s="22"/>
+      <c r="P4" s="22"/>
+      <c r="Q4" s="22"/>
     </row>
     <row r="5" spans="1:17">
       <c r="A5" s="22"/>
       <c r="B5" s="22"/>
       <c r="C5" s="22"/>
-      <c r="D5" s="23"/>
-      <c r="E5" s="23"/>
+      <c r="D5" s="24"/>
+      <c r="E5" s="24"/>
       <c r="F5" s="3" t="s">
         <v>29</v>
       </c>
@@ -1057,11 +1067,11 @@
       <c r="J5" s="21"/>
       <c r="K5" s="22"/>
       <c r="L5" s="22"/>
-      <c r="M5" s="28"/>
-      <c r="N5" s="7"/>
-      <c r="O5" s="7"/>
-      <c r="P5" s="7"/>
-      <c r="Q5" s="7"/>
+      <c r="M5" s="23"/>
+      <c r="N5" s="22"/>
+      <c r="O5" s="22"/>
+      <c r="P5" s="22"/>
+      <c r="Q5" s="22"/>
     </row>
     <row r="6" spans="1:17" ht="58">
       <c r="A6" s="13">
@@ -1073,23 +1083,23 @@
       <c r="C6" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="14" t="s">
+      <c r="D6" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="E6" s="14" t="s">
+      <c r="E6" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="F6" s="14" t="s">
+      <c r="F6" s="15" t="s">
         <v>33</v>
       </c>
       <c r="G6" s="13"/>
-      <c r="H6" s="15">
+      <c r="H6" s="12">
         <v>130000</v>
       </c>
-      <c r="I6" s="15">
+      <c r="I6" s="12">
         <v>120000</v>
       </c>
-      <c r="J6" s="15">
+      <c r="J6" s="12">
         <v>10000</v>
       </c>
       <c r="K6" s="13">
@@ -1098,58 +1108,58 @@
       <c r="L6" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="M6" s="16">
+      <c r="M6" s="14">
         <v>46113</v>
       </c>
       <c r="N6" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="O6" s="8"/>
-      <c r="P6" s="8"/>
-      <c r="Q6" s="8"/>
+      <c r="O6" s="13"/>
+      <c r="P6" s="13"/>
+      <c r="Q6" s="13"/>
     </row>
     <row r="7" spans="1:17">
-      <c r="A7" s="17">
+      <c r="A7" s="10">
         <v>4</v>
       </c>
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="E7" s="18" t="s">
+      <c r="E7" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="F7" s="18" t="s">
+      <c r="F7" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="G7" s="17"/>
-      <c r="H7" s="19">
+      <c r="G7" s="10"/>
+      <c r="H7" s="9">
         <v>300000</v>
       </c>
-      <c r="I7" s="19">
+      <c r="I7" s="9">
         <v>280000</v>
       </c>
-      <c r="J7" s="19">
+      <c r="J7" s="9">
         <v>20000</v>
       </c>
-      <c r="K7" s="17">
+      <c r="K7" s="10">
         <v>100</v>
       </c>
-      <c r="L7" s="17" t="s">
+      <c r="L7" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="M7" s="20">
+      <c r="M7" s="16">
         <v>46113</v>
       </c>
-      <c r="N7" s="7"/>
-      <c r="O7" s="7"/>
-      <c r="P7" s="7"/>
-      <c r="Q7" s="7"/>
+      <c r="N7" s="10"/>
+      <c r="O7" s="10"/>
+      <c r="P7" s="10"/>
+      <c r="Q7" s="10"/>
     </row>
     <row r="8" spans="1:17">
       <c r="A8" s="13">
@@ -1161,23 +1171,23 @@
       <c r="C8" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="D8" s="14" t="s">
+      <c r="D8" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="E8" s="14" t="s">
+      <c r="E8" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="F8" s="14" t="s">
+      <c r="F8" s="15" t="s">
         <v>41</v>
       </c>
       <c r="G8" s="13"/>
-      <c r="H8" s="15">
+      <c r="H8" s="12">
         <v>20000</v>
       </c>
-      <c r="I8" s="15">
+      <c r="I8" s="12">
         <v>18614.400000000001</v>
       </c>
-      <c r="J8" s="15">
+      <c r="J8" s="12">
         <v>1385.6</v>
       </c>
       <c r="K8" s="13">
@@ -1186,15 +1196,15 @@
       <c r="L8" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="M8" s="16">
+      <c r="M8" s="14">
         <v>46113</v>
       </c>
       <c r="N8" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="O8" s="8"/>
-      <c r="P8" s="8"/>
-      <c r="Q8" s="8"/>
+      <c r="O8" s="13"/>
+      <c r="P8" s="13"/>
+      <c r="Q8" s="13"/>
     </row>
     <row r="9" spans="1:17">
       <c r="A9" s="22">
@@ -1206,10 +1216,10 @@
       <c r="C9" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="D9" s="23" t="s">
+      <c r="D9" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="E9" s="23" t="s">
+      <c r="E9" s="24" t="s">
         <v>44</v>
       </c>
       <c r="F9" s="3" t="s">
@@ -1231,20 +1241,20 @@
       <c r="L9" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="M9" s="28">
+      <c r="M9" s="23">
         <v>46113</v>
       </c>
-      <c r="N9" s="7"/>
-      <c r="O9" s="7"/>
-      <c r="P9" s="7"/>
-      <c r="Q9" s="7"/>
+      <c r="N9" s="22"/>
+      <c r="O9" s="22"/>
+      <c r="P9" s="22"/>
+      <c r="Q9" s="22"/>
     </row>
     <row r="10" spans="1:17">
       <c r="A10" s="22"/>
       <c r="B10" s="22"/>
       <c r="C10" s="22"/>
-      <c r="D10" s="23"/>
-      <c r="E10" s="23"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
       <c r="F10" s="3" t="s">
         <v>46</v>
       </c>
@@ -1254,182 +1264,182 @@
       <c r="J10" s="22"/>
       <c r="K10" s="22"/>
       <c r="L10" s="22"/>
-      <c r="M10" s="28"/>
-      <c r="N10" s="7"/>
-      <c r="O10" s="7"/>
-      <c r="P10" s="7"/>
-      <c r="Q10" s="7"/>
+      <c r="M10" s="23"/>
+      <c r="N10" s="22"/>
+      <c r="O10" s="22"/>
+      <c r="P10" s="22"/>
+      <c r="Q10" s="22"/>
     </row>
     <row r="11" spans="1:17">
-      <c r="A11" s="25">
+      <c r="A11" s="18">
         <v>7</v>
       </c>
-      <c r="B11" s="25" t="s">
+      <c r="B11" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="25" t="s">
+      <c r="C11" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="D11" s="27" t="s">
+      <c r="D11" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="E11" s="27" t="s">
+      <c r="E11" s="20" t="s">
         <v>49</v>
       </c>
       <c r="F11" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G11" s="25"/>
-      <c r="H11" s="24">
+      <c r="G11" s="18"/>
+      <c r="H11" s="17">
         <v>1490000</v>
       </c>
-      <c r="I11" s="24">
+      <c r="I11" s="17">
         <v>1033230</v>
       </c>
-      <c r="J11" s="24">
+      <c r="J11" s="17">
         <v>456770</v>
       </c>
-      <c r="K11" s="25">
+      <c r="K11" s="18">
         <v>15</v>
       </c>
-      <c r="L11" s="25" t="s">
+      <c r="L11" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M11" s="26">
+      <c r="M11" s="19">
         <v>46113</v>
       </c>
-      <c r="N11" s="8"/>
-      <c r="O11" s="8"/>
-      <c r="P11" s="8"/>
-      <c r="Q11" s="8"/>
+      <c r="N11" s="18"/>
+      <c r="O11" s="18"/>
+      <c r="P11" s="18"/>
+      <c r="Q11" s="18"/>
     </row>
     <row r="12" spans="1:17" ht="29">
-      <c r="A12" s="25"/>
-      <c r="B12" s="25"/>
-      <c r="C12" s="25"/>
-      <c r="D12" s="27"/>
-      <c r="E12" s="27"/>
+      <c r="A12" s="18"/>
+      <c r="B12" s="18"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="20"/>
+      <c r="E12" s="20"/>
       <c r="F12" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="G12" s="25"/>
-      <c r="H12" s="24"/>
-      <c r="I12" s="24"/>
-      <c r="J12" s="24"/>
-      <c r="K12" s="25"/>
-      <c r="L12" s="25"/>
-      <c r="M12" s="26"/>
-      <c r="N12" s="8"/>
-      <c r="O12" s="8"/>
-      <c r="P12" s="8"/>
-      <c r="Q12" s="8"/>
+      <c r="G12" s="18"/>
+      <c r="H12" s="17"/>
+      <c r="I12" s="17"/>
+      <c r="J12" s="17"/>
+      <c r="K12" s="18"/>
+      <c r="L12" s="18"/>
+      <c r="M12" s="19"/>
+      <c r="N12" s="18"/>
+      <c r="O12" s="18"/>
+      <c r="P12" s="18"/>
+      <c r="Q12" s="18"/>
     </row>
     <row r="13" spans="1:17">
-      <c r="A13" s="17">
+      <c r="A13" s="10">
         <v>8</v>
       </c>
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="17" t="s">
+      <c r="C13" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="D13" s="18" t="s">
+      <c r="D13" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="E13" s="18" t="s">
+      <c r="E13" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="F13" s="18" t="s">
+      <c r="F13" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="G13" s="17"/>
-      <c r="H13" s="19">
+      <c r="G13" s="10"/>
+      <c r="H13" s="9">
         <v>400000</v>
       </c>
-      <c r="I13" s="19">
+      <c r="I13" s="9">
         <v>399690</v>
       </c>
-      <c r="J13" s="17">
+      <c r="J13" s="10">
         <v>310</v>
       </c>
-      <c r="K13" s="17">
+      <c r="K13" s="10">
         <v>10</v>
       </c>
-      <c r="L13" s="17" t="s">
+      <c r="L13" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="M13" s="20">
+      <c r="M13" s="16">
         <v>46113</v>
       </c>
-      <c r="N13" s="7"/>
-      <c r="O13" s="7"/>
-      <c r="P13" s="7"/>
-      <c r="Q13" s="7"/>
+      <c r="N13" s="10"/>
+      <c r="O13" s="10"/>
+      <c r="P13" s="10"/>
+      <c r="Q13" s="10"/>
     </row>
     <row r="14" spans="1:17">
-      <c r="A14" s="25">
+      <c r="A14" s="18">
         <v>9</v>
       </c>
-      <c r="B14" s="25" t="s">
+      <c r="B14" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="C14" s="25" t="s">
+      <c r="C14" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="D14" s="27" t="s">
+      <c r="D14" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="E14" s="27" t="s">
+      <c r="E14" s="20" t="s">
         <v>57</v>
       </c>
       <c r="F14" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="G14" s="25"/>
-      <c r="H14" s="24">
+      <c r="G14" s="18"/>
+      <c r="H14" s="17">
         <v>1200000</v>
       </c>
-      <c r="I14" s="24">
+      <c r="I14" s="17">
         <v>1100000</v>
       </c>
-      <c r="J14" s="24">
+      <c r="J14" s="17">
         <v>100000</v>
       </c>
-      <c r="K14" s="25">
+      <c r="K14" s="18">
         <v>10</v>
       </c>
-      <c r="L14" s="25" t="s">
+      <c r="L14" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M14" s="26">
+      <c r="M14" s="19">
         <v>46104</v>
       </c>
-      <c r="N14" s="8"/>
-      <c r="O14" s="8"/>
-      <c r="P14" s="8"/>
-      <c r="Q14" s="8"/>
+      <c r="N14" s="18"/>
+      <c r="O14" s="18"/>
+      <c r="P14" s="18"/>
+      <c r="Q14" s="18"/>
     </row>
     <row r="15" spans="1:17">
-      <c r="A15" s="25"/>
-      <c r="B15" s="25"/>
-      <c r="C15" s="25"/>
-      <c r="D15" s="27"/>
-      <c r="E15" s="27"/>
+      <c r="A15" s="18"/>
+      <c r="B15" s="18"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="20"/>
       <c r="F15" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="G15" s="25"/>
-      <c r="H15" s="24"/>
-      <c r="I15" s="24"/>
-      <c r="J15" s="24"/>
-      <c r="K15" s="25"/>
-      <c r="L15" s="25"/>
-      <c r="M15" s="26"/>
-      <c r="N15" s="8"/>
-      <c r="O15" s="8"/>
-      <c r="P15" s="8"/>
-      <c r="Q15" s="8"/>
+      <c r="G15" s="18"/>
+      <c r="H15" s="17"/>
+      <c r="I15" s="17"/>
+      <c r="J15" s="17"/>
+      <c r="K15" s="18"/>
+      <c r="L15" s="18"/>
+      <c r="M15" s="19"/>
+      <c r="N15" s="18"/>
+      <c r="O15" s="18"/>
+      <c r="P15" s="18"/>
+      <c r="Q15" s="18"/>
     </row>
     <row r="16" spans="1:17">
       <c r="A16" s="22">
@@ -1441,10 +1451,10 @@
       <c r="C16" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="D16" s="23" t="s">
+      <c r="D16" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="E16" s="23" t="s">
+      <c r="E16" s="24" t="s">
         <v>49</v>
       </c>
       <c r="F16" s="3" t="s">
@@ -1464,20 +1474,20 @@
       <c r="L16" s="22" t="s">
         <v>60</v>
       </c>
-      <c r="M16" s="28">
+      <c r="M16" s="23">
         <v>46104</v>
       </c>
-      <c r="N16" s="7"/>
-      <c r="O16" s="7"/>
-      <c r="P16" s="7"/>
-      <c r="Q16" s="7"/>
+      <c r="N16" s="22"/>
+      <c r="O16" s="22"/>
+      <c r="P16" s="22"/>
+      <c r="Q16" s="22"/>
     </row>
     <row r="17" spans="1:17" ht="29">
       <c r="A17" s="22"/>
       <c r="B17" s="22"/>
       <c r="C17" s="22"/>
-      <c r="D17" s="23"/>
-      <c r="E17" s="23"/>
+      <c r="D17" s="24"/>
+      <c r="E17" s="24"/>
       <c r="F17" s="3" t="s">
         <v>51</v>
       </c>
@@ -1487,11 +1497,11 @@
       <c r="J17" s="21"/>
       <c r="K17" s="22"/>
       <c r="L17" s="22"/>
-      <c r="M17" s="28"/>
-      <c r="N17" s="7"/>
-      <c r="O17" s="7"/>
-      <c r="P17" s="7"/>
-      <c r="Q17" s="7"/>
+      <c r="M17" s="23"/>
+      <c r="N17" s="22"/>
+      <c r="O17" s="22"/>
+      <c r="P17" s="22"/>
+      <c r="Q17" s="22"/>
     </row>
     <row r="18" spans="1:17">
       <c r="A18" s="13">
@@ -1503,32 +1513,32 @@
       <c r="C18" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="D18" s="14" t="s">
+      <c r="D18" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="E18" s="14" t="s">
+      <c r="E18" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="F18" s="14" t="s">
+      <c r="F18" s="15" t="s">
         <v>54</v>
       </c>
       <c r="G18" s="13"/>
-      <c r="H18" s="15">
+      <c r="H18" s="12">
         <v>450000</v>
       </c>
       <c r="I18" s="13"/>
-      <c r="J18" s="15">
+      <c r="J18" s="12">
         <v>450000</v>
       </c>
       <c r="K18" s="13"/>
       <c r="L18" s="13"/>
-      <c r="M18" s="16">
+      <c r="M18" s="14">
         <v>46104</v>
       </c>
-      <c r="N18" s="8"/>
-      <c r="O18" s="8"/>
-      <c r="P18" s="8"/>
-      <c r="Q18" s="8" t="s">
+      <c r="N18" s="13"/>
+      <c r="O18" s="13"/>
+      <c r="P18" s="13"/>
+      <c r="Q18" s="13" t="s">
         <v>61</v>
       </c>
     </row>
@@ -1542,10 +1552,10 @@
       <c r="C19" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="D19" s="23" t="s">
+      <c r="D19" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="E19" s="23" t="s">
+      <c r="E19" s="24" t="s">
         <v>49</v>
       </c>
       <c r="F19" s="3" t="s">
@@ -1565,20 +1575,20 @@
       <c r="L19" s="22" t="s">
         <v>60</v>
       </c>
-      <c r="M19" s="28">
+      <c r="M19" s="23">
         <v>46104</v>
       </c>
-      <c r="N19" s="7"/>
-      <c r="O19" s="7"/>
-      <c r="P19" s="7"/>
-      <c r="Q19" s="7"/>
+      <c r="N19" s="22"/>
+      <c r="O19" s="22"/>
+      <c r="P19" s="22"/>
+      <c r="Q19" s="22"/>
     </row>
     <row r="20" spans="1:17" ht="29">
       <c r="A20" s="22"/>
       <c r="B20" s="22"/>
       <c r="C20" s="22"/>
-      <c r="D20" s="23"/>
-      <c r="E20" s="23"/>
+      <c r="D20" s="24"/>
+      <c r="E20" s="24"/>
       <c r="F20" s="3" t="s">
         <v>51</v>
       </c>
@@ -1588,11 +1598,11 @@
       <c r="J20" s="21"/>
       <c r="K20" s="22"/>
       <c r="L20" s="22"/>
-      <c r="M20" s="28"/>
-      <c r="N20" s="7"/>
-      <c r="O20" s="7"/>
-      <c r="P20" s="7"/>
-      <c r="Q20" s="7"/>
+      <c r="M20" s="23"/>
+      <c r="N20" s="22"/>
+      <c r="O20" s="22"/>
+      <c r="P20" s="22"/>
+      <c r="Q20" s="22"/>
     </row>
     <row r="21" spans="1:17">
       <c r="A21" s="13">
@@ -1604,32 +1614,32 @@
       <c r="C21" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="D21" s="14" t="s">
+      <c r="D21" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="E21" s="14" t="s">
+      <c r="E21" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="F21" s="14" t="s">
+      <c r="F21" s="15" t="s">
         <v>54</v>
       </c>
       <c r="G21" s="13"/>
-      <c r="H21" s="15">
+      <c r="H21" s="12">
         <v>945000</v>
       </c>
       <c r="I21" s="13"/>
-      <c r="J21" s="15">
+      <c r="J21" s="12">
         <v>945000</v>
       </c>
       <c r="K21" s="13"/>
       <c r="L21" s="13"/>
-      <c r="M21" s="16">
+      <c r="M21" s="14">
         <v>46104</v>
       </c>
-      <c r="N21" s="8"/>
-      <c r="O21" s="8"/>
-      <c r="P21" s="8"/>
-      <c r="Q21" s="8" t="s">
+      <c r="N21" s="13"/>
+      <c r="O21" s="13"/>
+      <c r="P21" s="13"/>
+      <c r="Q21" s="13" t="s">
         <v>61</v>
       </c>
     </row>
@@ -1643,10 +1653,10 @@
       <c r="C22" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="D22" s="23" t="s">
+      <c r="D22" s="24" t="s">
         <v>64</v>
       </c>
-      <c r="E22" s="23" t="s">
+      <c r="E22" s="24" t="s">
         <v>65</v>
       </c>
       <c r="F22" s="3" t="s">
@@ -1670,20 +1680,20 @@
       <c r="L22" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="M22" s="28">
+      <c r="M22" s="23">
         <v>46114</v>
       </c>
-      <c r="N22" s="7"/>
-      <c r="O22" s="7"/>
-      <c r="P22" s="7"/>
-      <c r="Q22" s="7"/>
+      <c r="N22" s="22"/>
+      <c r="O22" s="22"/>
+      <c r="P22" s="22"/>
+      <c r="Q22" s="22"/>
     </row>
     <row r="23" spans="1:17">
       <c r="A23" s="22"/>
       <c r="B23" s="22"/>
       <c r="C23" s="22"/>
-      <c r="D23" s="23"/>
-      <c r="E23" s="23"/>
+      <c r="D23" s="24"/>
+      <c r="E23" s="24"/>
       <c r="F23" s="3" t="s">
         <v>67</v>
       </c>
@@ -1693,77 +1703,81 @@
       <c r="J23" s="22"/>
       <c r="K23" s="22"/>
       <c r="L23" s="22"/>
-      <c r="M23" s="28"/>
-      <c r="N23" s="7"/>
-      <c r="O23" s="7"/>
-      <c r="P23" s="7"/>
-      <c r="Q23" s="7"/>
+      <c r="M23" s="23"/>
+      <c r="N23" s="22"/>
+      <c r="O23" s="22"/>
+      <c r="P23" s="22"/>
+      <c r="Q23" s="22"/>
     </row>
     <row r="24" spans="1:17">
-      <c r="A24" s="25">
+      <c r="A24" s="18">
         <v>15</v>
       </c>
-      <c r="B24" s="25" t="s">
+      <c r="B24" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="C24" s="25" t="s">
+      <c r="C24" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="D24" s="27" t="s">
+      <c r="D24" s="20" t="s">
         <v>69</v>
       </c>
-      <c r="E24" s="27" t="s">
+      <c r="E24" s="20" t="s">
         <v>70</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="G24" s="25" t="s">
+      <c r="G24" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="H24" s="24">
+      <c r="H24" s="17">
         <v>370000</v>
       </c>
-      <c r="I24" s="24">
+      <c r="I24" s="17">
         <v>370000</v>
       </c>
-      <c r="J24" s="25">
+      <c r="J24" s="18">
         <v>0</v>
       </c>
-      <c r="K24" s="25">
+      <c r="K24" s="18">
         <v>70</v>
       </c>
-      <c r="L24" s="25" t="s">
+      <c r="L24" s="18" t="s">
         <v>126</v>
       </c>
-      <c r="M24" s="26">
+      <c r="M24" s="19">
         <v>46114</v>
       </c>
-      <c r="N24" s="8"/>
-      <c r="O24" s="8"/>
-      <c r="P24" s="8"/>
-      <c r="Q24" s="8"/>
+      <c r="N24" s="29" t="s">
+        <v>127</v>
+      </c>
+      <c r="O24" s="30" t="s">
+        <v>127</v>
+      </c>
+      <c r="P24" s="18"/>
+      <c r="Q24" s="18"/>
     </row>
     <row r="25" spans="1:17">
-      <c r="A25" s="25"/>
-      <c r="B25" s="25"/>
-      <c r="C25" s="25"/>
-      <c r="D25" s="27"/>
-      <c r="E25" s="27"/>
+      <c r="A25" s="18"/>
+      <c r="B25" s="18"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="20"/>
       <c r="F25" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="G25" s="25"/>
-      <c r="H25" s="24"/>
-      <c r="I25" s="24"/>
-      <c r="J25" s="25"/>
-      <c r="K25" s="25"/>
-      <c r="L25" s="25"/>
-      <c r="M25" s="26"/>
-      <c r="N25" s="8"/>
-      <c r="O25" s="8"/>
-      <c r="P25" s="8"/>
-      <c r="Q25" s="8"/>
+      <c r="G25" s="18"/>
+      <c r="H25" s="17"/>
+      <c r="I25" s="17"/>
+      <c r="J25" s="18"/>
+      <c r="K25" s="18"/>
+      <c r="L25" s="18"/>
+      <c r="M25" s="19"/>
+      <c r="N25" s="29"/>
+      <c r="O25" s="30"/>
+      <c r="P25" s="18"/>
+      <c r="Q25" s="18"/>
     </row>
     <row r="26" spans="1:17">
       <c r="A26" s="22">
@@ -1775,10 +1789,10 @@
       <c r="C26" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="D26" s="23" t="s">
+      <c r="D26" s="24" t="s">
         <v>74</v>
       </c>
-      <c r="E26" s="23" t="s">
+      <c r="E26" s="24" t="s">
         <v>75</v>
       </c>
       <c r="F26" s="3" t="s">
@@ -1800,20 +1814,20 @@
       <c r="L26" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="M26" s="28">
+      <c r="M26" s="23">
         <v>46114</v>
       </c>
-      <c r="N26" s="7"/>
-      <c r="O26" s="7"/>
-      <c r="P26" s="7"/>
-      <c r="Q26" s="7"/>
+      <c r="N26" s="22"/>
+      <c r="O26" s="22"/>
+      <c r="P26" s="22"/>
+      <c r="Q26" s="22"/>
     </row>
     <row r="27" spans="1:17">
       <c r="A27" s="22"/>
       <c r="B27" s="22"/>
       <c r="C27" s="22"/>
-      <c r="D27" s="23"/>
-      <c r="E27" s="23"/>
+      <c r="D27" s="24"/>
+      <c r="E27" s="24"/>
       <c r="F27" s="3" t="s">
         <v>77</v>
       </c>
@@ -1823,227 +1837,229 @@
       <c r="J27" s="21"/>
       <c r="K27" s="22"/>
       <c r="L27" s="22"/>
-      <c r="M27" s="28"/>
-      <c r="N27" s="7"/>
-      <c r="O27" s="7"/>
-      <c r="P27" s="7"/>
-      <c r="Q27" s="7"/>
+      <c r="M27" s="23"/>
+      <c r="N27" s="22"/>
+      <c r="O27" s="22"/>
+      <c r="P27" s="22"/>
+      <c r="Q27" s="22"/>
     </row>
     <row r="28" spans="1:17">
-      <c r="A28" s="25">
+      <c r="A28" s="18">
         <v>17</v>
       </c>
-      <c r="B28" s="25" t="s">
+      <c r="B28" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="C28" s="25" t="s">
+      <c r="C28" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="D28" s="27" t="s">
+      <c r="D28" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="E28" s="27" t="s">
+      <c r="E28" s="20" t="s">
         <v>79</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="G28" s="25"/>
-      <c r="H28" s="24">
+      <c r="G28" s="18"/>
+      <c r="H28" s="17">
         <v>110000</v>
       </c>
-      <c r="I28" s="25">
+      <c r="I28" s="18">
         <v>0</v>
       </c>
-      <c r="J28" s="24">
+      <c r="J28" s="17">
         <v>110000</v>
       </c>
-      <c r="K28" s="25">
+      <c r="K28" s="18">
         <v>5</v>
       </c>
-      <c r="L28" s="25" t="s">
+      <c r="L28" s="18" t="s">
         <v>60</v>
       </c>
-      <c r="M28" s="26">
+      <c r="M28" s="19">
         <v>46114</v>
       </c>
-      <c r="N28" s="8"/>
-      <c r="O28" s="8"/>
-      <c r="P28" s="8"/>
-      <c r="Q28" s="8"/>
+      <c r="N28" s="18"/>
+      <c r="O28" s="18"/>
+      <c r="P28" s="18"/>
+      <c r="Q28" s="18"/>
     </row>
     <row r="29" spans="1:17">
-      <c r="A29" s="25"/>
-      <c r="B29" s="25"/>
-      <c r="C29" s="25"/>
-      <c r="D29" s="27"/>
-      <c r="E29" s="27"/>
+      <c r="A29" s="18"/>
+      <c r="B29" s="18"/>
+      <c r="C29" s="18"/>
+      <c r="D29" s="20"/>
+      <c r="E29" s="20"/>
       <c r="F29" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="G29" s="25"/>
-      <c r="H29" s="24"/>
-      <c r="I29" s="25"/>
-      <c r="J29" s="24"/>
-      <c r="K29" s="25"/>
-      <c r="L29" s="25"/>
-      <c r="M29" s="26"/>
-      <c r="N29" s="8"/>
-      <c r="O29" s="8"/>
-      <c r="P29" s="8"/>
-      <c r="Q29" s="8"/>
+      <c r="G29" s="18"/>
+      <c r="H29" s="17"/>
+      <c r="I29" s="18"/>
+      <c r="J29" s="17"/>
+      <c r="K29" s="18"/>
+      <c r="L29" s="18"/>
+      <c r="M29" s="19"/>
+      <c r="N29" s="18"/>
+      <c r="O29" s="18"/>
+      <c r="P29" s="18"/>
+      <c r="Q29" s="18"/>
     </row>
     <row r="30" spans="1:17">
-      <c r="A30" s="17">
+      <c r="A30" s="10">
         <v>18</v>
       </c>
-      <c r="B30" s="17" t="s">
+      <c r="B30" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="C30" s="17" t="s">
+      <c r="C30" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="D30" s="18" t="s">
+      <c r="D30" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="E30" s="18" t="s">
+      <c r="E30" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="F30" s="18" t="s">
+      <c r="F30" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="G30" s="17" t="s">
+      <c r="G30" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="H30" s="19">
+      <c r="H30" s="9">
         <v>1000000</v>
       </c>
-      <c r="I30" s="19">
+      <c r="I30" s="9">
         <v>950000</v>
       </c>
-      <c r="J30" s="19">
+      <c r="J30" s="9">
         <v>50000</v>
       </c>
-      <c r="K30" s="17">
+      <c r="K30" s="10">
         <v>10</v>
       </c>
-      <c r="L30" s="17" t="s">
+      <c r="L30" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="M30" s="20">
+      <c r="M30" s="16">
         <v>46114</v>
       </c>
-      <c r="N30" s="7"/>
-      <c r="O30" s="7"/>
-      <c r="P30" s="7"/>
-      <c r="Q30" s="7"/>
+      <c r="N30" s="10"/>
+      <c r="O30" s="10"/>
+      <c r="P30" s="10"/>
+      <c r="Q30" s="10"/>
     </row>
     <row r="31" spans="1:17">
-      <c r="A31" s="25">
+      <c r="A31" s="18">
         <v>19</v>
       </c>
-      <c r="B31" s="25" t="s">
+      <c r="B31" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="C31" s="25" t="s">
+      <c r="C31" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="D31" s="27" t="s">
+      <c r="D31" s="20" t="s">
         <v>86</v>
       </c>
-      <c r="E31" s="27" t="s">
+      <c r="E31" s="20" t="s">
         <v>87</v>
       </c>
       <c r="F31" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="G31" s="25"/>
-      <c r="H31" s="24">
+      <c r="G31" s="18"/>
+      <c r="H31" s="17">
         <v>28000</v>
       </c>
-      <c r="I31" s="24">
+      <c r="I31" s="17">
         <v>20250</v>
       </c>
-      <c r="J31" s="24">
+      <c r="J31" s="17">
         <v>7750</v>
       </c>
-      <c r="K31" s="25">
+      <c r="K31" s="18">
         <v>10</v>
       </c>
-      <c r="L31" s="25" t="s">
+      <c r="L31" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M31" s="26">
+      <c r="M31" s="19">
         <v>46114</v>
       </c>
-      <c r="N31" s="8"/>
-      <c r="O31" s="8"/>
-      <c r="P31" s="8"/>
-      <c r="Q31" s="8"/>
+      <c r="N31" s="18"/>
+      <c r="O31" s="18"/>
+      <c r="P31" s="18"/>
+      <c r="Q31" s="18"/>
     </row>
     <row r="32" spans="1:17">
-      <c r="A32" s="25"/>
-      <c r="B32" s="25"/>
-      <c r="C32" s="25"/>
-      <c r="D32" s="27"/>
-      <c r="E32" s="27"/>
+      <c r="A32" s="18"/>
+      <c r="B32" s="18"/>
+      <c r="C32" s="18"/>
+      <c r="D32" s="20"/>
+      <c r="E32" s="20"/>
       <c r="F32" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="G32" s="25"/>
-      <c r="H32" s="24"/>
-      <c r="I32" s="24"/>
-      <c r="J32" s="24"/>
-      <c r="K32" s="25"/>
-      <c r="L32" s="25"/>
-      <c r="M32" s="26"/>
-      <c r="N32" s="8"/>
-      <c r="O32" s="8"/>
-      <c r="P32" s="8"/>
-      <c r="Q32" s="8"/>
+      <c r="G32" s="18"/>
+      <c r="H32" s="17"/>
+      <c r="I32" s="17"/>
+      <c r="J32" s="17"/>
+      <c r="K32" s="18"/>
+      <c r="L32" s="18"/>
+      <c r="M32" s="19"/>
+      <c r="N32" s="18"/>
+      <c r="O32" s="18"/>
+      <c r="P32" s="18"/>
+      <c r="Q32" s="18"/>
     </row>
     <row r="33" spans="1:17">
-      <c r="A33" s="17">
+      <c r="A33" s="10">
         <v>20</v>
       </c>
-      <c r="B33" s="17" t="s">
+      <c r="B33" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="C33" s="17" t="s">
+      <c r="C33" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="D33" s="18" t="s">
+      <c r="D33" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="E33" s="18" t="s">
+      <c r="E33" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="F33" s="18" t="s">
+      <c r="F33" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="G33" s="17"/>
-      <c r="H33" s="19">
+      <c r="G33" s="10"/>
+      <c r="H33" s="9">
         <v>140000</v>
       </c>
-      <c r="I33" s="19">
+      <c r="I33" s="9">
         <v>115000</v>
       </c>
-      <c r="J33" s="19">
+      <c r="J33" s="9">
         <v>25000</v>
       </c>
-      <c r="K33" s="17">
+      <c r="K33" s="10">
         <v>80</v>
       </c>
-      <c r="L33" s="17" t="s">
+      <c r="L33" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="M33" s="20">
+      <c r="M33" s="16">
         <v>46114</v>
       </c>
-      <c r="N33" s="7"/>
-      <c r="O33" s="7"/>
-      <c r="P33" s="7"/>
-      <c r="Q33" s="7"/>
+      <c r="N33" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="O33" s="10"/>
+      <c r="P33" s="10"/>
+      <c r="Q33" s="10"/>
     </row>
     <row r="34" spans="1:17">
       <c r="A34" s="13">
@@ -2055,23 +2071,23 @@
       <c r="C34" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="D34" s="14" t="s">
+      <c r="D34" s="15" t="s">
         <v>93</v>
       </c>
-      <c r="E34" s="14" t="s">
+      <c r="E34" s="15" t="s">
         <v>94</v>
       </c>
-      <c r="F34" s="14" t="s">
+      <c r="F34" s="15" t="s">
         <v>41</v>
       </c>
       <c r="G34" s="13"/>
-      <c r="H34" s="15">
+      <c r="H34" s="12">
         <v>20000</v>
       </c>
-      <c r="I34" s="15">
+      <c r="I34" s="12">
         <v>18614</v>
       </c>
-      <c r="J34" s="15">
+      <c r="J34" s="12">
         <v>1386</v>
       </c>
       <c r="K34" s="13">
@@ -2080,13 +2096,13 @@
       <c r="L34" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="M34" s="16">
+      <c r="M34" s="14">
         <v>46114</v>
       </c>
-      <c r="N34" s="8"/>
-      <c r="O34" s="8"/>
-      <c r="P34" s="8"/>
-      <c r="Q34" s="8"/>
+      <c r="N34" s="13"/>
+      <c r="O34" s="13"/>
+      <c r="P34" s="13"/>
+      <c r="Q34" s="13"/>
     </row>
     <row r="35" spans="1:17">
       <c r="A35" s="22">
@@ -2098,10 +2114,10 @@
       <c r="C35" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="D35" s="23" t="s">
+      <c r="D35" s="24" t="s">
         <v>95</v>
       </c>
-      <c r="E35" s="23" t="s">
+      <c r="E35" s="24" t="s">
         <v>96</v>
       </c>
       <c r="F35" s="3" t="s">
@@ -2125,20 +2141,20 @@
       <c r="L35" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="M35" s="28">
+      <c r="M35" s="23">
         <v>46114</v>
       </c>
-      <c r="N35" s="7"/>
-      <c r="O35" s="7"/>
-      <c r="P35" s="7"/>
-      <c r="Q35" s="7"/>
+      <c r="N35" s="22"/>
+      <c r="O35" s="22"/>
+      <c r="P35" s="22"/>
+      <c r="Q35" s="22"/>
     </row>
     <row r="36" spans="1:17">
       <c r="A36" s="22"/>
       <c r="B36" s="22"/>
       <c r="C36" s="22"/>
-      <c r="D36" s="23"/>
-      <c r="E36" s="23"/>
+      <c r="D36" s="24"/>
+      <c r="E36" s="24"/>
       <c r="F36" s="3" t="s">
         <v>98</v>
       </c>
@@ -2148,11 +2164,11 @@
       <c r="J36" s="21"/>
       <c r="K36" s="22"/>
       <c r="L36" s="22"/>
-      <c r="M36" s="28"/>
-      <c r="N36" s="7"/>
-      <c r="O36" s="7"/>
-      <c r="P36" s="7"/>
-      <c r="Q36" s="7"/>
+      <c r="M36" s="23"/>
+      <c r="N36" s="22"/>
+      <c r="O36" s="22"/>
+      <c r="P36" s="22"/>
+      <c r="Q36" s="22"/>
     </row>
     <row r="37" spans="1:17">
       <c r="A37" s="13">
@@ -2164,23 +2180,23 @@
       <c r="C37" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="D37" s="14" t="s">
+      <c r="D37" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="E37" s="14" t="s">
+      <c r="E37" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="F37" s="14" t="s">
+      <c r="F37" s="15" t="s">
         <v>102</v>
       </c>
       <c r="G37" s="13"/>
-      <c r="H37" s="15">
+      <c r="H37" s="12">
         <v>20000</v>
       </c>
-      <c r="I37" s="15">
+      <c r="I37" s="12">
         <v>15580</v>
       </c>
-      <c r="J37" s="15">
+      <c r="J37" s="12">
         <v>4420</v>
       </c>
       <c r="K37" s="13">
@@ -2189,13 +2205,13 @@
       <c r="L37" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="M37" s="16">
+      <c r="M37" s="14">
         <v>46114</v>
       </c>
-      <c r="N37" s="8"/>
-      <c r="O37" s="8"/>
-      <c r="P37" s="8"/>
-      <c r="Q37" s="8"/>
+      <c r="N37" s="13"/>
+      <c r="O37" s="13"/>
+      <c r="P37" s="13"/>
+      <c r="Q37" s="13"/>
     </row>
     <row r="38" spans="1:17">
       <c r="A38" s="22">
@@ -2207,10 +2223,10 @@
       <c r="C38" s="22" t="s">
         <v>47</v>
       </c>
-      <c r="D38" s="23" t="s">
+      <c r="D38" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="E38" s="23" t="s">
+      <c r="E38" s="24" t="s">
         <v>49</v>
       </c>
       <c r="F38" s="3" t="s">
@@ -2232,20 +2248,20 @@
       <c r="L38" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="M38" s="28">
+      <c r="M38" s="23">
         <v>46114</v>
       </c>
-      <c r="N38" s="7"/>
-      <c r="O38" s="7"/>
-      <c r="P38" s="7"/>
-      <c r="Q38" s="7"/>
+      <c r="N38" s="22"/>
+      <c r="O38" s="22"/>
+      <c r="P38" s="22"/>
+      <c r="Q38" s="22"/>
     </row>
     <row r="39" spans="1:17" ht="29">
       <c r="A39" s="22"/>
       <c r="B39" s="22"/>
       <c r="C39" s="22"/>
-      <c r="D39" s="23"/>
-      <c r="E39" s="23"/>
+      <c r="D39" s="24"/>
+      <c r="E39" s="24"/>
       <c r="F39" s="3" t="s">
         <v>51</v>
       </c>
@@ -2255,11 +2271,11 @@
       <c r="J39" s="21"/>
       <c r="K39" s="22"/>
       <c r="L39" s="22"/>
-      <c r="M39" s="28"/>
-      <c r="N39" s="7"/>
-      <c r="O39" s="7"/>
-      <c r="P39" s="7"/>
-      <c r="Q39" s="7"/>
+      <c r="M39" s="23"/>
+      <c r="N39" s="22"/>
+      <c r="O39" s="22"/>
+      <c r="P39" s="22"/>
+      <c r="Q39" s="22"/>
     </row>
     <row r="40" spans="1:17">
       <c r="A40" s="13">
@@ -2271,23 +2287,23 @@
       <c r="C40" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="D40" s="14" t="s">
+      <c r="D40" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="E40" s="14" t="s">
+      <c r="E40" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="F40" s="14" t="s">
+      <c r="F40" s="15" t="s">
         <v>54</v>
       </c>
       <c r="G40" s="13"/>
-      <c r="H40" s="15">
+      <c r="H40" s="12">
         <v>370000</v>
       </c>
-      <c r="I40" s="15">
+      <c r="I40" s="12">
         <v>225000</v>
       </c>
-      <c r="J40" s="15">
+      <c r="J40" s="12">
         <v>145000</v>
       </c>
       <c r="K40" s="13">
@@ -2296,44 +2312,52 @@
       <c r="L40" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="M40" s="16">
+      <c r="M40" s="14">
         <v>46114</v>
       </c>
-      <c r="N40" s="8"/>
-      <c r="O40" s="8"/>
-      <c r="P40" s="8"/>
-      <c r="Q40" s="8"/>
+      <c r="N40" s="13"/>
+      <c r="O40" s="13"/>
+      <c r="P40" s="13"/>
+      <c r="Q40" s="13"/>
     </row>
     <row r="41" spans="1:17">
-      <c r="A41" s="17">
+      <c r="A41" s="10">
         <v>26</v>
       </c>
-      <c r="B41" s="17" t="s">
+      <c r="B41" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="C41" s="17" t="s">
+      <c r="C41" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="D41" s="18" t="s">
+      <c r="D41" s="11" t="s">
         <v>104</v>
       </c>
-      <c r="E41" s="17"/>
-      <c r="F41" s="17"/>
-      <c r="G41" s="17"/>
-      <c r="H41" s="19">
+      <c r="E41" s="10"/>
+      <c r="F41" s="10"/>
+      <c r="G41" s="10"/>
+      <c r="H41" s="9">
         <v>2855104</v>
       </c>
-      <c r="I41" s="17"/>
-      <c r="J41" s="19">
-        <v>2855104</v>
-      </c>
-      <c r="K41" s="17"/>
-      <c r="L41" s="17"/>
-      <c r="M41" s="17"/>
-      <c r="N41" s="7"/>
-      <c r="O41" s="7"/>
-      <c r="P41" s="7"/>
-      <c r="Q41" s="7"/>
+      <c r="I41" s="9">
+        <v>2842504.32</v>
+      </c>
+      <c r="J41" s="9">
+        <v>12599.68</v>
+      </c>
+      <c r="K41" s="10">
+        <v>75</v>
+      </c>
+      <c r="L41" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="M41" s="16">
+        <v>46116</v>
+      </c>
+      <c r="N41" s="10"/>
+      <c r="O41" s="10"/>
+      <c r="P41" s="10"/>
+      <c r="Q41" s="10"/>
     </row>
     <row r="42" spans="1:17">
       <c r="A42" s="13">
@@ -2345,57 +2369,73 @@
       <c r="C42" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="D42" s="14" t="s">
+      <c r="D42" s="15" t="s">
         <v>105</v>
       </c>
       <c r="E42" s="13"/>
       <c r="F42" s="13"/>
       <c r="G42" s="13"/>
-      <c r="H42" s="15">
+      <c r="H42" s="12">
         <v>2610000</v>
       </c>
-      <c r="I42" s="13"/>
-      <c r="J42" s="15">
-        <v>2610000</v>
-      </c>
-      <c r="K42" s="13"/>
-      <c r="L42" s="13"/>
-      <c r="M42" s="13"/>
-      <c r="N42" s="8"/>
-      <c r="O42" s="8"/>
-      <c r="P42" s="8"/>
-      <c r="Q42" s="8"/>
+      <c r="I42" s="12">
+        <v>2266344.89</v>
+      </c>
+      <c r="J42" s="12">
+        <v>343655.11</v>
+      </c>
+      <c r="K42" s="13">
+        <v>80</v>
+      </c>
+      <c r="L42" s="13" t="s">
+        <v>126</v>
+      </c>
+      <c r="M42" s="14">
+        <v>46116</v>
+      </c>
+      <c r="N42" s="13"/>
+      <c r="O42" s="13"/>
+      <c r="P42" s="13"/>
+      <c r="Q42" s="13"/>
     </row>
     <row r="43" spans="1:17">
-      <c r="A43" s="17">
+      <c r="A43" s="10">
         <v>28</v>
       </c>
-      <c r="B43" s="17" t="s">
+      <c r="B43" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="C43" s="17" t="s">
+      <c r="C43" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="D43" s="18" t="s">
+      <c r="D43" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="E43" s="17"/>
-      <c r="F43" s="17"/>
-      <c r="G43" s="17"/>
-      <c r="H43" s="19">
+      <c r="E43" s="10"/>
+      <c r="F43" s="10"/>
+      <c r="G43" s="10"/>
+      <c r="H43" s="9">
         <v>3496000</v>
       </c>
-      <c r="I43" s="17"/>
-      <c r="J43" s="19">
-        <v>3496000</v>
-      </c>
-      <c r="K43" s="17"/>
-      <c r="L43" s="17"/>
-      <c r="M43" s="17"/>
-      <c r="N43" s="7"/>
-      <c r="O43" s="7"/>
-      <c r="P43" s="7"/>
-      <c r="Q43" s="7"/>
+      <c r="I43" s="9">
+        <v>2796000</v>
+      </c>
+      <c r="J43" s="9">
+        <v>700000</v>
+      </c>
+      <c r="K43" s="10">
+        <v>51</v>
+      </c>
+      <c r="L43" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="M43" s="16">
+        <v>46116</v>
+      </c>
+      <c r="N43" s="10"/>
+      <c r="O43" s="10"/>
+      <c r="P43" s="10"/>
+      <c r="Q43" s="10"/>
     </row>
     <row r="44" spans="1:17">
       <c r="A44" s="13">
@@ -2407,57 +2447,75 @@
       <c r="C44" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="D44" s="14" t="s">
+      <c r="D44" s="15" t="s">
         <v>107</v>
       </c>
       <c r="E44" s="13"/>
       <c r="F44" s="13"/>
       <c r="G44" s="13"/>
-      <c r="H44" s="15">
+      <c r="H44" s="12">
         <v>600000</v>
       </c>
-      <c r="I44" s="13"/>
-      <c r="J44" s="15">
-        <v>600000</v>
-      </c>
-      <c r="K44" s="13"/>
-      <c r="L44" s="13"/>
-      <c r="M44" s="13"/>
-      <c r="N44" s="8"/>
-      <c r="O44" s="8"/>
-      <c r="P44" s="8"/>
-      <c r="Q44" s="8"/>
-    </row>
-    <row r="45" spans="1:17">
-      <c r="A45" s="17">
+      <c r="I44" s="12">
+        <v>598400</v>
+      </c>
+      <c r="J44" s="12">
+        <v>1600</v>
+      </c>
+      <c r="K44" s="13">
+        <v>10</v>
+      </c>
+      <c r="L44" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="M44" s="14">
+        <v>46116</v>
+      </c>
+      <c r="N44" s="13"/>
+      <c r="O44" s="13"/>
+      <c r="P44" s="13"/>
+      <c r="Q44" s="13"/>
+    </row>
+    <row r="45" spans="1:17" ht="29">
+      <c r="A45" s="10">
         <v>30</v>
       </c>
-      <c r="B45" s="17" t="s">
+      <c r="B45" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="C45" s="17" t="s">
+      <c r="C45" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D45" s="18" t="s">
+      <c r="D45" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="E45" s="17"/>
-      <c r="F45" s="17"/>
-      <c r="G45" s="17"/>
-      <c r="H45" s="19">
+      <c r="E45" s="10"/>
+      <c r="F45" s="10"/>
+      <c r="G45" s="27" t="s">
+        <v>129</v>
+      </c>
+      <c r="H45" s="9">
         <v>640000</v>
       </c>
-      <c r="I45" s="17"/>
-      <c r="J45" s="19">
-        <v>640000</v>
-      </c>
-      <c r="K45" s="17"/>
-      <c r="L45" s="17"/>
-      <c r="M45" s="17"/>
-      <c r="N45" s="7"/>
-      <c r="O45" s="7"/>
-      <c r="P45" s="7"/>
-      <c r="Q45" s="7"/>
+      <c r="I45" s="9">
+        <v>598970</v>
+      </c>
+      <c r="J45" s="9">
+        <v>41030</v>
+      </c>
+      <c r="K45" s="10">
+        <v>100</v>
+      </c>
+      <c r="L45" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="M45" s="16">
+        <v>46116</v>
+      </c>
+      <c r="N45" s="10"/>
+      <c r="O45" s="10"/>
+      <c r="P45" s="10"/>
+      <c r="Q45" s="10"/>
     </row>
     <row r="46" spans="1:17">
       <c r="A46" s="13">
@@ -2469,57 +2527,73 @@
       <c r="C46" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="D46" s="14" t="s">
+      <c r="D46" s="15" t="s">
         <v>109</v>
       </c>
       <c r="E46" s="13"/>
       <c r="F46" s="13"/>
       <c r="G46" s="13"/>
-      <c r="H46" s="15">
+      <c r="H46" s="12">
         <v>650000</v>
       </c>
-      <c r="I46" s="13"/>
-      <c r="J46" s="15">
-        <v>650000</v>
-      </c>
-      <c r="K46" s="13"/>
-      <c r="L46" s="13"/>
-      <c r="M46" s="13"/>
-      <c r="N46" s="8"/>
-      <c r="O46" s="8"/>
-      <c r="P46" s="8"/>
-      <c r="Q46" s="8"/>
+      <c r="I46" s="12">
+        <v>530000</v>
+      </c>
+      <c r="J46" s="12">
+        <v>120000</v>
+      </c>
+      <c r="K46" s="13">
+        <v>15</v>
+      </c>
+      <c r="L46" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="M46" s="14">
+        <v>46116</v>
+      </c>
+      <c r="N46" s="13"/>
+      <c r="O46" s="13"/>
+      <c r="P46" s="13"/>
+      <c r="Q46" s="13"/>
     </row>
     <row r="47" spans="1:17">
-      <c r="A47" s="17">
+      <c r="A47" s="10">
         <v>32</v>
       </c>
-      <c r="B47" s="17" t="s">
+      <c r="B47" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="C47" s="17" t="s">
+      <c r="C47" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="D47" s="18" t="s">
+      <c r="D47" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="E47" s="17"/>
-      <c r="F47" s="17"/>
-      <c r="G47" s="17"/>
-      <c r="H47" s="19">
+      <c r="E47" s="10"/>
+      <c r="F47" s="10"/>
+      <c r="G47" s="10"/>
+      <c r="H47" s="9">
         <v>120000</v>
       </c>
-      <c r="I47" s="17"/>
-      <c r="J47" s="19">
+      <c r="I47" s="9">
         <v>120000</v>
       </c>
-      <c r="K47" s="17"/>
-      <c r="L47" s="17"/>
-      <c r="M47" s="17"/>
-      <c r="N47" s="7"/>
-      <c r="O47" s="7"/>
-      <c r="P47" s="7"/>
-      <c r="Q47" s="7"/>
+      <c r="J47" s="9">
+        <v>120000</v>
+      </c>
+      <c r="K47" s="10">
+        <v>100</v>
+      </c>
+      <c r="L47" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="M47" s="16">
+        <v>46116</v>
+      </c>
+      <c r="N47" s="10"/>
+      <c r="O47" s="10"/>
+      <c r="P47" s="10"/>
+      <c r="Q47" s="10"/>
     </row>
     <row r="48" spans="1:17">
       <c r="A48" s="13">
@@ -2531,57 +2605,75 @@
       <c r="C48" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="D48" s="14" t="s">
+      <c r="D48" s="15" t="s">
         <v>111</v>
       </c>
       <c r="E48" s="13"/>
       <c r="F48" s="13"/>
       <c r="G48" s="13"/>
-      <c r="H48" s="15">
+      <c r="H48" s="12">
         <v>222200</v>
       </c>
-      <c r="I48" s="13"/>
-      <c r="J48" s="15">
-        <v>222200</v>
-      </c>
-      <c r="K48" s="13"/>
-      <c r="L48" s="13"/>
-      <c r="M48" s="13"/>
-      <c r="N48" s="8"/>
-      <c r="O48" s="8"/>
-      <c r="P48" s="8"/>
-      <c r="Q48" s="8"/>
+      <c r="I48" s="12">
+        <v>222117</v>
+      </c>
+      <c r="J48" s="13">
+        <v>83</v>
+      </c>
+      <c r="K48" s="13">
+        <v>10</v>
+      </c>
+      <c r="L48" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="M48" s="14">
+        <v>46116</v>
+      </c>
+      <c r="N48" s="13"/>
+      <c r="O48" s="13"/>
+      <c r="P48" s="13"/>
+      <c r="Q48" s="13"/>
     </row>
     <row r="49" spans="1:17">
-      <c r="A49" s="17">
+      <c r="A49" s="10">
         <v>34</v>
       </c>
-      <c r="B49" s="17" t="s">
+      <c r="B49" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="C49" s="17" t="s">
+      <c r="C49" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="D49" s="18" t="s">
+      <c r="D49" s="11" t="s">
         <v>112</v>
       </c>
-      <c r="E49" s="17"/>
-      <c r="F49" s="17"/>
-      <c r="G49" s="17"/>
-      <c r="H49" s="19">
+      <c r="E49" s="10"/>
+      <c r="F49" s="10"/>
+      <c r="G49" s="27" t="s">
+        <v>130</v>
+      </c>
+      <c r="H49" s="9">
         <v>900000</v>
       </c>
-      <c r="I49" s="17"/>
-      <c r="J49" s="19">
-        <v>900000</v>
-      </c>
-      <c r="K49" s="17"/>
-      <c r="L49" s="17"/>
-      <c r="M49" s="17"/>
-      <c r="N49" s="7"/>
-      <c r="O49" s="7"/>
-      <c r="P49" s="7"/>
-      <c r="Q49" s="7"/>
+      <c r="I49" s="9">
+        <v>600000</v>
+      </c>
+      <c r="J49" s="9">
+        <v>300000</v>
+      </c>
+      <c r="K49" s="10">
+        <v>15</v>
+      </c>
+      <c r="L49" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="M49" s="16">
+        <v>46116</v>
+      </c>
+      <c r="N49" s="10"/>
+      <c r="O49" s="10"/>
+      <c r="P49" s="10"/>
+      <c r="Q49" s="10"/>
     </row>
     <row r="50" spans="1:17">
       <c r="A50" s="13">
@@ -2593,57 +2685,73 @@
       <c r="C50" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="D50" s="14" t="s">
+      <c r="D50" s="15" t="s">
         <v>113</v>
       </c>
       <c r="E50" s="13"/>
       <c r="F50" s="13"/>
-      <c r="G50" s="13"/>
-      <c r="H50" s="15">
+      <c r="G50" s="28" t="s">
+        <v>131</v>
+      </c>
+      <c r="H50" s="12">
         <v>278500</v>
       </c>
-      <c r="I50" s="13"/>
-      <c r="J50" s="15">
+      <c r="I50" s="12">
         <v>278500</v>
       </c>
-      <c r="K50" s="13"/>
-      <c r="L50" s="13"/>
-      <c r="M50" s="13"/>
-      <c r="N50" s="8"/>
-      <c r="O50" s="8"/>
-      <c r="P50" s="8"/>
-      <c r="Q50" s="8"/>
+      <c r="J50" s="13">
+        <v>0</v>
+      </c>
+      <c r="K50" s="13">
+        <v>15</v>
+      </c>
+      <c r="L50" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="M50" s="14">
+        <v>46116</v>
+      </c>
+      <c r="N50" s="13"/>
+      <c r="O50" s="13"/>
+      <c r="P50" s="13"/>
+      <c r="Q50" s="13"/>
     </row>
     <row r="51" spans="1:17">
-      <c r="A51" s="17">
+      <c r="A51" s="10">
         <v>36</v>
       </c>
-      <c r="B51" s="17" t="s">
+      <c r="B51" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="C51" s="17" t="s">
+      <c r="C51" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="D51" s="18" t="s">
+      <c r="D51" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="E51" s="17"/>
-      <c r="F51" s="17"/>
-      <c r="G51" s="17"/>
-      <c r="H51" s="19">
+      <c r="E51" s="10"/>
+      <c r="F51" s="10"/>
+      <c r="G51" s="10"/>
+      <c r="H51" s="9">
         <v>225000</v>
       </c>
-      <c r="I51" s="17"/>
-      <c r="J51" s="19">
+      <c r="I51" s="10"/>
+      <c r="J51" s="9">
         <v>225000</v>
       </c>
-      <c r="K51" s="17"/>
-      <c r="L51" s="17"/>
-      <c r="M51" s="17"/>
-      <c r="N51" s="7"/>
-      <c r="O51" s="7"/>
-      <c r="P51" s="7"/>
-      <c r="Q51" s="7"/>
+      <c r="K51" s="10">
+        <v>5</v>
+      </c>
+      <c r="L51" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="M51" s="16">
+        <v>46116</v>
+      </c>
+      <c r="N51" s="10"/>
+      <c r="O51" s="10"/>
+      <c r="P51" s="10"/>
+      <c r="Q51" s="10"/>
     </row>
     <row r="52" spans="1:17">
       <c r="A52" s="13">
@@ -2655,59 +2763,71 @@
       <c r="C52" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="D52" s="14" t="s">
+      <c r="D52" s="15" t="s">
         <v>115</v>
       </c>
       <c r="E52" s="13"/>
       <c r="F52" s="13"/>
       <c r="G52" s="13"/>
-      <c r="H52" s="15">
+      <c r="H52" s="12">
         <v>85000</v>
       </c>
       <c r="I52" s="13"/>
-      <c r="J52" s="15">
+      <c r="J52" s="12">
         <v>85000</v>
       </c>
-      <c r="K52" s="13"/>
-      <c r="L52" s="13"/>
-      <c r="M52" s="13"/>
-      <c r="N52" s="8"/>
-      <c r="O52" s="8"/>
-      <c r="P52" s="8"/>
-      <c r="Q52" s="8"/>
+      <c r="K52" s="13">
+        <v>5</v>
+      </c>
+      <c r="L52" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="M52" s="14">
+        <v>46116</v>
+      </c>
+      <c r="N52" s="13"/>
+      <c r="O52" s="13"/>
+      <c r="P52" s="13"/>
+      <c r="Q52" s="13"/>
     </row>
     <row r="53" spans="1:17">
-      <c r="A53" s="17">
+      <c r="A53" s="10">
         <v>38</v>
       </c>
-      <c r="B53" s="17" t="s">
+      <c r="B53" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="C53" s="17" t="s">
+      <c r="C53" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="D53" s="18" t="s">
+      <c r="D53" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="E53" s="11" t="s">
+      <c r="E53" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="F53" s="17"/>
-      <c r="G53" s="17"/>
-      <c r="H53" s="19">
+      <c r="F53" s="10"/>
+      <c r="G53" s="10"/>
+      <c r="H53" s="9">
         <v>1800000</v>
       </c>
-      <c r="I53" s="17"/>
-      <c r="J53" s="19">
+      <c r="I53" s="10"/>
+      <c r="J53" s="9">
         <v>1800000</v>
       </c>
-      <c r="K53" s="17"/>
-      <c r="L53" s="17"/>
-      <c r="M53" s="17"/>
-      <c r="N53" s="7"/>
-      <c r="O53" s="7"/>
-      <c r="P53" s="7"/>
-      <c r="Q53" s="7"/>
+      <c r="K53" s="10">
+        <v>5</v>
+      </c>
+      <c r="L53" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="M53" s="16">
+        <v>46116</v>
+      </c>
+      <c r="N53" s="10"/>
+      <c r="O53" s="10"/>
+      <c r="P53" s="10"/>
+      <c r="Q53" s="10"/>
     </row>
     <row r="54" spans="1:17">
       <c r="A54" s="13">
@@ -2719,61 +2839,73 @@
       <c r="C54" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="D54" s="14" t="s">
+      <c r="D54" s="15" t="s">
         <v>119</v>
       </c>
-      <c r="E54" s="12" t="s">
+      <c r="E54" s="8" t="s">
         <v>120</v>
       </c>
       <c r="F54" s="13"/>
       <c r="G54" s="13"/>
-      <c r="H54" s="15">
+      <c r="H54" s="12">
         <v>1120000</v>
       </c>
       <c r="I54" s="13"/>
-      <c r="J54" s="15">
+      <c r="J54" s="12">
         <v>1120000</v>
       </c>
-      <c r="K54" s="13"/>
-      <c r="L54" s="13"/>
-      <c r="M54" s="13"/>
-      <c r="N54" s="8"/>
-      <c r="O54" s="8"/>
-      <c r="P54" s="8"/>
-      <c r="Q54" s="8"/>
+      <c r="K54" s="13">
+        <v>5</v>
+      </c>
+      <c r="L54" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="M54" s="14">
+        <v>46116</v>
+      </c>
+      <c r="N54" s="13"/>
+      <c r="O54" s="13"/>
+      <c r="P54" s="13"/>
+      <c r="Q54" s="13"/>
     </row>
     <row r="55" spans="1:17">
-      <c r="A55" s="17">
+      <c r="A55" s="10">
         <v>40</v>
       </c>
-      <c r="B55" s="17" t="s">
+      <c r="B55" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="C55" s="17" t="s">
+      <c r="C55" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="D55" s="18" t="s">
+      <c r="D55" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="E55" s="11" t="s">
+      <c r="E55" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="F55" s="17"/>
-      <c r="G55" s="17"/>
-      <c r="H55" s="19">
+      <c r="F55" s="10"/>
+      <c r="G55" s="10"/>
+      <c r="H55" s="9">
         <v>860000</v>
       </c>
-      <c r="I55" s="17"/>
-      <c r="J55" s="19">
+      <c r="I55" s="10"/>
+      <c r="J55" s="9">
         <v>860000</v>
       </c>
-      <c r="K55" s="17"/>
-      <c r="L55" s="17"/>
-      <c r="M55" s="17"/>
-      <c r="N55" s="7"/>
-      <c r="O55" s="7"/>
-      <c r="P55" s="7"/>
-      <c r="Q55" s="7"/>
+      <c r="K55" s="10">
+        <v>5</v>
+      </c>
+      <c r="L55" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="M55" s="16">
+        <v>46116</v>
+      </c>
+      <c r="N55" s="10"/>
+      <c r="O55" s="10"/>
+      <c r="P55" s="10"/>
+      <c r="Q55" s="10"/>
     </row>
     <row r="56" spans="1:17">
       <c r="A56" s="13">
@@ -2785,55 +2917,73 @@
       <c r="C56" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="D56" s="14" t="s">
+      <c r="D56" s="15" t="s">
         <v>123</v>
       </c>
-      <c r="E56" s="12" t="s">
+      <c r="E56" s="8" t="s">
         <v>124</v>
       </c>
       <c r="F56" s="13"/>
       <c r="G56" s="13"/>
-      <c r="H56" s="15">
+      <c r="H56" s="12">
         <v>500000</v>
       </c>
       <c r="I56" s="13"/>
-      <c r="J56" s="15">
+      <c r="J56" s="12">
         <v>500000</v>
       </c>
-      <c r="K56" s="13"/>
-      <c r="L56" s="13"/>
-      <c r="M56" s="13"/>
-      <c r="N56" s="6"/>
-      <c r="O56" s="6"/>
-      <c r="P56" s="6"/>
-      <c r="Q56" s="6"/>
+      <c r="K56" s="13">
+        <v>5</v>
+      </c>
+      <c r="L56" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="M56" s="14">
+        <v>46116</v>
+      </c>
+      <c r="N56" s="13"/>
+      <c r="O56" s="13"/>
+      <c r="P56" s="13"/>
+      <c r="Q56" s="13"/>
     </row>
     <row r="57" spans="1:17">
-      <c r="A57" s="17">
+      <c r="A57" s="10">
         <v>42</v>
       </c>
-      <c r="B57" s="17" t="s">
+      <c r="B57" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="C57" s="17" t="s">
+      <c r="C57" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="D57" s="18" t="s">
+      <c r="D57" s="11" t="s">
         <v>125</v>
       </c>
-      <c r="E57" s="11"/>
-      <c r="F57" s="17"/>
-      <c r="G57" s="17"/>
-      <c r="H57" s="19">
+      <c r="E57" s="7"/>
+      <c r="F57" s="10"/>
+      <c r="G57" s="10"/>
+      <c r="H57" s="9">
         <v>380000</v>
       </c>
-      <c r="I57" s="17"/>
-      <c r="J57" s="19">
-        <v>380000</v>
-      </c>
-      <c r="K57" s="17"/>
-      <c r="L57" s="17"/>
-      <c r="M57" s="17"/>
+      <c r="I57" s="9">
+        <v>205456</v>
+      </c>
+      <c r="J57" s="9">
+        <v>174544</v>
+      </c>
+      <c r="K57" s="10">
+        <v>90</v>
+      </c>
+      <c r="L57" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="M57" s="16">
+        <v>46116</v>
+      </c>
+      <c r="N57" s="10"/>
+      <c r="O57" s="10"/>
+      <c r="P57" s="10"/>
+      <c r="Q57" s="10"/>
     </row>
     <row r="58" spans="1:17">
       <c r="A58" s="13">
@@ -2853,25 +3003,33 @@
       <c r="K58" s="13"/>
       <c r="L58" s="13"/>
       <c r="M58" s="13"/>
+      <c r="N58" s="13"/>
+      <c r="O58" s="13"/>
+      <c r="P58" s="13"/>
+      <c r="Q58" s="13"/>
     </row>
     <row r="59" spans="1:17">
-      <c r="A59" s="17">
+      <c r="A59" s="10">
         <v>44</v>
       </c>
-      <c r="B59" s="17"/>
-      <c r="C59" s="17"/>
-      <c r="D59" s="17"/>
-      <c r="E59" s="17"/>
-      <c r="F59" s="17"/>
-      <c r="G59" s="17"/>
-      <c r="H59" s="17"/>
-      <c r="I59" s="17"/>
-      <c r="J59" s="17">
+      <c r="B59" s="10"/>
+      <c r="C59" s="10"/>
+      <c r="D59" s="10"/>
+      <c r="E59" s="10"/>
+      <c r="F59" s="10"/>
+      <c r="G59" s="10"/>
+      <c r="H59" s="10"/>
+      <c r="I59" s="10"/>
+      <c r="J59" s="10">
         <v>0</v>
       </c>
-      <c r="K59" s="17"/>
-      <c r="L59" s="17"/>
-      <c r="M59" s="17"/>
+      <c r="K59" s="10"/>
+      <c r="L59" s="10"/>
+      <c r="M59" s="10"/>
+      <c r="N59" s="10"/>
+      <c r="O59" s="10"/>
+      <c r="P59" s="10"/>
+      <c r="Q59" s="10"/>
     </row>
     <row r="60" spans="1:17">
       <c r="A60" s="13">
@@ -2891,23 +3049,239 @@
       <c r="K60" s="13"/>
       <c r="L60" s="13"/>
       <c r="M60" s="13"/>
+      <c r="N60" s="13"/>
+      <c r="O60" s="13"/>
+      <c r="P60" s="13"/>
+      <c r="Q60" s="13"/>
     </row>
     <row r="61" spans="1:17">
       <c r="A61" t="s">
         <v>116</v>
       </c>
-      <c r="H61" s="10">
+      <c r="H61" s="6">
         <v>31071804</v>
       </c>
-      <c r="I61" s="10">
+      <c r="I61" s="6">
         <v>3872529.9</v>
       </c>
-      <c r="J61" s="10">
+      <c r="J61" s="6">
         <v>27199274.100000001</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="168">
+  <mergeCells count="224">
+    <mergeCell ref="N35:N36"/>
+    <mergeCell ref="O35:O36"/>
+    <mergeCell ref="P35:P36"/>
+    <mergeCell ref="Q35:Q36"/>
+    <mergeCell ref="N38:N39"/>
+    <mergeCell ref="O38:O39"/>
+    <mergeCell ref="P38:P39"/>
+    <mergeCell ref="Q38:Q39"/>
+    <mergeCell ref="N26:N27"/>
+    <mergeCell ref="O26:O27"/>
+    <mergeCell ref="P26:P27"/>
+    <mergeCell ref="Q26:Q27"/>
+    <mergeCell ref="N28:N29"/>
+    <mergeCell ref="O28:O29"/>
+    <mergeCell ref="P28:P29"/>
+    <mergeCell ref="Q28:Q29"/>
+    <mergeCell ref="N31:N32"/>
+    <mergeCell ref="O31:O32"/>
+    <mergeCell ref="P31:P32"/>
+    <mergeCell ref="Q31:Q32"/>
+    <mergeCell ref="N19:N20"/>
+    <mergeCell ref="O19:O20"/>
+    <mergeCell ref="P19:P20"/>
+    <mergeCell ref="Q19:Q20"/>
+    <mergeCell ref="N22:N23"/>
+    <mergeCell ref="O22:O23"/>
+    <mergeCell ref="P22:P23"/>
+    <mergeCell ref="Q22:Q23"/>
+    <mergeCell ref="N24:N25"/>
+    <mergeCell ref="O24:O25"/>
+    <mergeCell ref="P24:P25"/>
+    <mergeCell ref="Q24:Q25"/>
+    <mergeCell ref="N11:N12"/>
+    <mergeCell ref="O11:O12"/>
+    <mergeCell ref="P11:P12"/>
+    <mergeCell ref="Q11:Q12"/>
+    <mergeCell ref="N14:N15"/>
+    <mergeCell ref="O14:O15"/>
+    <mergeCell ref="P14:P15"/>
+    <mergeCell ref="Q14:Q15"/>
+    <mergeCell ref="N16:N17"/>
+    <mergeCell ref="O16:O17"/>
+    <mergeCell ref="P16:P17"/>
+    <mergeCell ref="Q16:Q17"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="O2:O3"/>
+    <mergeCell ref="P2:P3"/>
+    <mergeCell ref="Q2:Q3"/>
+    <mergeCell ref="N4:N5"/>
+    <mergeCell ref="O4:O5"/>
+    <mergeCell ref="P4:P5"/>
+    <mergeCell ref="Q4:Q5"/>
+    <mergeCell ref="N9:N10"/>
+    <mergeCell ref="O9:O10"/>
+    <mergeCell ref="P9:P10"/>
+    <mergeCell ref="Q9:Q10"/>
+    <mergeCell ref="H38:H39"/>
+    <mergeCell ref="I38:I39"/>
+    <mergeCell ref="J38:J39"/>
+    <mergeCell ref="K38:K39"/>
+    <mergeCell ref="L38:L39"/>
+    <mergeCell ref="M38:M39"/>
+    <mergeCell ref="A38:A39"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="D38:D39"/>
+    <mergeCell ref="E38:E39"/>
+    <mergeCell ref="G38:G39"/>
+    <mergeCell ref="H35:H36"/>
+    <mergeCell ref="I35:I36"/>
+    <mergeCell ref="J35:J36"/>
+    <mergeCell ref="K35:K36"/>
+    <mergeCell ref="L35:L36"/>
+    <mergeCell ref="M35:M36"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="C35:C36"/>
+    <mergeCell ref="D35:D36"/>
+    <mergeCell ref="E35:E36"/>
+    <mergeCell ref="G35:G36"/>
+    <mergeCell ref="H31:H32"/>
+    <mergeCell ref="I31:I32"/>
+    <mergeCell ref="J31:J32"/>
+    <mergeCell ref="K31:K32"/>
+    <mergeCell ref="L31:L32"/>
+    <mergeCell ref="M31:M32"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="C31:C32"/>
+    <mergeCell ref="D31:D32"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="G31:G32"/>
+    <mergeCell ref="H28:H29"/>
+    <mergeCell ref="I28:I29"/>
+    <mergeCell ref="J28:J29"/>
+    <mergeCell ref="K28:K29"/>
+    <mergeCell ref="L28:L29"/>
+    <mergeCell ref="M28:M29"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="C28:C29"/>
+    <mergeCell ref="D28:D29"/>
+    <mergeCell ref="E28:E29"/>
+    <mergeCell ref="G28:G29"/>
+    <mergeCell ref="H26:H27"/>
+    <mergeCell ref="I26:I27"/>
+    <mergeCell ref="J26:J27"/>
+    <mergeCell ref="K26:K27"/>
+    <mergeCell ref="L26:L27"/>
+    <mergeCell ref="M26:M27"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="C26:C27"/>
+    <mergeCell ref="D26:D27"/>
+    <mergeCell ref="E26:E27"/>
+    <mergeCell ref="G26:G27"/>
+    <mergeCell ref="H24:H25"/>
+    <mergeCell ref="I24:I25"/>
+    <mergeCell ref="J24:J25"/>
+    <mergeCell ref="K24:K25"/>
+    <mergeCell ref="L24:L25"/>
+    <mergeCell ref="M24:M25"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="E24:E25"/>
+    <mergeCell ref="G24:G25"/>
+    <mergeCell ref="H22:H23"/>
+    <mergeCell ref="I22:I23"/>
+    <mergeCell ref="J22:J23"/>
+    <mergeCell ref="K22:K23"/>
+    <mergeCell ref="L22:L23"/>
+    <mergeCell ref="M22:M23"/>
+    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="D22:D23"/>
+    <mergeCell ref="E22:E23"/>
+    <mergeCell ref="G22:G23"/>
+    <mergeCell ref="H19:H20"/>
+    <mergeCell ref="I19:I20"/>
+    <mergeCell ref="J19:J20"/>
+    <mergeCell ref="K19:K20"/>
+    <mergeCell ref="L19:L20"/>
+    <mergeCell ref="M19:M20"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="E19:E20"/>
+    <mergeCell ref="G19:G20"/>
+    <mergeCell ref="H16:H17"/>
+    <mergeCell ref="I16:I17"/>
+    <mergeCell ref="J16:J17"/>
+    <mergeCell ref="K16:K17"/>
+    <mergeCell ref="L16:L17"/>
+    <mergeCell ref="M16:M17"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="E16:E17"/>
+    <mergeCell ref="G16:G17"/>
+    <mergeCell ref="H14:H15"/>
+    <mergeCell ref="I14:I15"/>
+    <mergeCell ref="J14:J15"/>
+    <mergeCell ref="K14:K15"/>
+    <mergeCell ref="L14:L15"/>
+    <mergeCell ref="M14:M15"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="E14:E15"/>
+    <mergeCell ref="G14:G15"/>
+    <mergeCell ref="H11:H12"/>
+    <mergeCell ref="I11:I12"/>
+    <mergeCell ref="J11:J12"/>
+    <mergeCell ref="K11:K12"/>
+    <mergeCell ref="L11:L12"/>
+    <mergeCell ref="M11:M12"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="G11:G12"/>
+    <mergeCell ref="H9:H10"/>
+    <mergeCell ref="I9:I10"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="K9:K10"/>
+    <mergeCell ref="L9:L10"/>
+    <mergeCell ref="M9:M10"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="I4:I5"/>
+    <mergeCell ref="J4:J5"/>
+    <mergeCell ref="K4:K5"/>
+    <mergeCell ref="L4:L5"/>
+    <mergeCell ref="M4:M5"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="G4:G5"/>
     <mergeCell ref="H2:H3"/>
     <mergeCell ref="I2:I3"/>
     <mergeCell ref="J2:J3"/>
@@ -2920,163 +3294,14 @@
     <mergeCell ref="D2:D3"/>
     <mergeCell ref="E2:E3"/>
     <mergeCell ref="G2:G3"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="I4:I5"/>
-    <mergeCell ref="J4:J5"/>
-    <mergeCell ref="K4:K5"/>
-    <mergeCell ref="L4:L5"/>
-    <mergeCell ref="M4:M5"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="G4:G5"/>
-    <mergeCell ref="H9:H10"/>
-    <mergeCell ref="I9:I10"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="K9:K10"/>
-    <mergeCell ref="L9:L10"/>
-    <mergeCell ref="M9:M10"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="G9:G10"/>
-    <mergeCell ref="H11:H12"/>
-    <mergeCell ref="I11:I12"/>
-    <mergeCell ref="J11:J12"/>
-    <mergeCell ref="K11:K12"/>
-    <mergeCell ref="L11:L12"/>
-    <mergeCell ref="M11:M12"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="G11:G12"/>
-    <mergeCell ref="H14:H15"/>
-    <mergeCell ref="I14:I15"/>
-    <mergeCell ref="J14:J15"/>
-    <mergeCell ref="K14:K15"/>
-    <mergeCell ref="L14:L15"/>
-    <mergeCell ref="M14:M15"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="E14:E15"/>
-    <mergeCell ref="G14:G15"/>
-    <mergeCell ref="H16:H17"/>
-    <mergeCell ref="I16:I17"/>
-    <mergeCell ref="J16:J17"/>
-    <mergeCell ref="K16:K17"/>
-    <mergeCell ref="L16:L17"/>
-    <mergeCell ref="M16:M17"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="E16:E17"/>
-    <mergeCell ref="G16:G17"/>
-    <mergeCell ref="H19:H20"/>
-    <mergeCell ref="I19:I20"/>
-    <mergeCell ref="J19:J20"/>
-    <mergeCell ref="K19:K20"/>
-    <mergeCell ref="L19:L20"/>
-    <mergeCell ref="M19:M20"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="C19:C20"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="E19:E20"/>
-    <mergeCell ref="G19:G20"/>
-    <mergeCell ref="H22:H23"/>
-    <mergeCell ref="I22:I23"/>
-    <mergeCell ref="J22:J23"/>
-    <mergeCell ref="K22:K23"/>
-    <mergeCell ref="L22:L23"/>
-    <mergeCell ref="M22:M23"/>
-    <mergeCell ref="A22:A23"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="D22:D23"/>
-    <mergeCell ref="E22:E23"/>
-    <mergeCell ref="G22:G23"/>
-    <mergeCell ref="H24:H25"/>
-    <mergeCell ref="I24:I25"/>
-    <mergeCell ref="J24:J25"/>
-    <mergeCell ref="K24:K25"/>
-    <mergeCell ref="L24:L25"/>
-    <mergeCell ref="M24:M25"/>
-    <mergeCell ref="A24:A25"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="E24:E25"/>
-    <mergeCell ref="G24:G25"/>
-    <mergeCell ref="H26:H27"/>
-    <mergeCell ref="I26:I27"/>
-    <mergeCell ref="J26:J27"/>
-    <mergeCell ref="K26:K27"/>
-    <mergeCell ref="L26:L27"/>
-    <mergeCell ref="M26:M27"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="C26:C27"/>
-    <mergeCell ref="D26:D27"/>
-    <mergeCell ref="E26:E27"/>
-    <mergeCell ref="G26:G27"/>
-    <mergeCell ref="H28:H29"/>
-    <mergeCell ref="I28:I29"/>
-    <mergeCell ref="J28:J29"/>
-    <mergeCell ref="K28:K29"/>
-    <mergeCell ref="L28:L29"/>
-    <mergeCell ref="M28:M29"/>
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="B28:B29"/>
-    <mergeCell ref="C28:C29"/>
-    <mergeCell ref="D28:D29"/>
-    <mergeCell ref="E28:E29"/>
-    <mergeCell ref="G28:G29"/>
-    <mergeCell ref="H31:H32"/>
-    <mergeCell ref="I31:I32"/>
-    <mergeCell ref="J31:J32"/>
-    <mergeCell ref="K31:K32"/>
-    <mergeCell ref="L31:L32"/>
-    <mergeCell ref="M31:M32"/>
-    <mergeCell ref="A31:A32"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="C31:C32"/>
-    <mergeCell ref="D31:D32"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="G31:G32"/>
-    <mergeCell ref="H35:H36"/>
-    <mergeCell ref="I35:I36"/>
-    <mergeCell ref="J35:J36"/>
-    <mergeCell ref="K35:K36"/>
-    <mergeCell ref="L35:L36"/>
-    <mergeCell ref="M35:M36"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="B35:B36"/>
-    <mergeCell ref="C35:C36"/>
-    <mergeCell ref="D35:D36"/>
-    <mergeCell ref="E35:E36"/>
-    <mergeCell ref="G35:G36"/>
-    <mergeCell ref="H38:H39"/>
-    <mergeCell ref="I38:I39"/>
-    <mergeCell ref="J38:J39"/>
-    <mergeCell ref="K38:K39"/>
-    <mergeCell ref="L38:L39"/>
-    <mergeCell ref="M38:M39"/>
-    <mergeCell ref="A38:A39"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="C38:C39"/>
-    <mergeCell ref="D38:D39"/>
-    <mergeCell ref="E38:E39"/>
-    <mergeCell ref="G38:G39"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="N6" r:id="rId1" display="https://mitrphol-my.sharepoint.com/:i:/r/personal/waiyawatc_mitrphol_com/Documents/Investment_Report/Image/%E0%B8%87%E0%B8%B2%E0%B8%99%E0%B9%84%E0%B8%A5%E0%B8%99%E0%B9%8C%E0%B8%97%E0%B9%88%E0%B8%AD%E0%B9%81%E0%B8%AD%E0%B8%A5%E0%B8%81%E0%B8%AD%E0%B8%AE%E0%B8%AD%E0%B8%A5%E0%B9%8C.jpg?csf=1&amp;web=1&amp;e=Rcs21T"/>
+    <hyperlink ref="N8" r:id="rId2" display="https://mitrphol-my.sharepoint.com/:i:/p/waiyawatc/IQAjzQ3BolfaSZnAIilNyWWpAYcTBiiYxD2SYEFDW6J4XDw?e=fWngVV"/>
+    <hyperlink ref="N24" r:id="rId3"/>
+    <hyperlink ref="O24" r:id="rId4"/>
+    <hyperlink ref="N33" r:id="rId5"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>